<commit_message>
Correction Error in equation De Groote
</commit_message>
<xml_diff>
--- a/hypothetical_data.xlsx
+++ b/hypothetical_data.xlsx
@@ -507,7 +507,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-135.8181667586299</v>
+        <v>-7.039566080071809</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
@@ -525,36 +525,36 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06253281370900618</v>
+        <v>0.06253281370900747</v>
       </c>
       <c r="H2" t="n">
-        <v>0.05010332837589021</v>
+        <v>0.05879831855407186</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06205666365794821</v>
+        <v>0.06870583418279234</v>
       </c>
       <c r="J2" t="n">
-        <v>7.826424365587958</v>
+        <v>7.82642436558713</v>
       </c>
       <c r="K2" t="n">
-        <v>24.92592040365737</v>
+        <v>21.0463717756711</v>
       </c>
       <c r="L2" t="n">
-        <v>12.47889102060679</v>
+        <v>11.25455325770014</v>
       </c>
       <c r="M2" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2608155426260997</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3931429881010686</v>
+        <v>0.3863489999533918</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-9.761957293071108</v>
+        <v>-0.5319015639747097</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
@@ -572,10 +572,10 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.07286844709700198</v>
+        <v>0.07286844709700196</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05000784024966202</v>
+        <v>0.05137435493602627</v>
       </c>
       <c r="I3" t="n">
         <v>0.0602403748541654</v>
@@ -584,16 +584,16 @@
         <v>6.710793399280124</v>
       </c>
       <c r="K3" t="n">
-        <v>24.97677479812686</v>
+        <v>24.26888371734317</v>
       </c>
       <c r="L3" t="n">
-        <v>12.86148801950081</v>
+        <v>12.8614880195005</v>
       </c>
       <c r="M3" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2519441235097216</v>
+        <v>0.2504409517469803</v>
       </c>
       <c r="O3" t="n">
         <v>0.3855295790644589</v>
@@ -601,7 +601,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>-7.241951135882761e-12</v>
+        <v>-1.448390227176552e-11</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -619,22 +619,22 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.08290061396627721</v>
+        <v>0.08290061396627714</v>
       </c>
       <c r="H4" t="n">
-        <v>0.04252156913666626</v>
+        <v>0.04252156912705999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.05017595975382205</v>
+        <v>0.0501759597536128</v>
       </c>
       <c r="J4" t="n">
-        <v>5.895611618411004</v>
+        <v>5.895611618410959</v>
       </c>
       <c r="K4" t="n">
-        <v>29.77475551801597</v>
+        <v>29.77475552874706</v>
       </c>
       <c r="L4" t="n">
-        <v>15.50030379108039</v>
+        <v>15.50030379115225</v>
       </c>
       <c r="M4" t="n">
         <v>0.2233067431983749</v>
@@ -648,7 +648,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-2.289588808154755e-12</v>
+        <v>-1.52224861053265e-11</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
@@ -666,28 +666,28 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.09234950013810864</v>
+        <v>0.09234950013810865</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03367093419842721</v>
+        <v>0.03367093358486833</v>
       </c>
       <c r="I5" t="n">
-        <v>0.03983894166860114</v>
+        <v>0.03983894170351002</v>
       </c>
       <c r="J5" t="n">
-        <v>5.290573350413708</v>
+        <v>5.290573350413722</v>
       </c>
       <c r="K5" t="n">
-        <v>38.83825833721024</v>
+        <v>38.83825959591886</v>
       </c>
       <c r="L5" t="n">
-        <v>19.66896232948704</v>
+        <v>19.66896231467956</v>
       </c>
       <c r="M5" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N5" t="n">
-        <v>0.2503438825093872</v>
+        <v>0.2503438825093889</v>
       </c>
       <c r="O5" t="n">
         <v>0.3855295790644589</v>
@@ -695,7 +695,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4.932412295690425</v>
+        <v>0.1394103164094459</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
@@ -713,25 +713,25 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.09812542476084979</v>
+        <v>0.1009126975550348</v>
       </c>
       <c r="H6" t="n">
-        <v>0.02610340688884793</v>
+        <v>0.02610341344143545</v>
       </c>
       <c r="I6" t="n">
-        <v>0.02989360751453198</v>
+        <v>0.02989360895986806</v>
       </c>
       <c r="J6" t="n">
-        <v>4.978345196187929</v>
+        <v>4.840507364843518</v>
       </c>
       <c r="K6" t="n">
-        <v>53.99157408144779</v>
+        <v>53.99159103984579</v>
       </c>
       <c r="L6" t="n">
-        <v>26.65159361542443</v>
+        <v>26.65159221196385</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2262072674589311</v>
+        <v>0.2234097331711473</v>
       </c>
       <c r="N6" t="n">
         <v>0.2503438825093872</v>
@@ -742,7 +742,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>-113.0327475797165</v>
+        <v>-5.273799447132276</v>
       </c>
       <c r="B7" t="n">
         <v>90</v>
@@ -760,28 +760,28 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0.06253281370900644</v>
+        <v>0.06253281370900621</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05010332837589126</v>
+        <v>0.05879831855407187</v>
       </c>
       <c r="I7" t="n">
-        <v>0.05499992440104676</v>
+        <v>0.05499992440104683</v>
       </c>
       <c r="J7" t="n">
-        <v>7.826424365587854</v>
+        <v>7.826424365587948</v>
       </c>
       <c r="K7" t="n">
-        <v>24.92592040365654</v>
+        <v>21.0463717756711</v>
       </c>
       <c r="L7" t="n">
-        <v>14.11116142850675</v>
+        <v>14.11116142850689</v>
       </c>
       <c r="M7" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N7" t="n">
-        <v>0.2608155426260985</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O7" t="n">
         <v>0.3855295790644589</v>
@@ -789,7 +789,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-9.761957293070832</v>
+        <v>-0.5319015639573886</v>
       </c>
       <c r="B8" t="n">
         <v>90</v>
@@ -807,28 +807,28 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0728684470970019</v>
+        <v>0.07286844709700188</v>
       </c>
       <c r="H8" t="n">
-        <v>0.05000784024966202</v>
+        <v>0.05137435493607772</v>
       </c>
       <c r="I8" t="n">
-        <v>0.04618037325663626</v>
+        <v>0.04618037325653893</v>
       </c>
       <c r="J8" t="n">
-        <v>6.710793399280194</v>
+        <v>6.710793399280171</v>
       </c>
       <c r="K8" t="n">
-        <v>24.97677479812686</v>
+        <v>24.26888371728679</v>
       </c>
       <c r="L8" t="n">
-        <v>16.87985375458279</v>
+        <v>16.87985375461659</v>
       </c>
       <c r="M8" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N8" t="n">
-        <v>0.2519441235097216</v>
+        <v>0.2504409517469772</v>
       </c>
       <c r="O8" t="n">
         <v>0.3855295790644589</v>
@@ -836,7 +836,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-7.195245405540521e-12</v>
+        <v>-1.439049081108104e-11</v>
       </c>
       <c r="B9" t="n">
         <v>90</v>
@@ -854,22 +854,22 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0.08290061396627717</v>
+        <v>0.08290061396627715</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04252156911521876</v>
+        <v>0.04252156884973735</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03657296377746325</v>
+        <v>0.03657296386498159</v>
       </c>
       <c r="J9" t="n">
-        <v>5.895611618411039</v>
+        <v>5.895611618411028</v>
       </c>
       <c r="K9" t="n">
-        <v>29.77475554072043</v>
+        <v>29.77475582140898</v>
       </c>
       <c r="L9" t="n">
-        <v>21.50869238296757</v>
+        <v>21.50869233049583</v>
       </c>
       <c r="M9" t="n">
         <v>0.2233067431983749</v>
@@ -883,7 +883,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-4.238332112308011e-12</v>
+        <v>2.166644264400974e-12</v>
       </c>
       <c r="B10" t="n">
         <v>90</v>
@@ -904,25 +904,25 @@
         <v>0.09234950013810854</v>
       </c>
       <c r="H10" t="n">
-        <v>0.03367093354070443</v>
+        <v>0.03367093419804766</v>
       </c>
       <c r="I10" t="n">
-        <v>0.02685826388012297</v>
+        <v>0.02685826388011879</v>
       </c>
       <c r="J10" t="n">
-        <v>5.290573350413704</v>
+        <v>5.290573350413691</v>
       </c>
       <c r="K10" t="n">
-        <v>38.83825966879478</v>
+        <v>38.83825833590058</v>
       </c>
       <c r="L10" t="n">
-        <v>29.950910132739</v>
+        <v>29.95091013270286</v>
       </c>
       <c r="M10" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N10" t="n">
-        <v>0.2503438825093889</v>
+        <v>0.2503438825093872</v>
       </c>
       <c r="O10" t="n">
         <v>0.3855295790644563</v>
@@ -930,7 +930,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4.932412295693601</v>
+        <v>0.1394103164167488</v>
       </c>
       <c r="B11" t="n">
         <v>90</v>
@@ -948,25 +948,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0.09812542476084979</v>
+        <v>0.1009126975550342</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02610341344145064</v>
+        <v>0.0261034092055065</v>
       </c>
       <c r="I11" t="n">
-        <v>0.01827050420037458</v>
+        <v>0.0182705057050344</v>
       </c>
       <c r="J11" t="n">
-        <v>4.978345196187929</v>
+        <v>4.840507364843529</v>
       </c>
       <c r="K11" t="n">
-        <v>53.99159103979386</v>
+        <v>53.99158044128656</v>
       </c>
       <c r="L11" t="n">
-        <v>47.21650075176496</v>
+        <v>47.21651253749265</v>
       </c>
       <c r="M11" t="n">
-        <v>0.226207267458931</v>
+        <v>0.2234097331711478</v>
       </c>
       <c r="N11" t="n">
         <v>0.2503438825093872</v>
@@ -977,7 +977,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>-4911.710486395493</v>
+        <v>-44.2918429249067</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
@@ -995,36 +995,36 @@
         <v>0.2</v>
       </c>
       <c r="G12" t="n">
-        <v>0.06253281370900741</v>
+        <v>0.06253281370900596</v>
       </c>
       <c r="H12" t="n">
-        <v>0.03006399501375825</v>
+        <v>0.05595688151536371</v>
       </c>
       <c r="I12" t="n">
-        <v>0.03313496280983169</v>
+        <v>0.06322418848124187</v>
       </c>
       <c r="J12" t="n">
-        <v>7.826424365586904</v>
+        <v>7.826424365588025</v>
       </c>
       <c r="K12" t="n">
-        <v>44.61693756824135</v>
+        <v>22.1702109901435</v>
       </c>
       <c r="L12" t="n">
-        <v>23.87134363826997</v>
+        <v>12.2448414360043</v>
       </c>
       <c r="M12" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2848518123993384</v>
+        <v>0.2544321025474922</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4234331242134844</v>
+        <v>0.3919477541924257</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>-2531.736016658554</v>
+        <v>-45.72736374796879</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -1042,36 +1042,36 @@
         <v>0.2</v>
       </c>
       <c r="G13" t="n">
-        <v>0.07286844709700199</v>
+        <v>0.07286844709700198</v>
       </c>
       <c r="H13" t="n">
-        <v>0.02790720992479427</v>
+        <v>0.04800447130510598</v>
       </c>
       <c r="I13" t="n">
-        <v>0.03057424287508246</v>
+        <v>0.05450029248318126</v>
       </c>
       <c r="J13" t="n">
-        <v>6.710793399280155</v>
+        <v>6.710793399280178</v>
       </c>
       <c r="K13" t="n">
-        <v>49.16932139687304</v>
+        <v>26.09575469145531</v>
       </c>
       <c r="L13" t="n">
-        <v>26.01320393376207</v>
+        <v>14.24324468664562</v>
       </c>
       <c r="M13" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N13" t="n">
-        <v>0.2790287267999395</v>
+        <v>0.2541642780266629</v>
       </c>
       <c r="O13" t="n">
-        <v>0.4167817271826546</v>
+        <v>0.3914336357929759</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>-1161.108944587921</v>
+        <v>-39.63908644434673</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -1089,36 +1089,36 @@
         <v>0.2</v>
       </c>
       <c r="G14" t="n">
-        <v>0.08290061396627721</v>
+        <v>0.08290061396627717</v>
       </c>
       <c r="H14" t="n">
-        <v>0.02572985725183476</v>
+        <v>0.03978100212799024</v>
       </c>
       <c r="I14" t="n">
-        <v>0.02639661125988538</v>
+        <v>0.04539021101180237</v>
       </c>
       <c r="J14" t="n">
-        <v>5.895611618411024</v>
+        <v>5.895611618411023</v>
       </c>
       <c r="K14" t="n">
-        <v>55.15243049106029</v>
+        <v>32.05968856678492</v>
       </c>
       <c r="L14" t="n">
-        <v>30.52999637204829</v>
+        <v>17.18275348436881</v>
       </c>
       <c r="M14" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2725500234315529</v>
+        <v>0.2535377147241192</v>
       </c>
       <c r="O14" t="n">
-        <v>0.4111435178813576</v>
+        <v>0.3905162661265826</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>-556.8623735593249</v>
+        <v>-20.18107573841761</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -1136,36 +1136,36 @@
         <v>0.2</v>
       </c>
       <c r="G15" t="n">
-        <v>0.09234950013810871</v>
+        <v>0.09234950013810869</v>
       </c>
       <c r="H15" t="n">
-        <v>0.02321426834521982</v>
+        <v>0.0322277231779966</v>
       </c>
       <c r="I15" t="n">
-        <v>0.02174490167971082</v>
+        <v>0.03757339780549244</v>
       </c>
       <c r="J15" t="n">
-        <v>5.290573350413696</v>
+        <v>5.290573350413733</v>
       </c>
       <c r="K15" t="n">
-        <v>65.45105093625541</v>
+        <v>40.93540226951551</v>
       </c>
       <c r="L15" t="n">
-        <v>38.07259559568786</v>
+        <v>20.90871609805017</v>
       </c>
       <c r="M15" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N15" t="n">
-        <v>0.2669259824426789</v>
+        <v>0.2522244320985457</v>
       </c>
       <c r="O15" t="n">
-        <v>0.4059257984205063</v>
+        <v>0.3879448417572579</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>-236.2261806954866</v>
+        <v>-2.153098315464545</v>
       </c>
       <c r="B16" t="n">
         <v>0</v>
@@ -1183,36 +1183,36 @@
         <v>0.2</v>
       </c>
       <c r="G16" t="n">
-        <v>0.09812542476084979</v>
+        <v>0.1009126975550351</v>
       </c>
       <c r="H16" t="n">
-        <v>0.02157302656359518</v>
+        <v>0.02596742250262566</v>
       </c>
       <c r="I16" t="n">
-        <v>0.01761750130197971</v>
+        <v>0.0295959087237158</v>
       </c>
       <c r="J16" t="n">
-        <v>4.978345196187929</v>
+        <v>4.840507364843452</v>
       </c>
       <c r="K16" t="n">
-        <v>78.1833984805164</v>
+        <v>54.40652760547253</v>
       </c>
       <c r="L16" t="n">
-        <v>49.56386557354645</v>
+        <v>26.94121412734315</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2262072674589311</v>
+        <v>0.223409733171147</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2612724658908461</v>
+        <v>0.2505763556566254</v>
       </c>
       <c r="O16" t="n">
-        <v>0.4008203022103162</v>
+        <v>0.3858630948126691</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>-4479.65975841318</v>
+        <v>-40.31992125185201</v>
       </c>
       <c r="B17" t="n">
         <v>90</v>
@@ -1230,36 +1230,36 @@
         <v>0.2</v>
       </c>
       <c r="G17" t="n">
-        <v>0.06253281370900748</v>
+        <v>0.06253281370900741</v>
       </c>
       <c r="H17" t="n">
-        <v>0.03006399501375714</v>
+        <v>0.05595688151536353</v>
       </c>
       <c r="I17" t="n">
-        <v>0.02851920413217641</v>
+        <v>0.04970492329672653</v>
       </c>
       <c r="J17" t="n">
-        <v>7.8264243655871</v>
+        <v>7.826424365586924</v>
       </c>
       <c r="K17" t="n">
-        <v>44.61693756824598</v>
+        <v>22.17021099014357</v>
       </c>
       <c r="L17" t="n">
-        <v>28.04607006302142</v>
+        <v>15.65094155307737</v>
       </c>
       <c r="M17" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N17" t="n">
-        <v>0.284851812399338</v>
+        <v>0.2544321025474923</v>
       </c>
       <c r="O17" t="n">
-        <v>0.4136996666497542</v>
+        <v>0.3910078371000422</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>-2305.44968284216</v>
+        <v>-39.33887274528486</v>
       </c>
       <c r="B18" t="n">
         <v>90</v>
@@ -1280,33 +1280,33 @@
         <v>0.07286844709700185</v>
       </c>
       <c r="H18" t="n">
-        <v>0.02790720992479427</v>
+        <v>0.04800447130510594</v>
       </c>
       <c r="I18" t="n">
-        <v>0.02459530715608716</v>
+        <v>0.0421113236984067</v>
       </c>
       <c r="J18" t="n">
-        <v>6.710793399280168</v>
+        <v>6.710793399280155</v>
       </c>
       <c r="K18" t="n">
-        <v>49.16932139687306</v>
+        <v>26.09575469145533</v>
       </c>
       <c r="L18" t="n">
-        <v>33.03787877491924</v>
+        <v>18.56755891430156</v>
       </c>
       <c r="M18" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N18" t="n">
-        <v>0.2790287267999395</v>
+        <v>0.2541642780266629</v>
       </c>
       <c r="O18" t="n">
-        <v>0.4091018053831032</v>
+        <v>0.3898009241227303</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>-1028.724753318432</v>
+        <v>-27.52462928252122</v>
       </c>
       <c r="B19" t="n">
         <v>90</v>
@@ -1327,33 +1327,33 @@
         <v>0.08290061396627714</v>
       </c>
       <c r="H19" t="n">
-        <v>0.02572985725183666</v>
+        <v>0.03978100212799029</v>
       </c>
       <c r="I19" t="n">
-        <v>0.02032138004719498</v>
+        <v>0.03528979645683913</v>
       </c>
       <c r="J19" t="n">
-        <v>5.895611618410962</v>
+        <v>5.89561161841103</v>
       </c>
       <c r="K19" t="n">
-        <v>55.15243049106395</v>
+        <v>32.05968856678502</v>
       </c>
       <c r="L19" t="n">
-        <v>41.28894329764329</v>
+        <v>22.33206031740519</v>
       </c>
       <c r="M19" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2725500234315539</v>
+        <v>0.2535377147241191</v>
       </c>
       <c r="O19" t="n">
-        <v>0.4042863613438415</v>
+        <v>0.3869127087255597</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>-474.4915109611006</v>
+        <v>-13.90185350732268</v>
       </c>
       <c r="B20" t="n">
         <v>90</v>
@@ -1371,36 +1371,36 @@
         <v>0.2</v>
       </c>
       <c r="G20" t="n">
-        <v>0.09234950013810857</v>
+        <v>0.09234950013810855</v>
       </c>
       <c r="H20" t="n">
-        <v>0.02321426834521983</v>
+        <v>0.03222772317787639</v>
       </c>
       <c r="I20" t="n">
-        <v>0.01652535488526957</v>
+        <v>0.02665758037485857</v>
       </c>
       <c r="J20" t="n">
-        <v>5.290573350413706</v>
+        <v>5.290573350413704</v>
       </c>
       <c r="K20" t="n">
-        <v>65.45105093625541</v>
+        <v>40.93540226955198</v>
       </c>
       <c r="L20" t="n">
-        <v>54.23605840643538</v>
+        <v>30.19976054138429</v>
       </c>
       <c r="M20" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N20" t="n">
-        <v>0.2669259824426789</v>
+        <v>0.2522244320986587</v>
       </c>
       <c r="O20" t="n">
-        <v>0.3991428189884212</v>
+        <v>0.3857614841158369</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>-183.1999680663905</v>
+        <v>-1.519994853728176</v>
       </c>
       <c r="B21" t="n">
         <v>90</v>
@@ -1418,36 +1418,36 @@
         <v>0.2</v>
       </c>
       <c r="G21" t="n">
-        <v>0.09812542476084977</v>
+        <v>0.1009126975550386</v>
       </c>
       <c r="H21" t="n">
-        <v>0.02157302656359518</v>
+        <v>0.02596742250262559</v>
       </c>
       <c r="I21" t="n">
-        <v>0.01414294855322185</v>
+        <v>0.01821530714797301</v>
       </c>
       <c r="J21" t="n">
-        <v>4.978345196187929</v>
+        <v>4.840507364843543</v>
       </c>
       <c r="K21" t="n">
-        <v>78.18339848051647</v>
+        <v>54.40652760547272</v>
       </c>
       <c r="L21" t="n">
-        <v>71.46308253930113</v>
+        <v>47.40447945853752</v>
       </c>
       <c r="M21" t="n">
-        <v>0.226207267458931</v>
+        <v>0.2234097331711433</v>
       </c>
       <c r="N21" t="n">
-        <v>0.2612724658908461</v>
+        <v>0.2505763556566254</v>
       </c>
       <c r="O21" t="n">
-        <v>0.3934431845374702</v>
+        <v>0.3856109933526596</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>-7942.700755824923</v>
+        <v>-85.26549178532147</v>
       </c>
       <c r="B22" t="n">
         <v>0</v>
@@ -1465,42 +1465,42 @@
         <v>0.4</v>
       </c>
       <c r="G22" t="n">
-        <v>0.06253281370900743</v>
+        <v>0.06253281370900744</v>
       </c>
       <c r="H22" t="n">
-        <v>0.02772933509037412</v>
+        <v>0.05374012161169844</v>
       </c>
       <c r="I22" t="n">
-        <v>0.02862771760056411</v>
+        <v>0.05950604742358118</v>
       </c>
       <c r="J22" t="n">
-        <v>7.826424365586963</v>
+        <v>7.826424365586918</v>
       </c>
       <c r="K22" t="n">
-        <v>49.59649998774761</v>
+        <v>23.13664256803835</v>
       </c>
       <c r="L22" t="n">
-        <v>27.93043147706909</v>
+        <v>13.02297658713481</v>
       </c>
       <c r="M22" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N22" t="n">
-        <v>0.288278694792366</v>
+        <v>0.2568340937002475</v>
       </c>
       <c r="O22" t="n">
-        <v>0.4284405309596223</v>
+        <v>0.3957580667631155</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>-2226.587989865454</v>
+        <v>-86.88670164475485</v>
       </c>
       <c r="B23" t="n">
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>-7.499999999999999</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -1512,42 +1512,42 @@
         <v>0.4</v>
       </c>
       <c r="G23" t="n">
-        <v>0.08290061396627718</v>
+        <v>0.07286844709700201</v>
       </c>
       <c r="H23" t="n">
-        <v>0.02349421346465825</v>
+        <v>0.04595012646737649</v>
       </c>
       <c r="I23" t="n">
-        <v>0.02057784671680623</v>
+        <v>0.05120329271662814</v>
       </c>
       <c r="J23" t="n">
-        <v>5.895611618411026</v>
+        <v>6.710793399280138</v>
       </c>
       <c r="K23" t="n">
-        <v>63.99662806959222</v>
+        <v>27.35733293447957</v>
       </c>
       <c r="L23" t="n">
-        <v>40.66481588404725</v>
+        <v>15.18173681976454</v>
       </c>
       <c r="M23" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2769515104344058</v>
+        <v>0.2564642165968263</v>
       </c>
       <c r="O23" t="n">
-        <v>0.4182715813990082</v>
+        <v>0.3948422864299632</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>-1082.452632861721</v>
+        <v>-72.43319315347468</v>
       </c>
       <c r="B24" t="n">
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>17.5</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -1559,42 +1559,42 @@
         <v>0.4</v>
       </c>
       <c r="G24" t="n">
-        <v>0.09234950013810868</v>
+        <v>0.08290061396627721</v>
       </c>
       <c r="H24" t="n">
-        <v>0.02177347643886305</v>
+        <v>0.0381314253233536</v>
       </c>
       <c r="I24" t="n">
-        <v>0.01698274223226202</v>
+        <v>0.04285382631742522</v>
       </c>
       <c r="J24" t="n">
-        <v>5.290573350413703</v>
+        <v>5.895611618411013</v>
       </c>
       <c r="K24" t="n">
-        <v>75.88237765094338</v>
+        <v>33.62570084422529</v>
       </c>
       <c r="L24" t="n">
-        <v>52.1460853822725</v>
+        <v>18.2344175377716</v>
       </c>
       <c r="M24" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N24" t="n">
-        <v>0.2712599853895694</v>
+        <v>0.255500932980732</v>
       </c>
       <c r="O24" t="n">
-        <v>0.4126225736338159</v>
+        <v>0.3931787010556945</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>-397.7594623838605</v>
+        <v>-33.1637748406988</v>
       </c>
       <c r="B25" t="n">
         <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>30</v>
+        <v>17.5</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -1606,42 +1606,42 @@
         <v>0.4</v>
       </c>
       <c r="G25" t="n">
-        <v>0.09812542476084979</v>
+        <v>0.09234950013810868</v>
       </c>
       <c r="H25" t="n">
-        <v>0.02119133890695252</v>
+        <v>0.0314336665143293</v>
       </c>
       <c r="I25" t="n">
-        <v>0.01465521452068975</v>
+        <v>0.03651965914549558</v>
       </c>
       <c r="J25" t="n">
-        <v>4.978345196187929</v>
+        <v>5.290573350413685</v>
       </c>
       <c r="K25" t="n">
-        <v>85.1625076387383</v>
+        <v>42.20298227902114</v>
       </c>
       <c r="L25" t="n">
-        <v>66.20259806645926</v>
+        <v>21.54165341987351</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2262072674589311</v>
+        <v>0.2233067431983749</v>
       </c>
       <c r="N25" t="n">
-        <v>0.2639031197810077</v>
+        <v>0.2532857203499647</v>
       </c>
       <c r="O25" t="n">
-        <v>0.4063335795359244</v>
+        <v>0.3890752455606723</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>-7353.539880398374</v>
+        <v>-4.250303122409941</v>
       </c>
       <c r="B26" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -1653,42 +1653,42 @@
         <v>0.4</v>
       </c>
       <c r="G26" t="n">
-        <v>0.06253281370900748</v>
+        <v>0.1009126975550357</v>
       </c>
       <c r="H26" t="n">
-        <v>0.02772933509037384</v>
+        <v>0.02584876085598064</v>
       </c>
       <c r="I26" t="n">
-        <v>0.02251854165364469</v>
+        <v>0.02932870132767481</v>
       </c>
       <c r="J26" t="n">
-        <v>7.826424365587121</v>
+        <v>4.840507364843524</v>
       </c>
       <c r="K26" t="n">
-        <v>49.59649998774825</v>
+        <v>54.77566620013775</v>
       </c>
       <c r="L26" t="n">
-        <v>36.54640546095656</v>
+        <v>27.20683075441296</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2233067431983749</v>
+        <v>0.2234097331711464</v>
       </c>
       <c r="N26" t="n">
-        <v>0.2882786947923663</v>
+        <v>0.2507811527364971</v>
       </c>
       <c r="O26" t="n">
-        <v>0.4207790257869182</v>
+        <v>0.386163185670981</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>-3812.375893807456</v>
+        <v>-76.42160455465887</v>
       </c>
       <c r="B27" t="n">
         <v>90</v>
       </c>
       <c r="C27" t="n">
-        <v>-7.499999999999999</v>
+        <v>-20</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1700,42 +1700,42 @@
         <v>0.4</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0728684470970019</v>
+        <v>0.06253281370900748</v>
       </c>
       <c r="H27" t="n">
-        <v>0.02581131741266296</v>
+        <v>0.05374012161169874</v>
       </c>
       <c r="I27" t="n">
-        <v>0.01907748368838032</v>
+        <v>0.04664983748305211</v>
       </c>
       <c r="J27" t="n">
-        <v>6.710793399280193</v>
+        <v>7.826424365587124</v>
       </c>
       <c r="K27" t="n">
-        <v>54.89355730716976</v>
+        <v>23.13664256803824</v>
       </c>
       <c r="L27" t="n">
-        <v>44.65859616303742</v>
+        <v>16.70497128283071</v>
       </c>
       <c r="M27" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N27" t="n">
-        <v>0.2824311641419652</v>
+        <v>0.2568340937002471</v>
       </c>
       <c r="O27" t="n">
-        <v>0.4161503463209285</v>
+        <v>0.3941887549969388</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>-1954.956392311966</v>
+        <v>-72.03220577624967</v>
       </c>
       <c r="B28" t="n">
         <v>90</v>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>-7.499999999999999</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -1747,42 +1747,42 @@
         <v>0.4</v>
       </c>
       <c r="G28" t="n">
-        <v>0.08290061396627715</v>
+        <v>0.0728684470970019</v>
       </c>
       <c r="H28" t="n">
-        <v>0.02349421346465825</v>
+        <v>0.04595012646737646</v>
       </c>
       <c r="I28" t="n">
-        <v>0.01607636507038104</v>
+        <v>0.04018724477812761</v>
       </c>
       <c r="J28" t="n">
-        <v>5.895611618411039</v>
+        <v>6.710793399280202</v>
       </c>
       <c r="K28" t="n">
-        <v>63.99662806959221</v>
+        <v>27.35733293447959</v>
       </c>
       <c r="L28" t="n">
-        <v>56.52160854456393</v>
+        <v>19.49156123182588</v>
       </c>
       <c r="M28" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N28" t="n">
-        <v>0.2769515104344058</v>
+        <v>0.2564642165968263</v>
       </c>
       <c r="O28" t="n">
-        <v>0.4106875892983801</v>
+        <v>0.3918361654489949</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>-905.119936479218</v>
+        <v>-50.69076862697345</v>
       </c>
       <c r="B29" t="n">
         <v>90</v>
       </c>
       <c r="C29" t="n">
-        <v>17.5</v>
+        <v>5</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -1794,42 +1794,42 @@
         <v>0.4</v>
       </c>
       <c r="G29" t="n">
-        <v>0.09234950013810854</v>
+        <v>0.08290061396627713</v>
       </c>
       <c r="H29" t="n">
-        <v>0.02177347643886305</v>
+        <v>0.03813142532335364</v>
       </c>
       <c r="I29" t="n">
-        <v>0.0142085460208135</v>
+        <v>0.03458725640844369</v>
       </c>
       <c r="J29" t="n">
-        <v>5.290573350413744</v>
+        <v>5.895611618411039</v>
       </c>
       <c r="K29" t="n">
-        <v>75.88237765094335</v>
+        <v>33.62570084422526</v>
       </c>
       <c r="L29" t="n">
-        <v>70.68974325507207</v>
+        <v>22.81095729597294</v>
       </c>
       <c r="M29" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N29" t="n">
-        <v>0.2712599853895694</v>
+        <v>0.255500932980732</v>
       </c>
       <c r="O29" t="n">
-        <v>0.4041024856881931</v>
+        <v>0.3876735198590205</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>-289.5314919251023</v>
+        <v>-23.68013476016145</v>
       </c>
       <c r="B30" t="n">
         <v>90</v>
       </c>
       <c r="C30" t="n">
-        <v>30</v>
+        <v>17.5</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -1841,89 +1841,89 @@
         <v>0.4</v>
       </c>
       <c r="G30" t="n">
-        <v>0.09812542476084979</v>
+        <v>0.09234950013810853</v>
       </c>
       <c r="H30" t="n">
-        <v>0.02119133890695253</v>
+        <v>0.03143366651432928</v>
       </c>
       <c r="I30" t="n">
-        <v>0.01352565415579918</v>
+        <v>0.02646993929768662</v>
       </c>
       <c r="J30" t="n">
-        <v>4.978345196187928</v>
+        <v>5.290573350413702</v>
       </c>
       <c r="K30" t="n">
-        <v>85.16250763873882</v>
+        <v>42.20298227902117</v>
       </c>
       <c r="L30" t="n">
-        <v>82.47595940972234</v>
+        <v>30.4364344503653</v>
       </c>
       <c r="M30" t="n">
-        <v>0.226207267458931</v>
+        <v>0.2233067431983749</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2639031197810077</v>
+        <v>0.2532857203499647</v>
       </c>
       <c r="O30" t="n">
-        <v>0.396168370245494</v>
+        <v>0.3859788529987433</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>-10609.04053570915</v>
+        <v>-3.042554373959004</v>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="C31" t="n">
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="F31" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G31" t="n">
-        <v>0.06253281370900611</v>
+        <v>0.1009126975550355</v>
       </c>
       <c r="H31" t="n">
-        <v>0.02651142301746443</v>
+        <v>0.02584876085598057</v>
       </c>
       <c r="I31" t="n">
-        <v>0.02502861110400405</v>
+        <v>0.01816163491303752</v>
       </c>
       <c r="J31" t="n">
-        <v>7.826424365587974</v>
+        <v>4.840507364843425</v>
       </c>
       <c r="K31" t="n">
-        <v>52.79539415996996</v>
+        <v>54.77566620013794</v>
       </c>
       <c r="L31" t="n">
-        <v>32.39511412200125</v>
+        <v>47.5889694326049</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2233067431983749</v>
+        <v>0.2234097331711464</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2902214382562732</v>
+        <v>0.2507811527364971</v>
       </c>
       <c r="O31" t="n">
-        <v>0.4326001065570714</v>
+        <v>0.3856904333205084</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>-6026.663951565098</v>
+        <v>-125.5917593119504</v>
       </c>
       <c r="B32" t="n">
         <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>-7.499999999999999</v>
+        <v>-20</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -1935,42 +1935,42 @@
         <v>0.6</v>
       </c>
       <c r="G32" t="n">
-        <v>0.07286844709700203</v>
+        <v>0.06253281370900741</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0244825873719785</v>
+        <v>0.05206181221762846</v>
       </c>
       <c r="I32" t="n">
-        <v>0.02124336959630156</v>
+        <v>0.05693004634218402</v>
       </c>
       <c r="J32" t="n">
-        <v>6.710793399280195</v>
+        <v>7.826424365586893</v>
       </c>
       <c r="K32" t="n">
-        <v>59.59670163167768</v>
+        <v>23.92822840330427</v>
       </c>
       <c r="L32" t="n">
-        <v>39.14004545936502</v>
+        <v>13.62334758109314</v>
       </c>
       <c r="M32" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2848849502594457</v>
+        <v>0.2586645984557456</v>
       </c>
       <c r="O32" t="n">
-        <v>0.4277821125515866</v>
+        <v>0.3984052801340791</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>-3294.246709557159</v>
+        <v>-124.9726806302841</v>
       </c>
       <c r="B33" t="n">
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>-7.499999999999999</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1982,42 +1982,42 @@
         <v>0.6</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0829006139662772</v>
+        <v>0.07286844709700199</v>
       </c>
       <c r="H33" t="n">
-        <v>0.02242510796144937</v>
+        <v>0.04451004594634804</v>
       </c>
       <c r="I33" t="n">
-        <v>0.01768187717160039</v>
+        <v>0.04888505038247909</v>
       </c>
       <c r="J33" t="n">
-        <v>5.895611618410955</v>
+        <v>6.710793399280178</v>
       </c>
       <c r="K33" t="n">
-        <v>70.32483318693576</v>
+        <v>28.32071128784097</v>
       </c>
       <c r="L33" t="n">
-        <v>49.31968249202471</v>
+        <v>15.92033848923318</v>
       </c>
       <c r="M33" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N33" t="n">
-        <v>0.2797016922254016</v>
+        <v>0.2580927246502468</v>
       </c>
       <c r="O33" t="n">
-        <v>0.4223548726301237</v>
+        <v>0.3972485697777062</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>-1475.066020118312</v>
+        <v>-99.98753074873744</v>
       </c>
       <c r="B34" t="n">
         <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>17.5</v>
+        <v>5</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -2029,42 +2029,42 @@
         <v>0.6</v>
       </c>
       <c r="G34" t="n">
-        <v>0.09234950013810865</v>
+        <v>0.08290061396627717</v>
       </c>
       <c r="H34" t="n">
-        <v>0.02137004550449095</v>
+        <v>0.03697816719470168</v>
       </c>
       <c r="I34" t="n">
-        <v>0.01510333322500559</v>
+        <v>0.04131635721642449</v>
       </c>
       <c r="J34" t="n">
-        <v>5.290573350413684</v>
+        <v>5.895611618411033</v>
       </c>
       <c r="K34" t="n">
-        <v>81.15398477784365</v>
+        <v>34.82247882547946</v>
       </c>
       <c r="L34" t="n">
-        <v>62.60186934838094</v>
+        <v>18.93827692002484</v>
       </c>
       <c r="M34" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N34" t="n">
-        <v>0.2732845520766336</v>
+        <v>0.256895627735593</v>
       </c>
       <c r="O34" t="n">
-        <v>0.4160939254286245</v>
+        <v>0.3948007395673536</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>-480.3956493118317</v>
+        <v>-42.8854590676124</v>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>30</v>
+        <v>17.5</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -2076,42 +2076,42 @@
         <v>0.6</v>
       </c>
       <c r="G35" t="n">
-        <v>0.09812542476084977</v>
+        <v>0.09234950013810866</v>
       </c>
       <c r="H35" t="n">
-        <v>0.02113584368080331</v>
+        <v>0.03090256973461742</v>
       </c>
       <c r="I35" t="n">
-        <v>0.01385287525926209</v>
+        <v>0.03584782017393869</v>
       </c>
       <c r="J35" t="n">
-        <v>4.978345196187929</v>
+        <v>5.290573350413677</v>
       </c>
       <c r="K35" t="n">
-        <v>87.50784204646014</v>
+        <v>43.10238083566317</v>
       </c>
       <c r="L35" t="n">
-        <v>75.45991101892949</v>
+        <v>21.96616282057354</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2262072674589311</v>
+        <v>0.2233067431983749</v>
       </c>
       <c r="N35" t="n">
-        <v>0.2647711407334568</v>
+        <v>0.2540078126664956</v>
       </c>
       <c r="O35" t="n">
-        <v>0.4087691483660179</v>
+        <v>0.3897985936830507</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>-9753.597717995674</v>
+        <v>-6.198986441339853</v>
       </c>
       <c r="B36" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -2123,42 +2123,42 @@
         <v>0.6</v>
       </c>
       <c r="G36" t="n">
-        <v>0.06253281370900618</v>
+        <v>0.100912697555038</v>
       </c>
       <c r="H36" t="n">
-        <v>0.02651142301746442</v>
+        <v>0.02574301647282795</v>
       </c>
       <c r="I36" t="n">
-        <v>0.01928677081953861</v>
+        <v>0.02908495983905614</v>
       </c>
       <c r="J36" t="n">
-        <v>7.826424365587958</v>
+        <v>4.84050736484353</v>
       </c>
       <c r="K36" t="n">
-        <v>52.79539415996997</v>
+        <v>55.11038694463961</v>
       </c>
       <c r="L36" t="n">
-        <v>44.04743559135235</v>
+        <v>27.45394522316143</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2233067431983749</v>
+        <v>0.223409733171144</v>
       </c>
       <c r="N36" t="n">
-        <v>0.2902214382562732</v>
+        <v>0.2509652503076515</v>
       </c>
       <c r="O36" t="n">
-        <v>0.4250072103846321</v>
+        <v>0.3864375531806787</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>-5407.539851624317</v>
+        <v>-111.251353859879</v>
       </c>
       <c r="B37" t="n">
         <v>90</v>
       </c>
       <c r="C37" t="n">
-        <v>-7.499999999999999</v>
+        <v>-20</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -2170,42 +2170,42 @@
         <v>0.6</v>
       </c>
       <c r="G37" t="n">
-        <v>0.07286844709700187</v>
+        <v>0.06253281370900605</v>
       </c>
       <c r="H37" t="n">
-        <v>0.02448258737197851</v>
+        <v>0.05206181221762816</v>
       </c>
       <c r="I37" t="n">
-        <v>0.01653299075214278</v>
+        <v>0.04461769208977838</v>
       </c>
       <c r="J37" t="n">
-        <v>6.710793399280137</v>
+        <v>7.826424365587995</v>
       </c>
       <c r="K37" t="n">
-        <v>59.59670163167765</v>
+        <v>23.92822840330438</v>
       </c>
       <c r="L37" t="n">
-        <v>54.19933498041483</v>
+        <v>17.48976658697976</v>
       </c>
       <c r="M37" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N37" t="n">
-        <v>0.2848849502594456</v>
+        <v>0.2586645984557459</v>
       </c>
       <c r="O37" t="n">
-        <v>0.4200490496954367</v>
+        <v>0.3963148105333875</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>-2869.89946169388</v>
+        <v>-100.6355298706408</v>
       </c>
       <c r="B38" t="n">
         <v>90</v>
       </c>
       <c r="C38" t="n">
-        <v>5</v>
+        <v>-7.499999999999999</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -2217,42 +2217,42 @@
         <v>0.6</v>
       </c>
       <c r="G38" t="n">
-        <v>0.0829006139662771</v>
+        <v>0.07286844709700191</v>
       </c>
       <c r="H38" t="n">
-        <v>0.02242510796158142</v>
+        <v>0.04451004594627694</v>
       </c>
       <c r="I38" t="n">
-        <v>0.01456581593808897</v>
+        <v>0.03904829209155171</v>
       </c>
       <c r="J38" t="n">
-        <v>5.89561161841096</v>
+        <v>6.710793399280208</v>
       </c>
       <c r="K38" t="n">
-        <v>70.32483318693421</v>
+        <v>28.32071128788252</v>
       </c>
       <c r="L38" t="n">
-        <v>67.01303150825024</v>
+        <v>20.08417960251273</v>
       </c>
       <c r="M38" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N38" t="n">
-        <v>0.279701692225375</v>
+        <v>0.2580927246503267</v>
       </c>
       <c r="O38" t="n">
-        <v>0.4138674052310957</v>
+        <v>0.3930465745880456</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>-1206.696558243405</v>
+        <v>-71.14169096162492</v>
       </c>
       <c r="B39" t="n">
         <v>90</v>
       </c>
       <c r="C39" t="n">
-        <v>17.5</v>
+        <v>5</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -2264,42 +2264,42 @@
         <v>0.6</v>
       </c>
       <c r="G39" t="n">
-        <v>0.09234950013810853</v>
+        <v>0.08290061396627713</v>
       </c>
       <c r="H39" t="n">
-        <v>0.02137004550449095</v>
+        <v>0.03697816719472797</v>
       </c>
       <c r="I39" t="n">
-        <v>0.01366910147652461</v>
+        <v>0.0340953895554933</v>
       </c>
       <c r="J39" t="n">
-        <v>5.290573350413721</v>
+        <v>5.895611618411018</v>
       </c>
       <c r="K39" t="n">
-        <v>81.15398477784368</v>
+        <v>34.82247882546618</v>
       </c>
       <c r="L39" t="n">
-        <v>78.80912791553065</v>
+        <v>23.1590441140087</v>
       </c>
       <c r="M39" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N39" t="n">
-        <v>0.2732845520766336</v>
+        <v>0.2568956277355651</v>
       </c>
       <c r="O39" t="n">
-        <v>0.4061481423145948</v>
+        <v>0.3882078027014921</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>-333.4685346264427</v>
+        <v>-31.32232852951972</v>
       </c>
       <c r="B40" t="n">
         <v>90</v>
       </c>
       <c r="C40" t="n">
-        <v>30</v>
+        <v>17.5</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -2311,36 +2311,36 @@
         <v>0.6</v>
       </c>
       <c r="G40" t="n">
-        <v>0.09812542476084979</v>
+        <v>0.09234950013810853</v>
       </c>
       <c r="H40" t="n">
-        <v>0.02113584368080329</v>
+        <v>0.03090256973461725</v>
       </c>
       <c r="I40" t="n">
-        <v>0.01343900646455607</v>
+        <v>0.02629358878188278</v>
       </c>
       <c r="J40" t="n">
-        <v>4.978345196187929</v>
+        <v>5.290573350413688</v>
       </c>
       <c r="K40" t="n">
-        <v>87.50784204646015</v>
+        <v>43.10238083566342</v>
       </c>
       <c r="L40" t="n">
-        <v>86.18318174783947</v>
+        <v>30.66248226215295</v>
       </c>
       <c r="M40" t="n">
-        <v>0.226207267458931</v>
+        <v>0.2233067431983749</v>
       </c>
       <c r="N40" t="n">
-        <v>0.2647711407334566</v>
+        <v>0.2540078126664956</v>
       </c>
       <c r="O40" t="n">
-        <v>0.3970448573985396</v>
+        <v>0.3861836278148428</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>-52.73779622848618</v>
+        <v>-3.655407251398808</v>
       </c>
       <c r="B41" t="n">
         <v>0</v>
@@ -2358,36 +2358,36 @@
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0.04894223553167541</v>
+        <v>0.06081899508304547</v>
       </c>
       <c r="H41" t="n">
-        <v>0.05010332837588985</v>
+        <v>0.05879831855403968</v>
       </c>
       <c r="I41" t="n">
-        <v>0.06205666365794649</v>
+        <v>0.06870583418284261</v>
       </c>
       <c r="J41" t="n">
-        <v>10.01963682927531</v>
+        <v>8.048406845249401</v>
       </c>
       <c r="K41" t="n">
-        <v>24.92592040365766</v>
+        <v>21.04637177577536</v>
       </c>
       <c r="L41" t="n">
-        <v>12.47889102060729</v>
+        <v>11.25455325771339</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2370612953379955</v>
+        <v>0.2250371366478509</v>
       </c>
       <c r="N41" t="n">
-        <v>0.2608155426261001</v>
+        <v>0.2513760312601033</v>
       </c>
       <c r="O41" t="n">
-        <v>0.3931429881010704</v>
+        <v>0.3863489999533454</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>188.9640024532025</v>
+        <v>5.557509309267517</v>
       </c>
       <c r="B42" t="n">
         <v>0</v>
@@ -2405,28 +2405,28 @@
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0.05409016632291627</v>
+        <v>0.07001701422114186</v>
       </c>
       <c r="H42" t="n">
-        <v>0.05000784024966509</v>
+        <v>0.05137435493611166</v>
       </c>
       <c r="I42" t="n">
-        <v>0.06024037485416459</v>
+        <v>0.06024037485416532</v>
       </c>
       <c r="J42" t="n">
-        <v>9.057577133901955</v>
+        <v>6.985424616815118</v>
       </c>
       <c r="K42" t="n">
-        <v>24.9767747981245</v>
+        <v>24.26888371725413</v>
       </c>
       <c r="L42" t="n">
-        <v>12.86148801950237</v>
+        <v>12.86148801950014</v>
       </c>
       <c r="M42" t="n">
-        <v>0.2422602467840607</v>
+        <v>0.2261786568671618</v>
       </c>
       <c r="N42" t="n">
-        <v>0.2519441235097181</v>
+        <v>0.2504409517469713</v>
       </c>
       <c r="O42" t="n">
         <v>0.3855295790644589</v>
@@ -2434,7 +2434,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>445.6554147026658</v>
+        <v>6.884734885084504</v>
       </c>
       <c r="B43" t="n">
         <v>0</v>
@@ -2452,25 +2452,25 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>0.05886817512122013</v>
+        <v>0.07963111756833033</v>
       </c>
       <c r="H43" t="n">
-        <v>0.04252156896056231</v>
+        <v>0.04252156861879716</v>
       </c>
       <c r="I43" t="n">
-        <v>0.05017595975374158</v>
+        <v>0.05017595975381756</v>
       </c>
       <c r="J43" t="n">
-        <v>8.316979524372186</v>
+        <v>6.138585663218899</v>
       </c>
       <c r="K43" t="n">
-        <v>29.77475571091729</v>
+        <v>29.7747560647992</v>
       </c>
       <c r="L43" t="n">
-        <v>15.50030379111149</v>
+        <v>15.50030379108468</v>
       </c>
       <c r="M43" t="n">
-        <v>0.2475198133769966</v>
+        <v>0.2265943447717173</v>
       </c>
       <c r="N43" t="n">
         <v>0.2503438825093889</v>
@@ -2481,7 +2481,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>753.2746861014057</v>
+        <v>7.101596894685658</v>
       </c>
       <c r="B44" t="n">
         <v>0</v>
@@ -2499,25 +2499,25 @@
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>0.06455272573734153</v>
+        <v>0.08879812259790099</v>
       </c>
       <c r="H44" t="n">
-        <v>0.0336709333313158</v>
+        <v>0.03367092754744086</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0398389417216387</v>
+        <v>0.03983894172329831</v>
       </c>
       <c r="J44" t="n">
-        <v>7.580066048374966</v>
+        <v>5.502803974491978</v>
       </c>
       <c r="K44" t="n">
-        <v>38.83826008892519</v>
+        <v>38.83827133840433</v>
       </c>
       <c r="L44" t="n">
-        <v>19.66896230593819</v>
+        <v>19.66896230534421</v>
       </c>
       <c r="M44" t="n">
-        <v>0.2512741922203449</v>
+        <v>0.2268739265381451</v>
       </c>
       <c r="N44" t="n">
         <v>0.2503438825093889</v>
@@ -2528,7 +2528,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>914.1806155708947</v>
+        <v>6.804128092397171</v>
       </c>
       <c r="B45" t="n">
         <v>0</v>
@@ -2546,25 +2546,25 @@
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0.07134225588996737</v>
+        <v>0.09730058997241224</v>
       </c>
       <c r="H45" t="n">
-        <v>0.02610341213841486</v>
+        <v>0.02610341344139298</v>
       </c>
       <c r="I45" t="n">
-        <v>0.02989360655907775</v>
+        <v>0.02989360514136771</v>
       </c>
       <c r="J45" t="n">
-        <v>6.855035846997247</v>
+        <v>5.020655423512832</v>
       </c>
       <c r="K45" t="n">
-        <v>53.99158788151775</v>
+        <v>53.99159103998766</v>
       </c>
       <c r="L45" t="n">
-        <v>26.65159425253778</v>
+        <v>26.65159555175514</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2531302679849247</v>
+        <v>0.2270352522940929</v>
       </c>
       <c r="N45" t="n">
         <v>0.2503438825093872</v>
@@ -2575,7 +2575,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>-29.95237704935441</v>
+        <v>-1.889640618938181</v>
       </c>
       <c r="B46" t="n">
         <v>90</v>
@@ -2593,28 +2593,28 @@
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0.04894223553167538</v>
+        <v>0.06081899508307646</v>
       </c>
       <c r="H46" t="n">
-        <v>0.05010332837588984</v>
+        <v>0.05879831855407185</v>
       </c>
       <c r="I46" t="n">
-        <v>0.05499992440104685</v>
+        <v>0.05499992440104683</v>
       </c>
       <c r="J46" t="n">
-        <v>10.01963682927531</v>
+        <v>8.048406845232289</v>
       </c>
       <c r="K46" t="n">
-        <v>24.92592040365766</v>
+        <v>21.04637177567111</v>
       </c>
       <c r="L46" t="n">
-        <v>14.11116142850724</v>
+        <v>14.11116142850683</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2370612953379956</v>
+        <v>0.2250371366478364</v>
       </c>
       <c r="N46" t="n">
-        <v>0.2608155426261001</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O46" t="n">
         <v>0.3855295790644589</v>
@@ -2622,7 +2622,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>188.9640024550826</v>
+        <v>5.55750930685076</v>
       </c>
       <c r="B47" t="n">
         <v>90</v>
@@ -2640,28 +2640,28 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>0.05409016632291208</v>
+        <v>0.07001701422114175</v>
       </c>
       <c r="H47" t="n">
-        <v>0.05000784024966202</v>
+        <v>0.05137435493531307</v>
       </c>
       <c r="I47" t="n">
-        <v>0.04618037325665472</v>
+        <v>0.04618037325657966</v>
       </c>
       <c r="J47" t="n">
-        <v>9.05757713390269</v>
+        <v>6.985424616815129</v>
       </c>
       <c r="K47" t="n">
-        <v>24.97677479812686</v>
+        <v>24.2688837173064</v>
       </c>
       <c r="L47" t="n">
-        <v>16.87985375457368</v>
+        <v>16.87985375460553</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2422602467840648</v>
+        <v>0.2261786568671618</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2519441235097216</v>
+        <v>0.2504409517474094</v>
       </c>
       <c r="O47" t="n">
         <v>0.3855295790644589</v>
@@ -2669,7 +2669,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>445.6554147026663</v>
+        <v>6.88473488508447</v>
       </c>
       <c r="B48" t="n">
         <v>90</v>
@@ -2687,25 +2687,25 @@
         <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>0.05886817512121938</v>
+        <v>0.07963111756833031</v>
       </c>
       <c r="H48" t="n">
-        <v>0.042521569140039</v>
+        <v>0.04252156849193505</v>
       </c>
       <c r="I48" t="n">
-        <v>0.03657296385902965</v>
+        <v>0.0365729638148084</v>
       </c>
       <c r="J48" t="n">
-        <v>8.316979524372259</v>
+        <v>6.138585663218901</v>
       </c>
       <c r="K48" t="n">
-        <v>29.77475551434732</v>
+        <v>29.77475620664449</v>
       </c>
       <c r="L48" t="n">
-        <v>21.50869233433809</v>
+        <v>21.50869236001778</v>
       </c>
       <c r="M48" t="n">
-        <v>0.2475198133769972</v>
+        <v>0.2265943447717173</v>
       </c>
       <c r="N48" t="n">
         <v>0.2503438825093889</v>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>753.2746861023015</v>
+        <v>7.101596894692407</v>
       </c>
       <c r="B49" t="n">
         <v>90</v>
@@ -2734,28 +2734,28 @@
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>0.06455272573731528</v>
+        <v>0.08879812259790087</v>
       </c>
       <c r="H49" t="n">
-        <v>0.03367093419842811</v>
+        <v>0.03367093022427217</v>
       </c>
       <c r="I49" t="n">
-        <v>0.02685826388011667</v>
+        <v>0.02685826388012517</v>
       </c>
       <c r="J49" t="n">
-        <v>7.580066048377501</v>
+        <v>5.502803974491985</v>
       </c>
       <c r="K49" t="n">
-        <v>38.83825833721282</v>
+        <v>38.83826623782915</v>
       </c>
       <c r="L49" t="n">
-        <v>29.95091013268099</v>
+        <v>29.95091013275769</v>
       </c>
       <c r="M49" t="n">
-        <v>0.2512741922203712</v>
+        <v>0.2268739265381451</v>
       </c>
       <c r="N49" t="n">
-        <v>0.2503438825093872</v>
+        <v>0.2503438825093889</v>
       </c>
       <c r="O49" t="n">
         <v>0.3855295790644563</v>
@@ -2763,7 +2763,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>914.1806155708972</v>
+        <v>6.80412809240373</v>
       </c>
       <c r="B50" t="n">
         <v>90</v>
@@ -2781,25 +2781,25 @@
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0.07134225588996729</v>
+        <v>0.09730058997241217</v>
       </c>
       <c r="H50" t="n">
-        <v>0.0261034134414413</v>
+        <v>0.0261034134414523</v>
       </c>
       <c r="I50" t="n">
-        <v>0.01827050656380773</v>
+        <v>0.01827050818593128</v>
       </c>
       <c r="J50" t="n">
-        <v>6.855035846997257</v>
+        <v>5.020655423512836</v>
       </c>
       <c r="K50" t="n">
-        <v>53.99159103982687</v>
+        <v>53.99159103978782</v>
       </c>
       <c r="L50" t="n">
-        <v>47.21651887993671</v>
+        <v>47.21653013893759</v>
       </c>
       <c r="M50" t="n">
-        <v>0.2531302679849247</v>
+        <v>0.2270352522940929</v>
       </c>
       <c r="N50" t="n">
         <v>0.2503438825093872</v>
@@ -2810,7 +2810,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>73.68799423156585</v>
+        <v>-1.095359070369122</v>
       </c>
       <c r="B51" t="n">
         <v>0</v>
@@ -2828,36 +2828,36 @@
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>0.04360229518764636</v>
+        <v>0.0597754606461906</v>
       </c>
       <c r="H51" t="n">
-        <v>0.0501033283758902</v>
+        <v>0.05879831855406242</v>
       </c>
       <c r="I51" t="n">
-        <v>0.06205666365794564</v>
+        <v>0.06870583418291323</v>
       </c>
       <c r="J51" t="n">
-        <v>11.26187448899634</v>
+        <v>8.189868841214489</v>
       </c>
       <c r="K51" t="n">
-        <v>24.92592040365738</v>
+        <v>21.04637177567383</v>
       </c>
       <c r="L51" t="n">
-        <v>12.47889102060754</v>
+        <v>11.25455325771749</v>
       </c>
       <c r="M51" t="n">
-        <v>0.2424943473075481</v>
+        <v>0.226091236013598</v>
       </c>
       <c r="N51" t="n">
-        <v>0.2608155426260997</v>
+        <v>0.2513760312601757</v>
       </c>
       <c r="O51" t="n">
-        <v>0.3931429881010713</v>
+        <v>0.3863489999532742</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>373.8257762250587</v>
+        <v>10.93107156790965</v>
       </c>
       <c r="B52" t="n">
         <v>0</v>
@@ -2875,28 +2875,28 @@
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>0.05011308029999553</v>
+        <v>0.06826064423159683</v>
       </c>
       <c r="H52" t="n">
-        <v>0.05000784024966213</v>
+        <v>0.05137435493611001</v>
       </c>
       <c r="I52" t="n">
-        <v>0.0602403748541654</v>
+        <v>0.06024037485416543</v>
       </c>
       <c r="J52" t="n">
-        <v>9.783207071455124</v>
+        <v>7.166093084702359</v>
       </c>
       <c r="K52" t="n">
-        <v>24.97677479812678</v>
+        <v>24.26888371725536</v>
       </c>
       <c r="L52" t="n">
-        <v>12.86148801950034</v>
+        <v>12.86148801950031</v>
       </c>
       <c r="M52" t="n">
-        <v>0.246291620294762</v>
+        <v>0.2279485035725401</v>
       </c>
       <c r="N52" t="n">
-        <v>0.2519441235097215</v>
+        <v>0.2504409517469746</v>
       </c>
       <c r="O52" t="n">
         <v>0.3855295790644589</v>
@@ -2904,7 +2904,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>865.5590357549554</v>
+        <v>13.41554358600072</v>
       </c>
       <c r="B53" t="n">
         <v>0</v>
@@ -2922,25 +2922,25 @@
         <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>0.05475519700192417</v>
+        <v>0.07758019783380794</v>
       </c>
       <c r="H53" t="n">
-        <v>0.04252156894281751</v>
+        <v>0.04252156913998491</v>
       </c>
       <c r="I53" t="n">
-        <v>0.05017595975382197</v>
+        <v>0.05017595975382195</v>
       </c>
       <c r="J53" t="n">
-        <v>8.946659483326565</v>
+        <v>6.301514994819789</v>
       </c>
       <c r="K53" t="n">
-        <v>29.774755726359</v>
+        <v>29.77475551439551</v>
       </c>
       <c r="L53" t="n">
-        <v>15.50030379108009</v>
+        <v>15.50030379108002</v>
       </c>
       <c r="M53" t="n">
-        <v>0.2516798493657056</v>
+        <v>0.2286574074576231</v>
       </c>
       <c r="N53" t="n">
         <v>0.2503438825093889</v>
@@ -2951,7 +2951,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1752.454262548912</v>
+        <v>13.87773016767401</v>
       </c>
       <c r="B54" t="n">
         <v>0</v>
@@ -2969,28 +2969,28 @@
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>0.05926908052693579</v>
+        <v>0.08662349307731694</v>
       </c>
       <c r="H54" t="n">
-        <v>0.03367093419831405</v>
+        <v>0.0336709283629596</v>
       </c>
       <c r="I54" t="n">
-        <v>0.0398389416828507</v>
+        <v>0.03983894171491816</v>
       </c>
       <c r="J54" t="n">
-        <v>8.26032775589249</v>
+        <v>5.641391091044853</v>
       </c>
       <c r="K54" t="n">
-        <v>38.83825833683237</v>
+        <v>38.83826955727122</v>
       </c>
       <c r="L54" t="n">
-        <v>19.66896232462202</v>
+        <v>19.66896230913706</v>
       </c>
       <c r="M54" t="n">
-        <v>0.2566086297859878</v>
+        <v>0.2290588787963555</v>
       </c>
       <c r="N54" t="n">
-        <v>0.2503438825093872</v>
+        <v>0.2503438825093889</v>
       </c>
       <c r="O54" t="n">
         <v>0.3855295790644589</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2714.332296520763</v>
+        <v>13.4879342283176</v>
       </c>
       <c r="B55" t="n">
         <v>0</v>
@@ -3016,25 +3016,25 @@
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>0.06450223574079157</v>
+        <v>0.09500775693448212</v>
       </c>
       <c r="H55" t="n">
-        <v>0.0261034134413365</v>
+        <v>0.02610341043280203</v>
       </c>
       <c r="I55" t="n">
-        <v>0.02989360839898388</v>
+        <v>0.02989360187463532</v>
       </c>
       <c r="J55" t="n">
-        <v>7.586034349438881</v>
+        <v>5.142141953979941</v>
       </c>
       <c r="K55" t="n">
-        <v>53.99159104017117</v>
+        <v>53.99158363573753</v>
       </c>
       <c r="L55" t="n">
-        <v>26.65159276910841</v>
+        <v>26.65159814768304</v>
       </c>
       <c r="M55" t="n">
-        <v>0.2600248247441578</v>
+        <v>0.2293371307184592</v>
       </c>
       <c r="N55" t="n">
         <v>0.2503438825093872</v>
@@ -3045,7 +3045,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>96.47341340949858</v>
+        <v>0.6704075623623933</v>
       </c>
       <c r="B56" t="n">
         <v>90</v>
@@ -3063,28 +3063,28 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0.04360229518768486</v>
+        <v>0.05977546064619061</v>
       </c>
       <c r="H56" t="n">
-        <v>0.05010332837589129</v>
+        <v>0.05879831855407185</v>
       </c>
       <c r="I56" t="n">
-        <v>0.05499992440102419</v>
+        <v>0.05499992440104687</v>
       </c>
       <c r="J56" t="n">
-        <v>11.26187448900586</v>
+        <v>8.189868841214487</v>
       </c>
       <c r="K56" t="n">
-        <v>24.92592040365651</v>
+        <v>21.04637177567111</v>
       </c>
       <c r="L56" t="n">
-        <v>14.11116142851763</v>
+        <v>14.11116142850724</v>
       </c>
       <c r="M56" t="n">
-        <v>0.242494347307507</v>
+        <v>0.226091236013598</v>
       </c>
       <c r="N56" t="n">
-        <v>0.2608155426260984</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O56" t="n">
         <v>0.3855295790644589</v>
@@ -3092,7 +3092,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>373.8257762250608</v>
+        <v>10.93107156757111</v>
       </c>
       <c r="B57" t="n">
         <v>90</v>
@@ -3110,28 +3110,28 @@
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>0.05011308029999508</v>
+        <v>0.06826064423154656</v>
       </c>
       <c r="H57" t="n">
-        <v>0.05000784024966212</v>
+        <v>0.05137435493593547</v>
       </c>
       <c r="I57" t="n">
-        <v>0.04618037325663057</v>
+        <v>0.04618037325310269</v>
       </c>
       <c r="J57" t="n">
-        <v>9.783207071456047</v>
+        <v>7.166093084705172</v>
       </c>
       <c r="K57" t="n">
-        <v>24.97677479812679</v>
+        <v>24.26888371726409</v>
       </c>
       <c r="L57" t="n">
-        <v>16.87985375458472</v>
+        <v>16.87985375580388</v>
       </c>
       <c r="M57" t="n">
-        <v>0.2462916202947623</v>
+        <v>0.2279485035725902</v>
       </c>
       <c r="N57" t="n">
-        <v>0.2519441235097215</v>
+        <v>0.2504409517470676</v>
       </c>
       <c r="O57" t="n">
         <v>0.3855295790644589</v>
@@ -3139,7 +3139,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>865.5590357549556</v>
+        <v>13.41554358600082</v>
       </c>
       <c r="B58" t="n">
         <v>90</v>
@@ -3157,25 +3157,25 @@
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0.05475519700192417</v>
+        <v>0.07758019783380786</v>
       </c>
       <c r="H58" t="n">
-        <v>0.04252156875860854</v>
+        <v>0.04252156878117114</v>
       </c>
       <c r="I58" t="n">
-        <v>0.03657296380664613</v>
+        <v>0.03657296386974299</v>
       </c>
       <c r="J58" t="n">
-        <v>8.946659483326563</v>
+        <v>6.301514994819796</v>
       </c>
       <c r="K58" t="n">
-        <v>29.77475591951258</v>
+        <v>29.7747559002623</v>
       </c>
       <c r="L58" t="n">
-        <v>21.50869236355778</v>
+        <v>21.50869232775635</v>
       </c>
       <c r="M58" t="n">
-        <v>0.2516798493657056</v>
+        <v>0.2286574074576231</v>
       </c>
       <c r="N58" t="n">
         <v>0.2503438825093889</v>
@@ -3186,7 +3186,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1752.454262548894</v>
+        <v>13.87773016769158</v>
       </c>
       <c r="B59" t="n">
         <v>90</v>
@@ -3204,25 +3204,25 @@
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>0.05926908052693571</v>
+        <v>0.08662349307731682</v>
       </c>
       <c r="H59" t="n">
-        <v>0.03367093419806941</v>
+        <v>0.03367093419828415</v>
       </c>
       <c r="I59" t="n">
-        <v>0.02685826388012444</v>
+        <v>0.02685826388012501</v>
       </c>
       <c r="J59" t="n">
-        <v>8.260327755892503</v>
+        <v>5.64139109104486</v>
       </c>
       <c r="K59" t="n">
-        <v>38.8382583359868</v>
+        <v>38.83825833674</v>
       </c>
       <c r="L59" t="n">
-        <v>29.95091013275031</v>
+        <v>29.95091013275585</v>
       </c>
       <c r="M59" t="n">
-        <v>0.2566086297859877</v>
+        <v>0.2290588787963555</v>
       </c>
       <c r="N59" t="n">
         <v>0.2503438825093872</v>
@@ -3233,7 +3233,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>2714.332296520361</v>
+        <v>13.48793422832416</v>
       </c>
       <c r="B60" t="n">
         <v>90</v>
@@ -3251,25 +3251,25 @@
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>0.06450223574079476</v>
+        <v>0.09500775693448203</v>
       </c>
       <c r="H60" t="n">
-        <v>0.02610341214368897</v>
+        <v>0.02610341344138608</v>
       </c>
       <c r="I60" t="n">
-        <v>0.01827050818592893</v>
+        <v>0.01827050818592551</v>
       </c>
       <c r="J60" t="n">
-        <v>7.586034349438582</v>
+        <v>5.142141953979944</v>
       </c>
       <c r="K60" t="n">
-        <v>53.99158789631687</v>
+        <v>53.99159104000891</v>
       </c>
       <c r="L60" t="n">
-        <v>47.21653013894271</v>
+        <v>47.21653013895141</v>
       </c>
       <c r="M60" t="n">
-        <v>0.2600248247441546</v>
+        <v>0.2293371307184592</v>
       </c>
       <c r="N60" t="n">
         <v>0.2503438825093872</v>
@@ -3280,7 +3280,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>238.0200862278932</v>
+        <v>1.006592762977438</v>
       </c>
       <c r="B61" t="n">
         <v>0</v>
@@ -3298,36 +3298,36 @@
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>0.04012649946203461</v>
+        <v>0.05903166816745831</v>
       </c>
       <c r="H61" t="n">
-        <v>0.05010332837588984</v>
+        <v>0.05879831855407184</v>
       </c>
       <c r="I61" t="n">
-        <v>0.06205666365794582</v>
+        <v>0.06870583418279597</v>
       </c>
       <c r="J61" t="n">
-        <v>12.25190135880176</v>
+        <v>8.293782490621886</v>
       </c>
       <c r="K61" t="n">
-        <v>24.92592040365766</v>
+        <v>21.04637177567112</v>
       </c>
       <c r="L61" t="n">
-        <v>12.47889102060749</v>
+        <v>11.2545532577046</v>
       </c>
       <c r="M61" t="n">
-        <v>0.24604449185056</v>
+        <v>0.2268427903534432</v>
       </c>
       <c r="N61" t="n">
-        <v>0.2608155426261001</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O61" t="n">
-        <v>0.3931429881010711</v>
+        <v>0.3863489999533896</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>605.1034945463281</v>
+        <v>15.75462235979659</v>
       </c>
       <c r="B62" t="n">
         <v>0</v>
@@ -3345,28 +3345,28 @@
         <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>0.04721755726960467</v>
+        <v>0.06701563290022199</v>
       </c>
       <c r="H62" t="n">
-        <v>0.05000784024966202</v>
+        <v>0.05137435493521213</v>
       </c>
       <c r="I62" t="n">
-        <v>0.06024037485416536</v>
+        <v>0.0602403748541654</v>
       </c>
       <c r="J62" t="n">
-        <v>10.38960670839317</v>
+        <v>7.299942556417405</v>
       </c>
       <c r="K62" t="n">
-        <v>24.97677479812686</v>
+        <v>24.26888371730844</v>
       </c>
       <c r="L62" t="n">
-        <v>12.86148801950018</v>
+        <v>12.86148801950035</v>
       </c>
       <c r="M62" t="n">
-        <v>0.2492325556532542</v>
+        <v>0.2292035009334855</v>
       </c>
       <c r="N62" t="n">
-        <v>0.2519441235097216</v>
+        <v>0.2504409517474718</v>
       </c>
       <c r="O62" t="n">
         <v>0.3855295790644589</v>
@@ -3374,7 +3374,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1243.443664328614</v>
+        <v>19.71352536279179</v>
       </c>
       <c r="B63" t="n">
         <v>0</v>
@@ -3392,25 +3392,25 @@
         <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>0.05249864710215551</v>
+        <v>0.07608296003688896</v>
       </c>
       <c r="H63" t="n">
-        <v>0.04252156860437417</v>
+        <v>0.04252156914029156</v>
       </c>
       <c r="I63" t="n">
-        <v>0.05017595975375774</v>
+        <v>0.05017595975382203</v>
       </c>
       <c r="J63" t="n">
-        <v>9.334579782591135</v>
+        <v>6.426040084236152</v>
       </c>
       <c r="K63" t="n">
-        <v>29.77475607688664</v>
+        <v>29.77475551406071</v>
       </c>
       <c r="L63" t="n">
-        <v>15.50030379110745</v>
+        <v>15.50030379108042</v>
       </c>
       <c r="M63" t="n">
-        <v>0.2539654096762484</v>
+        <v>0.2301639272572328</v>
       </c>
       <c r="N63" t="n">
         <v>0.2503438825093889</v>
@@ -3421,7 +3421,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>2627.645779618219</v>
+        <v>20.44940414633806</v>
       </c>
       <c r="B64" t="n">
         <v>0</v>
@@ -3439,28 +3439,28 @@
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>0.05672746540153414</v>
+        <v>0.08505071721380514</v>
       </c>
       <c r="H64" t="n">
-        <v>0.03367093031520068</v>
+        <v>0.03367093419836017</v>
       </c>
       <c r="I64" t="n">
-        <v>0.03983894172141884</v>
+        <v>0.03983894172554594</v>
       </c>
       <c r="J64" t="n">
-        <v>8.633187556839303</v>
+        <v>5.74606082105436</v>
       </c>
       <c r="K64" t="n">
-        <v>38.83826609270182</v>
+        <v>38.83825833699155</v>
       </c>
       <c r="L64" t="n">
-        <v>19.66896230601378</v>
+        <v>19.66896230413592</v>
       </c>
       <c r="M64" t="n">
-        <v>0.2591781030763006</v>
+        <v>0.2306394518561364</v>
       </c>
       <c r="N64" t="n">
-        <v>0.2503438825093889</v>
+        <v>0.2503438825093872</v>
       </c>
       <c r="O64" t="n">
         <v>0.3855295790644589</v>
@@ -3468,7 +3468,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>4559.673952679768</v>
+        <v>20.03325283343451</v>
       </c>
       <c r="B65" t="n">
         <v>0</v>
@@ -3486,25 +3486,25 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>0.06123585081844354</v>
+        <v>0.09335794916455857</v>
       </c>
       <c r="H65" t="n">
-        <v>0.02610341344135324</v>
+        <v>0.02610341344142007</v>
       </c>
       <c r="I65" t="n">
-        <v>0.02989360823599165</v>
+        <v>0.02989360553035909</v>
       </c>
       <c r="J65" t="n">
-        <v>7.993258789178625</v>
+        <v>5.23326444453608</v>
       </c>
       <c r="K65" t="n">
-        <v>53.99159104012012</v>
+        <v>53.99159103989754</v>
       </c>
       <c r="L65" t="n">
-        <v>26.65159288139327</v>
+        <v>26.65159529825701</v>
       </c>
       <c r="M65" t="n">
-        <v>0.2633216106331737</v>
+        <v>0.230993723657685</v>
       </c>
       <c r="N65" t="n">
         <v>0.2503438825093872</v>
@@ -3515,7 +3515,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>260.805505406638</v>
+        <v>2.772359395912148</v>
       </c>
       <c r="B66" t="n">
         <v>90</v>
@@ -3533,28 +3533,28 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0.04012649946203449</v>
+        <v>0.05903166816745828</v>
       </c>
       <c r="H66" t="n">
-        <v>0.05010332837589032</v>
+        <v>0.05879831855407187</v>
       </c>
       <c r="I66" t="n">
         <v>0.05499992440104687</v>
       </c>
       <c r="J66" t="n">
-        <v>12.25190135880179</v>
+        <v>8.29378249062189</v>
       </c>
       <c r="K66" t="n">
-        <v>24.92592040365729</v>
+        <v>21.0463717756711</v>
       </c>
       <c r="L66" t="n">
-        <v>14.11116142850717</v>
+        <v>14.11116142850729</v>
       </c>
       <c r="M66" t="n">
-        <v>0.2460444918505601</v>
+        <v>0.2268427903534432</v>
       </c>
       <c r="N66" t="n">
-        <v>0.2608155426260996</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O66" t="n">
         <v>0.3855295790644589</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>605.1034945460722</v>
+        <v>15.75462236170907</v>
       </c>
       <c r="B67" t="n">
         <v>90</v>
@@ -3580,28 +3580,28 @@
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>0.04721755726961872</v>
+        <v>0.0670156329004253</v>
       </c>
       <c r="H67" t="n">
-        <v>0.05000784024966202</v>
+        <v>0.05137435493611199</v>
       </c>
       <c r="I67" t="n">
-        <v>0.04618037325603636</v>
+        <v>0.04618037325637122</v>
       </c>
       <c r="J67" t="n">
-        <v>10.38960670838812</v>
+        <v>7.299942556377307</v>
       </c>
       <c r="K67" t="n">
-        <v>24.97677479812686</v>
+        <v>24.2688837172543</v>
       </c>
       <c r="L67" t="n">
-        <v>16.87985375479992</v>
+        <v>16.87985375467656</v>
       </c>
       <c r="M67" t="n">
-        <v>0.2492325556532408</v>
+        <v>0.229203500933285</v>
       </c>
       <c r="N67" t="n">
-        <v>0.2519441235097216</v>
+        <v>0.2504409517469712</v>
       </c>
       <c r="O67" t="n">
         <v>0.3855295790644589</v>
@@ -3609,7 +3609,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1243.443664328604</v>
+        <v>19.71352536272262</v>
       </c>
       <c r="B68" t="n">
         <v>90</v>
@@ -3627,25 +3627,25 @@
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>0.05249864710215534</v>
+        <v>0.07608296003690386</v>
       </c>
       <c r="H68" t="n">
-        <v>0.04252156914014884</v>
+        <v>0.04252156885610379</v>
       </c>
       <c r="I68" t="n">
-        <v>0.03657296385540446</v>
+        <v>0.03657296354684112</v>
       </c>
       <c r="J68" t="n">
-        <v>9.33457978259119</v>
+        <v>6.426040084236164</v>
       </c>
       <c r="K68" t="n">
-        <v>29.77475551420917</v>
+        <v>29.77475581601517</v>
       </c>
       <c r="L68" t="n">
-        <v>21.50869233594755</v>
+        <v>21.50869251057282</v>
       </c>
       <c r="M68" t="n">
-        <v>0.2539654096762485</v>
+        <v>0.230163927257218</v>
       </c>
       <c r="N68" t="n">
         <v>0.2503438825093889</v>
@@ -3656,7 +3656,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2627.645779618329</v>
+        <v>20.44940414633417</v>
       </c>
       <c r="B69" t="n">
         <v>90</v>
@@ -3674,25 +3674,25 @@
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>0.05672746540154244</v>
+        <v>0.08505071721380503</v>
       </c>
       <c r="H69" t="n">
-        <v>0.03367093338469729</v>
+        <v>0.03367093100260194</v>
       </c>
       <c r="I69" t="n">
-        <v>0.02685826388012589</v>
+        <v>0.02685826388012208</v>
       </c>
       <c r="J69" t="n">
-        <v>8.633187556839811</v>
+        <v>5.746060821054368</v>
       </c>
       <c r="K69" t="n">
-        <v>38.83826000119848</v>
+        <v>38.83826468293864</v>
       </c>
       <c r="L69" t="n">
-        <v>29.95091013276306</v>
+        <v>29.95091013273048</v>
       </c>
       <c r="M69" t="n">
-        <v>0.2591781030762917</v>
+        <v>0.2306394518561365</v>
       </c>
       <c r="N69" t="n">
         <v>0.2503438825093889</v>
@@ -3703,7 +3703,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>4559.673952679737</v>
+        <v>20.03325283344107</v>
       </c>
       <c r="B70" t="n">
         <v>90</v>
@@ -3721,25 +3721,25 @@
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>0.06123585081844355</v>
+        <v>0.09335794916455843</v>
       </c>
       <c r="H70" t="n">
-        <v>0.02610341344138774</v>
+        <v>0.02610340955973183</v>
       </c>
       <c r="I70" t="n">
-        <v>0.01827050818593215</v>
+        <v>0.01827050818592998</v>
       </c>
       <c r="J70" t="n">
-        <v>7.993258789178625</v>
+        <v>5.233264444536087</v>
       </c>
       <c r="K70" t="n">
-        <v>53.99159104000383</v>
+        <v>53.99158146858644</v>
       </c>
       <c r="L70" t="n">
-        <v>47.2165301389356</v>
+        <v>47.21653013894045</v>
       </c>
       <c r="M70" t="n">
-        <v>0.2633216106331736</v>
+        <v>0.230993723657685</v>
       </c>
       <c r="N70" t="n">
         <v>0.2503438825093872</v>

</xml_diff>

<commit_message>
NLP working (no err in x0) - EXIT: Optimal Solution Found.
3 constraints by muscle
</commit_message>
<xml_diff>
--- a/hypothetical_data.xlsx
+++ b/hypothetical_data.xlsx
@@ -507,7 +507,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-7.039566079966283</v>
+        <v>-7.039566079340734</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
@@ -525,36 +525,36 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06253281370900747</v>
+        <v>0.06253281370900593</v>
       </c>
       <c r="H2" t="n">
-        <v>0.05879831855407183</v>
+        <v>0.0587983185539618</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06870583418284333</v>
+        <v>0.06870583418309242</v>
       </c>
       <c r="J2" t="n">
-        <v>7.826424365587129</v>
+        <v>7.82642436558803</v>
       </c>
       <c r="K2" t="n">
-        <v>21.04637177567112</v>
+        <v>21.04637177578298</v>
       </c>
       <c r="L2" t="n">
-        <v>11.25455325771263</v>
+        <v>11.254553257684</v>
       </c>
       <c r="M2" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2513760312601657</v>
+        <v>0.2513760312601548</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3863489999533446</v>
+        <v>0.3863489999530916</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-0.5319015639526551</v>
+        <v>-0.5319015639358142</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
@@ -572,28 +572,28 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.07286844709700201</v>
+        <v>0.07286844709700198</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05137435493610843</v>
+        <v>0.05137435493611127</v>
       </c>
       <c r="I3" t="n">
         <v>0.06024037485416539</v>
       </c>
       <c r="J3" t="n">
-        <v>6.710793399280155</v>
+        <v>6.710793399280099</v>
       </c>
       <c r="K3" t="n">
-        <v>24.26888371725578</v>
+        <v>24.26888371725499</v>
       </c>
       <c r="L3" t="n">
-        <v>12.86148801950038</v>
+        <v>12.86148801950027</v>
       </c>
       <c r="M3" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2504409517469763</v>
+        <v>0.2504409517469732</v>
       </c>
       <c r="O3" t="n">
         <v>0.3855295790644589</v>
@@ -619,22 +619,22 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.08290061396627722</v>
+        <v>0.08290061396627721</v>
       </c>
       <c r="H4" t="n">
-        <v>0.04252156913766904</v>
+        <v>0.04252156903451807</v>
       </c>
       <c r="I4" t="n">
-        <v>0.05017595975382191</v>
+        <v>0.05017595975382204</v>
       </c>
       <c r="J4" t="n">
-        <v>5.895611618411027</v>
+        <v>5.895611618410995</v>
       </c>
       <c r="K4" t="n">
-        <v>29.77475551681599</v>
+        <v>29.77475562725355</v>
       </c>
       <c r="L4" t="n">
-        <v>15.5003037910799</v>
+        <v>15.50030379108042</v>
       </c>
       <c r="M4" t="n">
         <v>0.2233067431983749</v>
@@ -648,7 +648,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-1.52224861053265e-11</v>
+        <v>-4.579177616309509e-12</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
@@ -669,25 +669,25 @@
         <v>0.09234950013810869</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03367093101206951</v>
+        <v>0.03367093419842672</v>
       </c>
       <c r="I5" t="n">
-        <v>0.03983894172232585</v>
+        <v>0.03983894172509973</v>
       </c>
       <c r="J5" t="n">
-        <v>5.290573350413712</v>
+        <v>5.290573350413695</v>
       </c>
       <c r="K5" t="n">
-        <v>38.83826466785862</v>
+        <v>38.83825833720865</v>
       </c>
       <c r="L5" t="n">
-        <v>19.66896230569752</v>
+        <v>19.668962304287</v>
       </c>
       <c r="M5" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N5" t="n">
-        <v>0.2503438825093889</v>
+        <v>0.2503438825093872</v>
       </c>
       <c r="O5" t="n">
         <v>0.3855295790644589</v>
@@ -695,7 +695,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.1394103164166142</v>
+        <v>0.1394103164101905</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
@@ -716,28 +716,28 @@
         <v>0.1009126975550343</v>
       </c>
       <c r="H6" t="n">
-        <v>0.02610341164461799</v>
+        <v>0.02610341344144656</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0298936105430747</v>
+        <v>0.02989360968548715</v>
       </c>
       <c r="J6" t="n">
-        <v>4.840507364843531</v>
+        <v>4.840507364843515</v>
       </c>
       <c r="K6" t="n">
-        <v>53.99158663458693</v>
+        <v>53.99159103980826</v>
       </c>
       <c r="L6" t="n">
-        <v>26.65159076495555</v>
+        <v>26.65159158803702</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2234097331711477</v>
+        <v>0.2234097331711478</v>
       </c>
       <c r="N6" t="n">
         <v>0.2503438825093872</v>
       </c>
       <c r="O6" t="n">
-        <v>0.3855295790644563</v>
+        <v>0.3855295790644589</v>
       </c>
     </row>
     <row r="7">
@@ -760,22 +760,22 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0.06253281370900746</v>
+        <v>0.06253281370900593</v>
       </c>
       <c r="H7" t="n">
         <v>0.05879831855407187</v>
       </c>
       <c r="I7" t="n">
-        <v>0.05499992440104289</v>
+        <v>0.05499992440104687</v>
       </c>
       <c r="J7" t="n">
-        <v>7.826424365587125</v>
+        <v>7.82642436558804</v>
       </c>
       <c r="K7" t="n">
         <v>21.0463717756711</v>
       </c>
       <c r="L7" t="n">
-        <v>14.11116142851065</v>
+        <v>14.11116142850703</v>
       </c>
       <c r="M7" t="n">
         <v>0.2233067431983749</v>
@@ -789,7 +789,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-0.5319015640881622</v>
+        <v>-0.5319015639460549</v>
       </c>
       <c r="B8" t="n">
         <v>90</v>
@@ -807,28 +807,28 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.07286844709700184</v>
+        <v>0.07286844709700188</v>
       </c>
       <c r="H8" t="n">
-        <v>0.05137435493605979</v>
+        <v>0.05137435493610945</v>
       </c>
       <c r="I8" t="n">
-        <v>0.04618037325639714</v>
+        <v>0.04618037325665933</v>
       </c>
       <c r="J8" t="n">
-        <v>6.710793399280111</v>
+        <v>6.71079339928013</v>
       </c>
       <c r="K8" t="n">
-        <v>24.26888371725514</v>
+        <v>24.26888371725546</v>
       </c>
       <c r="L8" t="n">
-        <v>16.87985375466988</v>
+        <v>16.87985375456994</v>
       </c>
       <c r="M8" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N8" t="n">
-        <v>0.2504409517470009</v>
+        <v>0.2504409517469751</v>
       </c>
       <c r="O8" t="n">
         <v>0.3855295790644589</v>
@@ -854,22 +854,22 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0.08290061396627714</v>
+        <v>0.08290061396627715</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04252156914041136</v>
+        <v>0.04252156913504121</v>
       </c>
       <c r="I9" t="n">
-        <v>0.03657296373902767</v>
+        <v>0.03657296380366366</v>
       </c>
       <c r="J9" t="n">
-        <v>5.895611618411032</v>
+        <v>5.895611618411001</v>
       </c>
       <c r="K9" t="n">
-        <v>29.77475551392967</v>
+        <v>29.77475551991866</v>
       </c>
       <c r="L9" t="n">
-        <v>21.50869239936085</v>
+        <v>21.50869236481925</v>
       </c>
       <c r="M9" t="n">
         <v>0.2233067431983749</v>
@@ -883,7 +883,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.166644264400974e-12</v>
+        <v>-8.476664224616022e-12</v>
       </c>
       <c r="B10" t="n">
         <v>90</v>
@@ -904,25 +904,25 @@
         <v>0.09234950013810855</v>
       </c>
       <c r="H10" t="n">
-        <v>0.03367093419820232</v>
+        <v>0.03367093325895628</v>
       </c>
       <c r="I10" t="n">
-        <v>0.02685826388012495</v>
+        <v>0.02685826388012597</v>
       </c>
       <c r="J10" t="n">
-        <v>5.290573350413708</v>
+        <v>5.290573350413707</v>
       </c>
       <c r="K10" t="n">
-        <v>38.83825833645791</v>
+        <v>38.83826020610323</v>
       </c>
       <c r="L10" t="n">
-        <v>29.95091013275549</v>
+        <v>29.95091013276352</v>
       </c>
       <c r="M10" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N10" t="n">
-        <v>0.2503438825093872</v>
+        <v>0.2503438825093889</v>
       </c>
       <c r="O10" t="n">
         <v>0.3855295790644563</v>
@@ -930,7 +930,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.1394103164125602</v>
+        <v>0.1394103164164791</v>
       </c>
       <c r="B11" t="n">
         <v>90</v>
@@ -948,25 +948,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1009126975550372</v>
+        <v>0.1009126975550343</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02610341223799564</v>
+        <v>0.02610341196157462</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0182705081859313</v>
+        <v>0.01827050818593021</v>
       </c>
       <c r="J11" t="n">
-        <v>4.84050736484353</v>
+        <v>4.840507364843507</v>
       </c>
       <c r="K11" t="n">
-        <v>53.99158815915724</v>
+        <v>53.99158752203915</v>
       </c>
       <c r="L11" t="n">
-        <v>47.21653013893754</v>
+        <v>47.21653013893997</v>
       </c>
       <c r="M11" t="n">
-        <v>0.2234097331711447</v>
+        <v>0.2234097331711476</v>
       </c>
       <c r="N11" t="n">
         <v>0.2503438825093872</v>
@@ -977,7 +977,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>-24.75191021747457</v>
+        <v>-24.75191021747483</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
@@ -995,22 +995,22 @@
         <v>0.1</v>
       </c>
       <c r="G12" t="n">
-        <v>0.06253281370900744</v>
+        <v>0.06253281370900746</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05730837172727809</v>
+        <v>0.05730837172727807</v>
       </c>
       <c r="I12" t="n">
-        <v>0.06571230143582209</v>
+        <v>0.06571230143582202</v>
       </c>
       <c r="J12" t="n">
-        <v>7.82642436558695</v>
+        <v>7.826424365587109</v>
       </c>
       <c r="K12" t="n">
-        <v>21.62068397000089</v>
+        <v>21.6206839700009</v>
       </c>
       <c r="L12" t="n">
-        <v>11.77442990840427</v>
+        <v>11.77442990840429</v>
       </c>
       <c r="M12" t="n">
         <v>0.2233067431983749</v>
@@ -1024,7 +1024,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>-23.52416809768336</v>
+        <v>-23.52416809768309</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -1042,22 +1042,22 @@
         <v>0.1</v>
       </c>
       <c r="G13" t="n">
-        <v>0.07286844709700201</v>
+        <v>0.07286844709700198</v>
       </c>
       <c r="H13" t="n">
         <v>0.04946501093929172</v>
       </c>
       <c r="I13" t="n">
-        <v>0.05686766231240566</v>
+        <v>0.05686766231240574</v>
       </c>
       <c r="J13" t="n">
-        <v>6.710793399280144</v>
+        <v>6.710793399280128</v>
       </c>
       <c r="K13" t="n">
         <v>25.27001295149489</v>
       </c>
       <c r="L13" t="n">
-        <v>13.63858109067641</v>
+        <v>13.6385810906764</v>
       </c>
       <c r="M13" t="n">
         <v>0.2233067431983749</v>
@@ -1066,7 +1066,7 @@
         <v>0.2525436709112036</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3889944520214331</v>
+        <v>0.388994452021433</v>
       </c>
     </row>
     <row r="14">
@@ -1089,7 +1089,7 @@
         <v>0.1</v>
       </c>
       <c r="G14" t="n">
-        <v>0.08290061396627718</v>
+        <v>0.08290061396627717</v>
       </c>
       <c r="H14" t="n">
         <v>0.04093815692345399</v>
@@ -1098,7 +1098,7 @@
         <v>0.04735766927932555</v>
       </c>
       <c r="J14" t="n">
-        <v>5.895611618410976</v>
+        <v>5.895611618411038</v>
       </c>
       <c r="K14" t="n">
         <v>31.0508641752185</v>
@@ -1113,12 +1113,12 @@
         <v>0.2521798207005737</v>
       </c>
       <c r="O14" t="n">
-        <v>0.3884609668667924</v>
+        <v>0.3884609668667923</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>-11.4789937207829</v>
+        <v>-11.47899372055169</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -1136,28 +1136,28 @@
         <v>0.1</v>
       </c>
       <c r="G15" t="n">
-        <v>0.09234950013810869</v>
+        <v>0.09234950013810866</v>
       </c>
       <c r="H15" t="n">
-        <v>0.03281854674466999</v>
+        <v>0.03281854674478776</v>
       </c>
       <c r="I15" t="n">
-        <v>0.03842775810114049</v>
+        <v>0.03842775810114052</v>
       </c>
       <c r="J15" t="n">
-        <v>5.29057335041372</v>
+        <v>5.290573350413707</v>
       </c>
       <c r="K15" t="n">
-        <v>40.04673104699245</v>
+        <v>40.04673104719279</v>
       </c>
       <c r="L15" t="n">
-        <v>20.42283886642783</v>
+        <v>20.42283886642781</v>
       </c>
       <c r="M15" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N15" t="n">
-        <v>0.2514475745120108</v>
+        <v>0.2514475745119788</v>
       </c>
       <c r="O15" t="n">
         <v>0.3870317353001125</v>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>-1.035134726097748</v>
+        <v>-1.035134726097601</v>
       </c>
       <c r="B16" t="n">
         <v>0</v>
@@ -1183,31 +1183,31 @@
         <v>0.1</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1009126975550354</v>
+        <v>0.1009126975550343</v>
       </c>
       <c r="H16" t="n">
-        <v>0.02603288517006376</v>
+        <v>0.02603288517006377</v>
       </c>
       <c r="I16" t="n">
-        <v>0.02974036282445704</v>
+        <v>0.02974036282445738</v>
       </c>
       <c r="J16" t="n">
-        <v>4.840507364843439</v>
+        <v>4.840507364843528</v>
       </c>
       <c r="K16" t="n">
-        <v>54.20572601913344</v>
+        <v>54.20572601913314</v>
       </c>
       <c r="L16" t="n">
-        <v>26.79986341395706</v>
+        <v>26.79986341395968</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2234097331711467</v>
+        <v>0.2234097331711478</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2504641573933862</v>
+        <v>0.2504641573933863</v>
       </c>
       <c r="O16" t="n">
-        <v>0.3857011563325844</v>
+        <v>0.3857011563325847</v>
       </c>
     </row>
     <row r="17">
@@ -1230,19 +1230,19 @@
         <v>0.1</v>
       </c>
       <c r="G17" t="n">
-        <v>0.06253281370900743</v>
+        <v>0.06253281370900636</v>
       </c>
       <c r="H17" t="n">
-        <v>0.05730837172727807</v>
+        <v>0.05730837172727809</v>
       </c>
       <c r="I17" t="n">
-        <v>0.05190222593196153</v>
+        <v>0.0519022259319615</v>
       </c>
       <c r="J17" t="n">
-        <v>7.826424365586933</v>
+        <v>7.826424365587894</v>
       </c>
       <c r="K17" t="n">
-        <v>21.6206839700009</v>
+        <v>21.62068397000089</v>
       </c>
       <c r="L17" t="n">
         <v>14.9724746412667</v>
@@ -1277,19 +1277,19 @@
         <v>0.1</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0728684470970019</v>
+        <v>0.07286844709700192</v>
       </c>
       <c r="H18" t="n">
-        <v>0.04946501093929172</v>
+        <v>0.0494650109392917</v>
       </c>
       <c r="I18" t="n">
-        <v>0.04371179011867187</v>
+        <v>0.04371179011867188</v>
       </c>
       <c r="J18" t="n">
-        <v>6.710793399280204</v>
+        <v>6.710793399280177</v>
       </c>
       <c r="K18" t="n">
-        <v>25.27001295149489</v>
+        <v>25.2700129514949</v>
       </c>
       <c r="L18" t="n">
         <v>17.86431470931674</v>
@@ -1306,7 +1306,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>-14.53528163706801</v>
+        <v>-14.53528163706778</v>
       </c>
       <c r="B19" t="n">
         <v>90</v>
@@ -1324,22 +1324,22 @@
         <v>0.1</v>
       </c>
       <c r="G19" t="n">
-        <v>0.08290061396627714</v>
+        <v>0.08290061396627713</v>
       </c>
       <c r="H19" t="n">
         <v>0.04093815692345398</v>
       </c>
       <c r="I19" t="n">
-        <v>0.03580503034823525</v>
+        <v>0.03580503034823536</v>
       </c>
       <c r="J19" t="n">
-        <v>5.895611618411002</v>
+        <v>5.895611618410979</v>
       </c>
       <c r="K19" t="n">
         <v>31.05086417521851</v>
       </c>
       <c r="L19" t="n">
-        <v>21.99378335069485</v>
+        <v>21.9937833506948</v>
       </c>
       <c r="M19" t="n">
         <v>0.2233067431983749</v>
@@ -1348,12 +1348,12 @@
         <v>0.2521798207005737</v>
       </c>
       <c r="O19" t="n">
-        <v>0.3863563720944934</v>
+        <v>0.3863563720944933</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>-7.683344919469722</v>
+        <v>-7.683344919454074</v>
       </c>
       <c r="B20" t="n">
         <v>90</v>
@@ -1371,36 +1371,36 @@
         <v>0.1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.09234950013810858</v>
+        <v>0.09234950013810854</v>
       </c>
       <c r="H20" t="n">
-        <v>0.03281854674478244</v>
+        <v>0.03281854674475673</v>
       </c>
       <c r="I20" t="n">
-        <v>0.02675616544362131</v>
+        <v>0.02675616544327385</v>
       </c>
       <c r="J20" t="n">
-        <v>5.290573350413724</v>
+        <v>5.290573350413706</v>
       </c>
       <c r="K20" t="n">
-        <v>40.04673104718408</v>
+        <v>40.04673104714015</v>
       </c>
       <c r="L20" t="n">
-        <v>30.07696894315752</v>
+        <v>30.07696894144157</v>
       </c>
       <c r="M20" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N20" t="n">
-        <v>0.2514475745119802</v>
+        <v>0.2514475745119872</v>
       </c>
       <c r="O20" t="n">
-        <v>0.3856474886781584</v>
+        <v>0.3856474886781326</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>-0.7100947334600101</v>
+        <v>-0.7100947334647261</v>
       </c>
       <c r="B21" t="n">
         <v>90</v>
@@ -1421,19 +1421,19 @@
         <v>0.1009126975550357</v>
       </c>
       <c r="H21" t="n">
-        <v>0.02603288517006366</v>
+        <v>0.02603288517006367</v>
       </c>
       <c r="I21" t="n">
-        <v>0.01824271150191096</v>
+        <v>0.01824271150280669</v>
       </c>
       <c r="J21" t="n">
-        <v>4.840507364843528</v>
+        <v>4.840507364843416</v>
       </c>
       <c r="K21" t="n">
-        <v>54.20572601913371</v>
+        <v>54.20572601913353</v>
       </c>
       <c r="L21" t="n">
-        <v>47.31094684614971</v>
+        <v>47.31094684236052</v>
       </c>
       <c r="M21" t="n">
         <v>0.2234097331711463</v>
@@ -1442,12 +1442,12 @@
         <v>0.2504641573933862</v>
       </c>
       <c r="O21" t="n">
-        <v>0.3855705393695402</v>
+        <v>0.3855705393695419</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>-44.29184292490903</v>
+        <v>-44.29184292491333</v>
       </c>
       <c r="B22" t="n">
         <v>0</v>
@@ -1465,36 +1465,36 @@
         <v>0.2</v>
       </c>
       <c r="G22" t="n">
-        <v>0.06253281370900744</v>
+        <v>0.06253281370900741</v>
       </c>
       <c r="H22" t="n">
-        <v>0.05595688151536346</v>
+        <v>0.05595688151536338</v>
       </c>
       <c r="I22" t="n">
-        <v>0.06322418848124188</v>
+        <v>0.06322418848124088</v>
       </c>
       <c r="J22" t="n">
-        <v>7.82642436558713</v>
+        <v>7.826424365586952</v>
       </c>
       <c r="K22" t="n">
-        <v>22.17021099014359</v>
+        <v>22.17021099014362</v>
       </c>
       <c r="L22" t="n">
-        <v>12.2448414360043</v>
+        <v>12.24484143600442</v>
       </c>
       <c r="M22" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N22" t="n">
-        <v>0.2544321025474924</v>
+        <v>0.2544321025474925</v>
       </c>
       <c r="O22" t="n">
-        <v>0.3919477541924257</v>
+        <v>0.3919477541924267</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>-45.72736374796932</v>
+        <v>-45.72736374796879</v>
       </c>
       <c r="B23" t="n">
         <v>0</v>
@@ -1512,22 +1512,22 @@
         <v>0.2</v>
       </c>
       <c r="G23" t="n">
-        <v>0.07286844709700198</v>
+        <v>0.07286844709700201</v>
       </c>
       <c r="H23" t="n">
-        <v>0.04800447130510595</v>
+        <v>0.04800447130510596</v>
       </c>
       <c r="I23" t="n">
-        <v>0.05450029248318129</v>
+        <v>0.05450029248318133</v>
       </c>
       <c r="J23" t="n">
-        <v>6.710793399280194</v>
+        <v>6.710793399280184</v>
       </c>
       <c r="K23" t="n">
         <v>26.09575469145532</v>
       </c>
       <c r="L23" t="n">
-        <v>14.24324468664561</v>
+        <v>14.2432446866456</v>
       </c>
       <c r="M23" t="n">
         <v>0.2233067431983749</v>
@@ -1541,7 +1541,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>-39.63908644434589</v>
+        <v>-39.63908644434623</v>
       </c>
       <c r="B24" t="n">
         <v>0</v>
@@ -1562,16 +1562,16 @@
         <v>0.08290061396627718</v>
       </c>
       <c r="H24" t="n">
-        <v>0.03978100212799033</v>
+        <v>0.03978100212799031</v>
       </c>
       <c r="I24" t="n">
-        <v>0.0453902110118024</v>
+        <v>0.04539021101180242</v>
       </c>
       <c r="J24" t="n">
-        <v>5.895611618410981</v>
+        <v>5.895611618411031</v>
       </c>
       <c r="K24" t="n">
-        <v>32.05968856678505</v>
+        <v>32.05968856678507</v>
       </c>
       <c r="L24" t="n">
         <v>17.18275348436879</v>
@@ -1588,7 +1588,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>-20.18107573840153</v>
+        <v>-20.18107573846943</v>
       </c>
       <c r="B25" t="n">
         <v>0</v>
@@ -1606,19 +1606,19 @@
         <v>0.2</v>
       </c>
       <c r="G25" t="n">
-        <v>0.09234950013810866</v>
+        <v>0.09234950013810869</v>
       </c>
       <c r="H25" t="n">
-        <v>0.03222772317799887</v>
+        <v>0.0322277231779901</v>
       </c>
       <c r="I25" t="n">
-        <v>0.03757339780549243</v>
+        <v>0.03757339780549242</v>
       </c>
       <c r="J25" t="n">
-        <v>5.290573350413703</v>
+        <v>5.290573350413693</v>
       </c>
       <c r="K25" t="n">
-        <v>40.93540226951523</v>
+        <v>40.93540226951827</v>
       </c>
       <c r="L25" t="n">
         <v>20.90871609805018</v>
@@ -1627,7 +1627,7 @@
         <v>0.2233067431983749</v>
       </c>
       <c r="N25" t="n">
-        <v>0.2522244320985437</v>
+        <v>0.2522244320985522</v>
       </c>
       <c r="O25" t="n">
         <v>0.3879448417572579</v>
@@ -1635,7 +1635,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>-2.153098315480481</v>
+        <v>-2.153098315254923</v>
       </c>
       <c r="B26" t="n">
         <v>0</v>
@@ -1653,22 +1653,22 @@
         <v>0.2</v>
       </c>
       <c r="G26" t="n">
-        <v>0.100912697555035</v>
+        <v>0.1009126975550349</v>
       </c>
       <c r="H26" t="n">
         <v>0.02596742250262568</v>
       </c>
       <c r="I26" t="n">
-        <v>0.02959590872373442</v>
+        <v>0.02959590872349823</v>
       </c>
       <c r="J26" t="n">
-        <v>4.840507364843519</v>
+        <v>4.84050736484352</v>
       </c>
       <c r="K26" t="n">
-        <v>54.40652760547247</v>
+        <v>54.40652760547246</v>
       </c>
       <c r="L26" t="n">
-        <v>26.94121412742172</v>
+        <v>26.9412141263707</v>
       </c>
       <c r="M26" t="n">
         <v>0.2234097331711471</v>
@@ -1677,7 +1677,7 @@
         <v>0.2505763556566254</v>
       </c>
       <c r="O26" t="n">
-        <v>0.3858630948126754</v>
+        <v>0.3858630948125871</v>
       </c>
     </row>
     <row r="27">
@@ -1700,19 +1700,19 @@
         <v>0.2</v>
       </c>
       <c r="G27" t="n">
-        <v>0.06253281370900748</v>
+        <v>0.06253281370900643</v>
       </c>
       <c r="H27" t="n">
-        <v>0.05595688151536373</v>
+        <v>0.05595688151536369</v>
       </c>
       <c r="I27" t="n">
-        <v>0.04970492329672653</v>
+        <v>0.04970492329672654</v>
       </c>
       <c r="J27" t="n">
-        <v>7.8264243655871</v>
+        <v>7.826424365587871</v>
       </c>
       <c r="K27" t="n">
-        <v>22.1702109901435</v>
+        <v>22.17021099014351</v>
       </c>
       <c r="L27" t="n">
         <v>15.65094155307737</v>
@@ -1729,7 +1729,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>-39.33887274528458</v>
+        <v>-39.3388727452851</v>
       </c>
       <c r="B28" t="n">
         <v>90</v>
@@ -1747,19 +1747,19 @@
         <v>0.2</v>
       </c>
       <c r="G28" t="n">
-        <v>0.07286844709700188</v>
+        <v>0.0728684470970019</v>
       </c>
       <c r="H28" t="n">
-        <v>0.04800447130510592</v>
+        <v>0.04800447130510588</v>
       </c>
       <c r="I28" t="n">
-        <v>0.04211132369840671</v>
+        <v>0.04211132369840673</v>
       </c>
       <c r="J28" t="n">
-        <v>6.710793399280172</v>
+        <v>6.710793399280184</v>
       </c>
       <c r="K28" t="n">
-        <v>26.09575469145535</v>
+        <v>26.09575469145537</v>
       </c>
       <c r="L28" t="n">
         <v>18.56755891430156</v>
@@ -1794,22 +1794,22 @@
         <v>0.2</v>
       </c>
       <c r="G29" t="n">
-        <v>0.08290061396627713</v>
+        <v>0.08290061396627711</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0397810021279903</v>
+        <v>0.03978100212799031</v>
       </c>
       <c r="I29" t="n">
-        <v>0.03528979645683911</v>
+        <v>0.03528979645683909</v>
       </c>
       <c r="J29" t="n">
-        <v>5.895611618411035</v>
+        <v>5.895611618411013</v>
       </c>
       <c r="K29" t="n">
-        <v>32.05968856678508</v>
+        <v>32.05968856678507</v>
       </c>
       <c r="L29" t="n">
-        <v>22.33206031740519</v>
+        <v>22.3320603174052</v>
       </c>
       <c r="M29" t="n">
         <v>0.2233067431983749</v>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>-13.9018535064225</v>
+        <v>-13.90185350703722</v>
       </c>
       <c r="B30" t="n">
         <v>90</v>
@@ -1841,36 +1841,36 @@
         <v>0.2</v>
       </c>
       <c r="G30" t="n">
-        <v>0.09234950013810858</v>
+        <v>0.09234950013810855</v>
       </c>
       <c r="H30" t="n">
-        <v>0.03222772317799556</v>
+        <v>0.03222772317791427</v>
       </c>
       <c r="I30" t="n">
-        <v>0.02665758037485855</v>
+        <v>0.02665758037485861</v>
       </c>
       <c r="J30" t="n">
-        <v>5.290573350413717</v>
+        <v>5.290573350413714</v>
       </c>
       <c r="K30" t="n">
-        <v>40.93540226951615</v>
+        <v>40.93540226954071</v>
       </c>
       <c r="L30" t="n">
-        <v>30.19976054138432</v>
+        <v>30.19976054138424</v>
       </c>
       <c r="M30" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2522244320985468</v>
+        <v>0.2522244320986232</v>
       </c>
       <c r="O30" t="n">
-        <v>0.3857614841158369</v>
+        <v>0.3857614841158368</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>-1.519994855945454</v>
+        <v>-1.519994855943522</v>
       </c>
       <c r="B31" t="n">
         <v>90</v>
@@ -1888,28 +1888,28 @@
         <v>0.2</v>
       </c>
       <c r="G31" t="n">
-        <v>0.1009126975550357</v>
+        <v>0.1009126975550351</v>
       </c>
       <c r="H31" t="n">
-        <v>0.02596742250262544</v>
+        <v>0.02596742250262559</v>
       </c>
       <c r="I31" t="n">
         <v>0.0182153071948747</v>
       </c>
       <c r="J31" t="n">
-        <v>4.840507364843532</v>
+        <v>4.840507364843527</v>
       </c>
       <c r="K31" t="n">
-        <v>54.40652760547281</v>
+        <v>54.40652760547272</v>
       </c>
       <c r="L31" t="n">
         <v>47.40447901570864</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2234097331711462</v>
+        <v>0.2234097331711468</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2505763556566256</v>
+        <v>0.2505763556566254</v>
       </c>
       <c r="O31" t="n">
         <v>0.3856109933535384</v>
@@ -1917,7 +1917,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>-64.67598060275154</v>
+        <v>-64.6759806027019</v>
       </c>
       <c r="B32" t="n">
         <v>0</v>
@@ -1935,36 +1935,36 @@
         <v>0.3</v>
       </c>
       <c r="G32" t="n">
-        <v>0.06253281370900747</v>
+        <v>0.06253281370900748</v>
       </c>
       <c r="H32" t="n">
-        <v>0.05477021046838707</v>
+        <v>0.0547702104683875</v>
       </c>
       <c r="I32" t="n">
-        <v>0.06118689698525605</v>
+        <v>0.06118689698526585</v>
       </c>
       <c r="J32" t="n">
-        <v>7.826424365587119</v>
+        <v>7.8264243655871</v>
       </c>
       <c r="K32" t="n">
-        <v>22.67698033117222</v>
+        <v>22.67698033117209</v>
       </c>
       <c r="L32" t="n">
-        <v>12.65919959526171</v>
+        <v>12.65919959526029</v>
       </c>
       <c r="M32" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2557158255412278</v>
+        <v>0.2557158255412273</v>
       </c>
       <c r="O32" t="n">
-        <v>0.3940341098998117</v>
+        <v>0.3940341098998018</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>-66.76846482667963</v>
+        <v>-66.76846482667901</v>
       </c>
       <c r="B33" t="n">
         <v>0</v>
@@ -1982,28 +1982,28 @@
         <v>0.3</v>
       </c>
       <c r="G33" t="n">
-        <v>0.07286844709700203</v>
+        <v>0.07286844709700201</v>
       </c>
       <c r="H33" t="n">
-        <v>0.04687097787738431</v>
+        <v>0.04687097787738437</v>
       </c>
       <c r="I33" t="n">
-        <v>0.05268210191718711</v>
+        <v>0.05268210191718713</v>
       </c>
       <c r="J33" t="n">
-        <v>6.71079339928017</v>
+        <v>6.710793399280173</v>
       </c>
       <c r="K33" t="n">
-        <v>26.77642175659013</v>
+        <v>26.7764217565901</v>
       </c>
       <c r="L33" t="n">
-        <v>14.7457630649831</v>
+        <v>14.74576306498309</v>
       </c>
       <c r="M33" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N33" t="n">
-        <v>0.2554301184612997</v>
+        <v>0.2554301184612996</v>
       </c>
       <c r="O33" t="n">
         <v>0.3933115807589476</v>
@@ -2011,7 +2011,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>-56.78667999206619</v>
+        <v>-56.7866799920658</v>
       </c>
       <c r="B34" t="n">
         <v>0</v>
@@ -2029,22 +2029,22 @@
         <v>0.3</v>
       </c>
       <c r="G34" t="n">
-        <v>0.0829006139662772</v>
+        <v>0.08290061396627721</v>
       </c>
       <c r="H34" t="n">
-        <v>0.03887310520032512</v>
+        <v>0.03887310520032511</v>
       </c>
       <c r="I34" t="n">
-        <v>0.04394681108915043</v>
+        <v>0.04394681108915048</v>
       </c>
       <c r="J34" t="n">
-        <v>5.895611618411029</v>
+        <v>5.895611618411025</v>
       </c>
       <c r="K34" t="n">
         <v>32.90171245377912</v>
       </c>
       <c r="L34" t="n">
-        <v>17.76558528959739</v>
+        <v>17.76558528959737</v>
       </c>
       <c r="M34" t="n">
         <v>0.2233067431983749</v>
@@ -2079,19 +2079,19 @@
         <v>0.09234950013810868</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0317843903225057</v>
+        <v>0.03178439032250569</v>
       </c>
       <c r="I35" t="n">
-        <v>0.03697526810927927</v>
+        <v>0.03697526810927934</v>
       </c>
       <c r="J35" t="n">
-        <v>5.29057335041369</v>
+        <v>5.290573350413694</v>
       </c>
       <c r="K35" t="n">
-        <v>41.63222117314146</v>
+        <v>41.63222117314147</v>
       </c>
       <c r="L35" t="n">
-        <v>21.26322624629508</v>
+        <v>21.26322624629507</v>
       </c>
       <c r="M35" t="n">
         <v>0.2233067431983749</v>
@@ -2105,7 +2105,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>-3.222690133882169</v>
+        <v>-3.222690134021492</v>
       </c>
       <c r="B36" t="n">
         <v>0</v>
@@ -2123,36 +2123,36 @@
         <v>0.3</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1009126975550343</v>
+        <v>0.1009126975550344</v>
       </c>
       <c r="H36" t="n">
-        <v>0.02590624890179347</v>
+        <v>0.02590624890179282</v>
       </c>
       <c r="I36" t="n">
-        <v>0.02945900841150244</v>
+        <v>0.02945900841203259</v>
       </c>
       <c r="J36" t="n">
-        <v>4.840507364843521</v>
+        <v>4.840507364843511</v>
       </c>
       <c r="K36" t="n">
-        <v>54.59598932066348</v>
+        <v>54.59598932066549</v>
       </c>
       <c r="L36" t="n">
-        <v>27.07661881849552</v>
+        <v>27.07661881970247</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2234097331711478</v>
+        <v>0.2234097331711477</v>
       </c>
       <c r="N36" t="n">
-        <v>0.2506817028059683</v>
+        <v>0.2506817028059694</v>
       </c>
       <c r="O36" t="n">
-        <v>0.3860167536994653</v>
+        <v>0.3860167536995164</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>-58.41499067826359</v>
+        <v>-58.414990678258</v>
       </c>
       <c r="B37" t="n">
         <v>90</v>
@@ -2170,19 +2170,19 @@
         <v>0.3</v>
       </c>
       <c r="G37" t="n">
-        <v>0.06253281370900744</v>
+        <v>0.06253281370900746</v>
       </c>
       <c r="H37" t="n">
-        <v>0.05477021046838668</v>
+        <v>0.05477021046838711</v>
       </c>
       <c r="I37" t="n">
-        <v>0.04800927887740836</v>
+        <v>0.04800927887740835</v>
       </c>
       <c r="J37" t="n">
-        <v>7.82642436558691</v>
+        <v>7.826424365587132</v>
       </c>
       <c r="K37" t="n">
-        <v>22.67698033117234</v>
+        <v>22.67698033117205</v>
       </c>
       <c r="L37" t="n">
         <v>16.21868797572033</v>
@@ -2191,7 +2191,7 @@
         <v>0.2233067431983749</v>
       </c>
       <c r="N37" t="n">
-        <v>0.2557158255412282</v>
+        <v>0.2557158255412276</v>
       </c>
       <c r="O37" t="n">
         <v>0.3927712192567968</v>
@@ -2199,7 +2199,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>-56.34182778959218</v>
+        <v>-56.34182778959648</v>
       </c>
       <c r="B38" t="n">
         <v>90</v>
@@ -2217,28 +2217,28 @@
         <v>0.3</v>
       </c>
       <c r="G38" t="n">
-        <v>0.07286844709700187</v>
+        <v>0.07286844709700191</v>
       </c>
       <c r="H38" t="n">
-        <v>0.04687097787738437</v>
+        <v>0.046870977877384</v>
       </c>
       <c r="I38" t="n">
-        <v>0.04100303527273607</v>
+        <v>0.04100303527273605</v>
       </c>
       <c r="J38" t="n">
-        <v>6.710793399280122</v>
+        <v>6.710793399280149</v>
       </c>
       <c r="K38" t="n">
-        <v>26.7764217565901</v>
+        <v>26.77642175659028</v>
       </c>
       <c r="L38" t="n">
-        <v>19.08857150676737</v>
+        <v>19.08857150676738</v>
       </c>
       <c r="M38" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N38" t="n">
-        <v>0.2554301184612996</v>
+        <v>0.2554301184613</v>
       </c>
       <c r="O38" t="n">
         <v>0.3909718561542017</v>
@@ -2246,7 +2246,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>-39.50063140780722</v>
+        <v>-39.5006314078354</v>
       </c>
       <c r="B39" t="n">
         <v>90</v>
@@ -2264,36 +2264,36 @@
         <v>0.3</v>
       </c>
       <c r="G39" t="n">
-        <v>0.08290061396627711</v>
+        <v>0.08290061396627717</v>
       </c>
       <c r="H39" t="n">
-        <v>0.0388731052003251</v>
+        <v>0.03887310520032364</v>
       </c>
       <c r="I39" t="n">
-        <v>0.03490083800272518</v>
+        <v>0.03490083800272054</v>
       </c>
       <c r="J39" t="n">
-        <v>5.895611618411033</v>
+        <v>5.895611618411015</v>
       </c>
       <c r="K39" t="n">
-        <v>32.90171245377913</v>
+        <v>32.90171245377864</v>
       </c>
       <c r="L39" t="n">
-        <v>22.59461131889639</v>
+        <v>22.59461131890243</v>
       </c>
       <c r="M39" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N39" t="n">
-        <v>0.2546139382195903</v>
+        <v>0.2546139382195914</v>
       </c>
       <c r="O39" t="n">
-        <v>0.3873336017418968</v>
+        <v>0.3873336017419022</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>-19.13936725131468</v>
+        <v>-19.13936725131445</v>
       </c>
       <c r="B40" t="n">
         <v>90</v>
@@ -2311,22 +2311,22 @@
         <v>0.3</v>
       </c>
       <c r="G40" t="n">
-        <v>0.09234950013810854</v>
+        <v>0.09234950013810857</v>
       </c>
       <c r="H40" t="n">
         <v>0.03178439032250571</v>
       </c>
       <c r="I40" t="n">
-        <v>0.02656224850296427</v>
+        <v>0.02656224850296426</v>
       </c>
       <c r="J40" t="n">
-        <v>5.290573350413744</v>
+        <v>5.2905733504137</v>
       </c>
       <c r="K40" t="n">
-        <v>41.63222117314144</v>
+        <v>41.63222117314145</v>
       </c>
       <c r="L40" t="n">
-        <v>30.31951443557996</v>
+        <v>30.31951443557998</v>
       </c>
       <c r="M40" t="n">
         <v>0.2233067431983749</v>
@@ -2340,7 +2340,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>-2.295992522491225</v>
+        <v>-2.295992522491678</v>
       </c>
       <c r="B41" t="n">
         <v>90</v>
@@ -2358,36 +2358,36 @@
         <v>0.3</v>
       </c>
       <c r="G41" t="n">
-        <v>0.1009126975550348</v>
+        <v>0.1009126975550361</v>
       </c>
       <c r="H41" t="n">
-        <v>0.0259062489017934</v>
+        <v>0.02590624890179339</v>
       </c>
       <c r="I41" t="n">
-        <v>0.01818828496080611</v>
+        <v>0.0181882849606895</v>
       </c>
       <c r="J41" t="n">
-        <v>4.840507364843522</v>
+        <v>4.840507364843391</v>
       </c>
       <c r="K41" t="n">
-        <v>54.59598932066366</v>
+        <v>54.5959893206637</v>
       </c>
       <c r="L41" t="n">
-        <v>47.49714676747381</v>
+        <v>47.49714676739512</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2234097331711472</v>
+        <v>0.2234097331711458</v>
       </c>
       <c r="N41" t="n">
         <v>0.2506817028059683</v>
       </c>
       <c r="O41" t="n">
-        <v>0.3856509538834834</v>
+        <v>0.3856509538834829</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>-85.26549178531374</v>
+        <v>-85.26549178530766</v>
       </c>
       <c r="B42" t="n">
         <v>0</v>
@@ -2405,28 +2405,28 @@
         <v>0.4</v>
       </c>
       <c r="G42" t="n">
-        <v>0.06253281370900743</v>
+        <v>0.06253281370900748</v>
       </c>
       <c r="H42" t="n">
-        <v>0.05374012161169822</v>
+        <v>0.05374012161169874</v>
       </c>
       <c r="I42" t="n">
-        <v>0.05950604742358306</v>
+        <v>0.05950604742358296</v>
       </c>
       <c r="J42" t="n">
-        <v>7.82642436558696</v>
+        <v>7.826424365587127</v>
       </c>
       <c r="K42" t="n">
-        <v>23.13664256803842</v>
+        <v>23.13664256803824</v>
       </c>
       <c r="L42" t="n">
-        <v>13.02297658713453</v>
+        <v>13.02297658713455</v>
       </c>
       <c r="M42" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N42" t="n">
-        <v>0.2568340937002477</v>
+        <v>0.2568340937002471</v>
       </c>
       <c r="O42" t="n">
         <v>0.3957580667631136</v>
@@ -2452,22 +2452,22 @@
         <v>0.4</v>
       </c>
       <c r="G43" t="n">
-        <v>0.07286844709700199</v>
+        <v>0.07286844709700194</v>
       </c>
       <c r="H43" t="n">
-        <v>0.04595012646737655</v>
+        <v>0.04595012646737652</v>
       </c>
       <c r="I43" t="n">
-        <v>0.05120329271662809</v>
+        <v>0.05120329271662811</v>
       </c>
       <c r="J43" t="n">
-        <v>6.710793399280135</v>
+        <v>6.710793399280083</v>
       </c>
       <c r="K43" t="n">
-        <v>27.35733293447954</v>
+        <v>27.35733293447955</v>
       </c>
       <c r="L43" t="n">
-        <v>15.18173681976456</v>
+        <v>15.18173681976455</v>
       </c>
       <c r="M43" t="n">
         <v>0.2233067431983749</v>
@@ -2481,7 +2481,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>-72.43319315347443</v>
+        <v>-72.43319315347468</v>
       </c>
       <c r="B44" t="n">
         <v>0</v>
@@ -2499,19 +2499,19 @@
         <v>0.4</v>
       </c>
       <c r="G44" t="n">
-        <v>0.08290061396627718</v>
+        <v>0.0829006139662772</v>
       </c>
       <c r="H44" t="n">
-        <v>0.03813142532335363</v>
+        <v>0.03813142532335365</v>
       </c>
       <c r="I44" t="n">
-        <v>0.04285382631742517</v>
+        <v>0.04285382631742519</v>
       </c>
       <c r="J44" t="n">
-        <v>5.895611618411005</v>
+        <v>5.895611618410998</v>
       </c>
       <c r="K44" t="n">
-        <v>33.62570084422528</v>
+        <v>33.62570084422525</v>
       </c>
       <c r="L44" t="n">
         <v>18.23441753777161</v>
@@ -2520,7 +2520,7 @@
         <v>0.2233067431983749</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2555009329807319</v>
+        <v>0.255500932980732</v>
       </c>
       <c r="O44" t="n">
         <v>0.3931787010556945</v>
@@ -2546,22 +2546,22 @@
         <v>0.4</v>
       </c>
       <c r="G45" t="n">
-        <v>0.09234950013810866</v>
+        <v>0.09234950013810871</v>
       </c>
       <c r="H45" t="n">
-        <v>0.03143366651432928</v>
+        <v>0.03143366651432929</v>
       </c>
       <c r="I45" t="n">
-        <v>0.03651965914549592</v>
+        <v>0.03651965914549555</v>
       </c>
       <c r="J45" t="n">
-        <v>5.290573350413714</v>
+        <v>5.290573350413711</v>
       </c>
       <c r="K45" t="n">
-        <v>42.20298227902118</v>
+        <v>42.20298227902115</v>
       </c>
       <c r="L45" t="n">
-        <v>21.54165341987479</v>
+        <v>21.54165341987366</v>
       </c>
       <c r="M45" t="n">
         <v>0.2233067431983749</v>
@@ -2570,12 +2570,12 @@
         <v>0.2532857203499647</v>
       </c>
       <c r="O45" t="n">
-        <v>0.3890752455606723</v>
+        <v>0.3890752455606724</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>-4.250303122410516</v>
+        <v>-4.250303122410211</v>
       </c>
       <c r="B46" t="n">
         <v>0</v>
@@ -2593,36 +2593,36 @@
         <v>0.4</v>
       </c>
       <c r="G46" t="n">
-        <v>0.1009126975550364</v>
+        <v>0.1009126975550359</v>
       </c>
       <c r="H46" t="n">
-        <v>0.02584876085598063</v>
+        <v>0.02584876085598064</v>
       </c>
       <c r="I46" t="n">
-        <v>0.02932870132767478</v>
+        <v>0.0293287013276748</v>
       </c>
       <c r="J46" t="n">
-        <v>4.840507364843528</v>
+        <v>4.840507364843524</v>
       </c>
       <c r="K46" t="n">
-        <v>54.77566620013776</v>
+        <v>54.77566620013771</v>
       </c>
       <c r="L46" t="n">
-        <v>27.20683075441298</v>
+        <v>27.20683075441296</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2234097331711457</v>
+        <v>0.2234097331711462</v>
       </c>
       <c r="N46" t="n">
         <v>0.2507811527364971</v>
       </c>
       <c r="O46" t="n">
-        <v>0.3861631856709811</v>
+        <v>0.386163185670981</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>-76.42160455465952</v>
+        <v>-76.42160455473605</v>
       </c>
       <c r="B47" t="n">
         <v>90</v>
@@ -2640,19 +2640,19 @@
         <v>0.4</v>
       </c>
       <c r="G47" t="n">
-        <v>0.06253281370900612</v>
+        <v>0.06253281370900741</v>
       </c>
       <c r="H47" t="n">
-        <v>0.05374012161169871</v>
+        <v>0.05374012161169264</v>
       </c>
       <c r="I47" t="n">
-        <v>0.0466498374830521</v>
+        <v>0.04664983748305208</v>
       </c>
       <c r="J47" t="n">
-        <v>7.826424365587972</v>
+        <v>7.826424365586904</v>
       </c>
       <c r="K47" t="n">
-        <v>23.13664256803825</v>
+        <v>23.13664256804039</v>
       </c>
       <c r="L47" t="n">
         <v>16.70497128283072</v>
@@ -2661,7 +2661,7 @@
         <v>0.2233067431983749</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2568340937002471</v>
+        <v>0.2568340937002536</v>
       </c>
       <c r="O47" t="n">
         <v>0.3941887549969388</v>
@@ -2690,19 +2690,19 @@
         <v>0.07286844709700188</v>
       </c>
       <c r="H48" t="n">
-        <v>0.04595012646737649</v>
+        <v>0.04595012646737647</v>
       </c>
       <c r="I48" t="n">
-        <v>0.04018724477812764</v>
+        <v>0.04018724477812765</v>
       </c>
       <c r="J48" t="n">
-        <v>6.710793399280202</v>
+        <v>6.7107933992802</v>
       </c>
       <c r="K48" t="n">
-        <v>27.35733293447958</v>
+        <v>27.35733293447959</v>
       </c>
       <c r="L48" t="n">
-        <v>19.49156123182587</v>
+        <v>19.49156123182586</v>
       </c>
       <c r="M48" t="n">
         <v>0.2233067431983749</v>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>-50.69076862725352</v>
+        <v>-50.69076862697345</v>
       </c>
       <c r="B49" t="n">
         <v>90</v>
@@ -2734,28 +2734,28 @@
         <v>0.4</v>
       </c>
       <c r="G49" t="n">
-        <v>0.08290061396627713</v>
+        <v>0.08290061396627714</v>
       </c>
       <c r="H49" t="n">
-        <v>0.03813142532332501</v>
+        <v>0.03813142532335366</v>
       </c>
       <c r="I49" t="n">
-        <v>0.03458725640844371</v>
+        <v>0.03458725640844367</v>
       </c>
       <c r="J49" t="n">
-        <v>5.895611618410974</v>
+        <v>5.895611618411034</v>
       </c>
       <c r="K49" t="n">
-        <v>33.62570084427983</v>
+        <v>33.62570084422525</v>
       </c>
       <c r="L49" t="n">
-        <v>22.81095729597293</v>
+        <v>22.81095729597295</v>
       </c>
       <c r="M49" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N49" t="n">
-        <v>0.2555009329807549</v>
+        <v>0.255500932980732</v>
       </c>
       <c r="O49" t="n">
         <v>0.3876735198590205</v>
@@ -2781,22 +2781,22 @@
         <v>0.4</v>
       </c>
       <c r="G50" t="n">
-        <v>0.09234950013810855</v>
+        <v>0.09234950013810858</v>
       </c>
       <c r="H50" t="n">
-        <v>0.03143366651432927</v>
+        <v>0.03143366651432929</v>
       </c>
       <c r="I50" t="n">
-        <v>0.02646993929768663</v>
+        <v>0.02646993929768673</v>
       </c>
       <c r="J50" t="n">
-        <v>5.290573350413738</v>
+        <v>5.290573350413736</v>
       </c>
       <c r="K50" t="n">
-        <v>42.20298227902118</v>
+        <v>42.20298227902116</v>
       </c>
       <c r="L50" t="n">
-        <v>30.4364344503652</v>
+        <v>30.43643445036488</v>
       </c>
       <c r="M50" t="n">
         <v>0.2233067431983749</v>
@@ -2810,7 +2810,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>-3.042554373986383</v>
+        <v>-3.042554374020402</v>
       </c>
       <c r="B51" t="n">
         <v>90</v>
@@ -2828,36 +2828,36 @@
         <v>0.4</v>
       </c>
       <c r="G51" t="n">
-        <v>0.1009126975550345</v>
+        <v>0.1009126975550343</v>
       </c>
       <c r="H51" t="n">
         <v>0.02584876085598058</v>
       </c>
       <c r="I51" t="n">
-        <v>0.01816163491276473</v>
+        <v>0.01816163491234823</v>
       </c>
       <c r="J51" t="n">
-        <v>4.840507364843493</v>
+        <v>4.840507364843507</v>
       </c>
       <c r="K51" t="n">
-        <v>54.77566620013793</v>
+        <v>54.77566620013792</v>
       </c>
       <c r="L51" t="n">
-        <v>47.58896943276076</v>
+        <v>47.58896943295241</v>
       </c>
       <c r="M51" t="n">
-        <v>0.2234097331711475</v>
+        <v>0.2234097331711476</v>
       </c>
       <c r="N51" t="n">
         <v>0.2507811527364971</v>
       </c>
       <c r="O51" t="n">
-        <v>0.3856904333205197</v>
+        <v>0.3856904333205332</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>-105.6007045617834</v>
+        <v>-105.6007045617824</v>
       </c>
       <c r="B52" t="n">
         <v>0</v>
@@ -2875,31 +2875,31 @@
         <v>0.5</v>
       </c>
       <c r="G52" t="n">
-        <v>0.06253281370900604</v>
+        <v>0.06253281370900747</v>
       </c>
       <c r="H52" t="n">
-        <v>0.05284501332225697</v>
+        <v>0.05284501332225705</v>
       </c>
       <c r="I52" t="n">
-        <v>0.05811454416478454</v>
+        <v>0.05811454416478445</v>
       </c>
       <c r="J52" t="n">
-        <v>7.826424365588002</v>
+        <v>7.826424365587113</v>
       </c>
       <c r="K52" t="n">
-        <v>23.55197526790209</v>
+        <v>23.55197526790207</v>
       </c>
       <c r="L52" t="n">
-        <v>13.34048898254781</v>
+        <v>13.34048898254783</v>
       </c>
       <c r="M52" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N52" t="n">
-        <v>0.2578090018825936</v>
+        <v>0.2578090018825935</v>
       </c>
       <c r="O52" t="n">
-        <v>0.3971872205136741</v>
+        <v>0.3971872205136742</v>
       </c>
     </row>
     <row r="53">
@@ -2922,22 +2922,22 @@
         <v>0.5</v>
       </c>
       <c r="G53" t="n">
-        <v>0.07286844709700201</v>
+        <v>0.07286844709700198</v>
       </c>
       <c r="H53" t="n">
         <v>0.04517647695346255</v>
       </c>
       <c r="I53" t="n">
-        <v>0.04995746552036978</v>
+        <v>0.04995746552036975</v>
       </c>
       <c r="J53" t="n">
-        <v>6.710793399280155</v>
+        <v>6.710793399280168</v>
       </c>
       <c r="K53" t="n">
-        <v>27.86618434622165</v>
+        <v>27.86618434622164</v>
       </c>
       <c r="L53" t="n">
-        <v>15.56981144556587</v>
+        <v>15.56981144556588</v>
       </c>
       <c r="M53" t="n">
         <v>0.2233067431983749</v>
@@ -2951,7 +2951,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>-86.77298660120758</v>
+        <v>-86.77298660120849</v>
       </c>
       <c r="B54" t="n">
         <v>0</v>
@@ -2969,22 +2969,22 @@
         <v>0.5</v>
       </c>
       <c r="G54" t="n">
-        <v>0.08290061396627717</v>
+        <v>0.08290061396627715</v>
       </c>
       <c r="H54" t="n">
-        <v>0.03750949946203072</v>
+        <v>0.03750949946203073</v>
       </c>
       <c r="I54" t="n">
-        <v>0.04200095174734981</v>
+        <v>0.04200095174734971</v>
       </c>
       <c r="J54" t="n">
-        <v>5.895611618410962</v>
+        <v>5.895611618410975</v>
       </c>
       <c r="K54" t="n">
-        <v>34.25983519634898</v>
+        <v>34.25983519634897</v>
       </c>
       <c r="L54" t="n">
-        <v>18.61814204367815</v>
+        <v>18.61814204367817</v>
       </c>
       <c r="M54" t="n">
         <v>0.2233067431983749</v>
@@ -2993,12 +2993,12 @@
         <v>0.256250594914497</v>
       </c>
       <c r="O54" t="n">
-        <v>0.3940776594204369</v>
+        <v>0.3940776594204371</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>-38.31889955855554</v>
+        <v>-38.31889955680907</v>
       </c>
       <c r="B55" t="n">
         <v>0</v>
@@ -3016,36 +3016,36 @@
         <v>0.5</v>
       </c>
       <c r="G55" t="n">
-        <v>0.09234950013810868</v>
+        <v>0.09234950013810865</v>
       </c>
       <c r="H55" t="n">
-        <v>0.03114566494696002</v>
+        <v>0.03114566494700652</v>
       </c>
       <c r="I55" t="n">
-        <v>0.0361533932154845</v>
+        <v>0.0361533932154844</v>
       </c>
       <c r="J55" t="n">
-        <v>5.29057335041369</v>
+        <v>5.29057335041371</v>
       </c>
       <c r="K55" t="n">
-        <v>42.68528109967677</v>
+        <v>42.68528109921959</v>
       </c>
       <c r="L55" t="n">
-        <v>21.77097090044414</v>
+        <v>21.77097090044437</v>
       </c>
       <c r="M55" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N55" t="n">
-        <v>0.2536759968997472</v>
+        <v>0.2536759968995701</v>
       </c>
       <c r="O55" t="n">
-        <v>0.3894693273209706</v>
+        <v>0.3894693273209707</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>-5.241026242514176</v>
+        <v>-5.241026242617323</v>
       </c>
       <c r="B56" t="n">
         <v>0</v>
@@ -3063,36 +3063,36 @@
         <v>0.5</v>
       </c>
       <c r="G56" t="n">
-        <v>0.1009126975550345</v>
+        <v>0.1009126975550369</v>
       </c>
       <c r="H56" t="n">
-        <v>0.02579447917698827</v>
+        <v>0.02579447917697798</v>
       </c>
       <c r="I56" t="n">
-        <v>0.02920422465186822</v>
+        <v>0.02920422465186813</v>
       </c>
       <c r="J56" t="n">
-        <v>4.840507364843496</v>
+        <v>4.840507364843523</v>
       </c>
       <c r="K56" t="n">
-        <v>54.94679715556396</v>
+        <v>54.94679715558353</v>
       </c>
       <c r="L56" t="n">
-        <v>27.33244577281044</v>
+        <v>27.33244577281015</v>
       </c>
       <c r="M56" t="n">
-        <v>0.2234097331711475</v>
+        <v>0.2234097331711451</v>
       </c>
       <c r="N56" t="n">
-        <v>0.2508754639120787</v>
+        <v>0.2508754639120936</v>
       </c>
       <c r="O56" t="n">
-        <v>0.3863032263745172</v>
+        <v>0.3863032263745174</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>-94.08159725243644</v>
+        <v>-94.08159725244244</v>
       </c>
       <c r="B57" t="n">
         <v>90</v>
@@ -3110,28 +3110,28 @@
         <v>0.5</v>
       </c>
       <c r="G57" t="n">
-        <v>0.06253281370900646</v>
+        <v>0.06253281370900746</v>
       </c>
       <c r="H57" t="n">
-        <v>0.05284501332225697</v>
+        <v>0.05284501332225648</v>
       </c>
       <c r="I57" t="n">
-        <v>0.04553845952396245</v>
+        <v>0.04553845952396243</v>
       </c>
       <c r="J57" t="n">
-        <v>7.826424365587863</v>
+        <v>7.826424365586936</v>
       </c>
       <c r="K57" t="n">
-        <v>23.55197526790209</v>
+        <v>23.55197526790228</v>
       </c>
       <c r="L57" t="n">
-        <v>17.12508515582563</v>
+        <v>17.12508515582564</v>
       </c>
       <c r="M57" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N57" t="n">
-        <v>0.2578090018825936</v>
+        <v>0.2578090018825941</v>
       </c>
       <c r="O57" t="n">
         <v>0.3953503805418446</v>
@@ -3157,22 +3157,22 @@
         <v>0.5</v>
       </c>
       <c r="G58" t="n">
-        <v>0.07286844709700188</v>
+        <v>0.07286844709700187</v>
       </c>
       <c r="H58" t="n">
         <v>0.0451764769534625</v>
       </c>
       <c r="I58" t="n">
-        <v>0.03955602594162057</v>
+        <v>0.03955602594162056</v>
       </c>
       <c r="J58" t="n">
-        <v>6.710793399280131</v>
+        <v>6.710793399280186</v>
       </c>
       <c r="K58" t="n">
         <v>27.86618434622168</v>
       </c>
       <c r="L58" t="n">
-        <v>19.81550707233749</v>
+        <v>19.8155070723375</v>
       </c>
       <c r="M58" t="n">
         <v>0.2233067431983749</v>
@@ -3186,7 +3186,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>-61.21310125306579</v>
+        <v>-61.21310125306553</v>
       </c>
       <c r="B59" t="n">
         <v>90</v>
@@ -3207,16 +3207,16 @@
         <v>0.08290061396627711</v>
       </c>
       <c r="H59" t="n">
-        <v>0.03750949946203075</v>
+        <v>0.03750949946203074</v>
       </c>
       <c r="I59" t="n">
         <v>0.03432360740363118</v>
       </c>
       <c r="J59" t="n">
-        <v>5.895611618410967</v>
+        <v>5.895611618410983</v>
       </c>
       <c r="K59" t="n">
-        <v>34.25983519634895</v>
+        <v>34.25983519634896</v>
       </c>
       <c r="L59" t="n">
         <v>22.99618550237965</v>
@@ -3233,7 +3233,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>-27.70191178770897</v>
+        <v>-27.70191178772084</v>
       </c>
       <c r="B60" t="n">
         <v>90</v>
@@ -3251,36 +3251,36 @@
         <v>0.5</v>
       </c>
       <c r="G60" t="n">
-        <v>0.09234950013810857</v>
+        <v>0.09234950013810855</v>
       </c>
       <c r="H60" t="n">
-        <v>0.03114566494713082</v>
+        <v>0.03114566494708874</v>
       </c>
       <c r="I60" t="n">
-        <v>0.02638044736320578</v>
+        <v>0.02638044736324819</v>
       </c>
       <c r="J60" t="n">
-        <v>5.290573350413696</v>
+        <v>5.2905733504137</v>
       </c>
       <c r="K60" t="n">
-        <v>42.68528109966964</v>
+        <v>42.68528109955214</v>
       </c>
       <c r="L60" t="n">
-        <v>30.55070260528415</v>
+        <v>30.55070260500082</v>
       </c>
       <c r="M60" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N60" t="n">
-        <v>0.253675996899602</v>
+        <v>0.2536759968995991</v>
       </c>
       <c r="O60" t="n">
-        <v>0.3860827097131312</v>
+        <v>0.3860827097131461</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>-125.591759311951</v>
+        <v>-125.5917593119707</v>
       </c>
       <c r="B61" t="n">
         <v>0</v>
@@ -3301,33 +3301,33 @@
         <v>0.06253281370900748</v>
       </c>
       <c r="H61" t="n">
-        <v>0.05206181221762847</v>
+        <v>0.05206181221762722</v>
       </c>
       <c r="I61" t="n">
-        <v>0.056930046342184</v>
+        <v>0.05693004634218404</v>
       </c>
       <c r="J61" t="n">
-        <v>7.826424365587129</v>
+        <v>7.826424365587116</v>
       </c>
       <c r="K61" t="n">
-        <v>23.92822840330427</v>
+        <v>23.92822840330471</v>
       </c>
       <c r="L61" t="n">
-        <v>13.62334758109314</v>
+        <v>13.62334758109313</v>
       </c>
       <c r="M61" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N61" t="n">
-        <v>0.2586645984557456</v>
+        <v>0.258664598455747</v>
       </c>
       <c r="O61" t="n">
-        <v>0.3984052801340792</v>
+        <v>0.3984052801340791</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>-124.9726806301973</v>
+        <v>-124.9726806301006</v>
       </c>
       <c r="B62" t="n">
         <v>0</v>
@@ -3351,16 +3351,16 @@
         <v>0.04451004594634805</v>
       </c>
       <c r="I62" t="n">
-        <v>0.04888505038249234</v>
+        <v>0.04888505038250703</v>
       </c>
       <c r="J62" t="n">
-        <v>6.710793399280183</v>
+        <v>6.710793399280194</v>
       </c>
       <c r="K62" t="n">
         <v>28.32071128784096</v>
       </c>
       <c r="L62" t="n">
-        <v>15.92033848923271</v>
+        <v>15.92033848923236</v>
       </c>
       <c r="M62" t="n">
         <v>0.2233067431983749</v>
@@ -3369,12 +3369,12 @@
         <v>0.2580927246502468</v>
       </c>
       <c r="O62" t="n">
-        <v>0.3972485697776933</v>
+        <v>0.3972485697776791</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>-99.98753074832327</v>
+        <v>-99.9875307495395</v>
       </c>
       <c r="B63" t="n">
         <v>0</v>
@@ -3392,19 +3392,19 @@
         <v>0.6</v>
       </c>
       <c r="G63" t="n">
-        <v>0.08290061396627717</v>
+        <v>0.08290061396627718</v>
       </c>
       <c r="H63" t="n">
-        <v>0.03697816719472796</v>
+        <v>0.03697816719465051</v>
       </c>
       <c r="I63" t="n">
-        <v>0.04131635721642441</v>
+        <v>0.04131635721642452</v>
       </c>
       <c r="J63" t="n">
-        <v>5.895611618411015</v>
+        <v>5.895611618411031</v>
       </c>
       <c r="K63" t="n">
-        <v>34.82247882546618</v>
+        <v>34.82247882550449</v>
       </c>
       <c r="L63" t="n">
         <v>18.93827692002482</v>
@@ -3413,10 +3413,10 @@
         <v>0.2233067431983749</v>
       </c>
       <c r="N63" t="n">
-        <v>0.2568956277355651</v>
+        <v>0.2568956277356471</v>
       </c>
       <c r="O63" t="n">
-        <v>0.3948007395673536</v>
+        <v>0.3948007395673535</v>
       </c>
     </row>
     <row r="64">
@@ -3442,19 +3442,19 @@
         <v>0.09234950013810865</v>
       </c>
       <c r="H64" t="n">
-        <v>0.0309025697346174</v>
+        <v>0.03090256973461741</v>
       </c>
       <c r="I64" t="n">
-        <v>0.03584782017393863</v>
+        <v>0.03584782017393866</v>
       </c>
       <c r="J64" t="n">
-        <v>5.290573350413692</v>
+        <v>5.290573350413734</v>
       </c>
       <c r="K64" t="n">
-        <v>43.10238083566319</v>
+        <v>43.10238083566318</v>
       </c>
       <c r="L64" t="n">
-        <v>21.96616282057358</v>
+        <v>21.96616282057355</v>
       </c>
       <c r="M64" t="n">
         <v>0.2233067431983749</v>
@@ -3468,7 +3468,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>-6.198986441398104</v>
+        <v>-6.198986441340729</v>
       </c>
       <c r="B65" t="n">
         <v>0</v>
@@ -3486,31 +3486,31 @@
         <v>0.6</v>
       </c>
       <c r="G65" t="n">
-        <v>0.1009126975550362</v>
+        <v>0.1009126975550345</v>
       </c>
       <c r="H65" t="n">
-        <v>0.02574301647281753</v>
+        <v>0.02574301647282797</v>
       </c>
       <c r="I65" t="n">
-        <v>0.02908495983906084</v>
+        <v>0.02908495983905512</v>
       </c>
       <c r="J65" t="n">
-        <v>4.840507364843384</v>
+        <v>4.840507364843498</v>
       </c>
       <c r="K65" t="n">
-        <v>55.11038694465446</v>
+        <v>55.11038694463954</v>
       </c>
       <c r="L65" t="n">
-        <v>27.45394522318793</v>
+        <v>27.45394522315731</v>
       </c>
       <c r="M65" t="n">
-        <v>0.2234097331711458</v>
+        <v>0.2234097331711476</v>
       </c>
       <c r="N65" t="n">
-        <v>0.2509652503076652</v>
+        <v>0.2509652503076515</v>
       </c>
       <c r="O65" t="n">
-        <v>0.3864375531806671</v>
+        <v>0.3864375531806808</v>
       </c>
     </row>
     <row r="66">
@@ -3533,19 +3533,19 @@
         <v>0.6</v>
       </c>
       <c r="G66" t="n">
-        <v>0.06253281370900744</v>
+        <v>0.06253281370900746</v>
       </c>
       <c r="H66" t="n">
-        <v>0.0520618122176285</v>
+        <v>0.05206181221762846</v>
       </c>
       <c r="I66" t="n">
-        <v>0.04461769208977837</v>
+        <v>0.04461769208977839</v>
       </c>
       <c r="J66" t="n">
-        <v>7.826424365586902</v>
+        <v>7.826424365587132</v>
       </c>
       <c r="K66" t="n">
-        <v>23.92822840330425</v>
+        <v>23.92822840330427</v>
       </c>
       <c r="L66" t="n">
         <v>17.48976658697977</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>-100.6355298693539</v>
+        <v>-100.6355298693543</v>
       </c>
       <c r="B67" t="n">
         <v>90</v>
@@ -3580,22 +3580,22 @@
         <v>0.6</v>
       </c>
       <c r="G67" t="n">
-        <v>0.07286844709700187</v>
+        <v>0.07286844709700185</v>
       </c>
       <c r="H67" t="n">
-        <v>0.04451004594634798</v>
+        <v>0.04451004594634796</v>
       </c>
       <c r="I67" t="n">
-        <v>0.03904829209155163</v>
+        <v>0.03904829209155155</v>
       </c>
       <c r="J67" t="n">
-        <v>6.710793399280161</v>
+        <v>6.710793399280164</v>
       </c>
       <c r="K67" t="n">
-        <v>28.32071128784101</v>
+        <v>28.32071128784102</v>
       </c>
       <c r="L67" t="n">
-        <v>20.08417960251279</v>
+        <v>20.08417960251285</v>
       </c>
       <c r="M67" t="n">
         <v>0.2233067431983749</v>
@@ -3604,12 +3604,12 @@
         <v>0.2580927246502468</v>
       </c>
       <c r="O67" t="n">
-        <v>0.3930465745880458</v>
+        <v>0.3930465745880459</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>-71.14169096218303</v>
+        <v>-71.14169096172411</v>
       </c>
       <c r="B68" t="n">
         <v>90</v>
@@ -3627,28 +3627,28 @@
         <v>0.6</v>
       </c>
       <c r="G68" t="n">
-        <v>0.08290061396627713</v>
+        <v>0.08290061396627715</v>
       </c>
       <c r="H68" t="n">
-        <v>0.03697816719469263</v>
+        <v>0.03697816719472178</v>
       </c>
       <c r="I68" t="n">
-        <v>0.03409538955549331</v>
+        <v>0.03409538955549326</v>
       </c>
       <c r="J68" t="n">
-        <v>5.895611618411012</v>
+        <v>5.895611618411038</v>
       </c>
       <c r="K68" t="n">
-        <v>34.8224788254841</v>
+        <v>34.82247882546947</v>
       </c>
       <c r="L68" t="n">
-        <v>23.15904411400869</v>
+        <v>23.15904411400875</v>
       </c>
       <c r="M68" t="n">
         <v>0.2233067431983749</v>
       </c>
       <c r="N68" t="n">
-        <v>0.2568956277356027</v>
+        <v>0.2568956277355718</v>
       </c>
       <c r="O68" t="n">
         <v>0.3882078027014921</v>
@@ -3656,7 +3656,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>-31.32232852952007</v>
+        <v>-31.3223285295203</v>
       </c>
       <c r="B69" t="n">
         <v>90</v>
@@ -3674,22 +3674,22 @@
         <v>0.6</v>
       </c>
       <c r="G69" t="n">
-        <v>0.09234950013810855</v>
+        <v>0.09234950013810854</v>
       </c>
       <c r="H69" t="n">
-        <v>0.03090256973461743</v>
+        <v>0.03090256973461742</v>
       </c>
       <c r="I69" t="n">
-        <v>0.02629358878188282</v>
+        <v>0.02629358878188277</v>
       </c>
       <c r="J69" t="n">
-        <v>5.290573350413714</v>
+        <v>5.29057335041372</v>
       </c>
       <c r="K69" t="n">
         <v>43.10238083566315</v>
       </c>
       <c r="L69" t="n">
-        <v>30.6624822621529</v>
+        <v>30.66248226215296</v>
       </c>
       <c r="M69" t="n">
         <v>0.2233067431983749</v>
@@ -3703,7 +3703,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>-5.204632781733212</v>
+        <v>-5.204632782141784</v>
       </c>
       <c r="B70" t="n">
         <v>0</v>
@@ -3721,36 +3721,36 @@
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>0.06154629117246532</v>
+        <v>0.06154629117246606</v>
       </c>
       <c r="H70" t="n">
-        <v>0.0587983185540708</v>
+        <v>0.05879831855407184</v>
       </c>
       <c r="I70" t="n">
-        <v>0.0687058341830261</v>
+        <v>0.06870583418290459</v>
       </c>
       <c r="J70" t="n">
-        <v>7.952679075938929</v>
+        <v>7.952679075938698</v>
       </c>
       <c r="K70" t="n">
-        <v>21.04637177567141</v>
+        <v>21.04637177567112</v>
       </c>
       <c r="L70" t="n">
-        <v>11.25455325771212</v>
+        <v>11.25455325771582</v>
       </c>
       <c r="M70" t="n">
-        <v>0.2243026922815005</v>
+        <v>0.2243026922814998</v>
       </c>
       <c r="N70" t="n">
-        <v>0.2513760312601668</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O70" t="n">
-        <v>0.3863489999530983</v>
+        <v>0.3863489999532831</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2.616182374182528</v>
+        <v>2.616182374159362</v>
       </c>
       <c r="B71" t="n">
         <v>0</v>
@@ -3768,28 +3768,28 @@
         <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>0.07123578465959628</v>
+        <v>0.07123578465959625</v>
       </c>
       <c r="H71" t="n">
-        <v>0.05137435493582272</v>
+        <v>0.05137435493611308</v>
       </c>
       <c r="I71" t="n">
-        <v>0.06024037485416535</v>
+        <v>0.06024037485416537</v>
       </c>
       <c r="J71" t="n">
-        <v>6.865330878014234</v>
+        <v>6.865330878014237</v>
       </c>
       <c r="K71" t="n">
-        <v>24.2688837176025</v>
+        <v>24.26888371725402</v>
       </c>
       <c r="L71" t="n">
-        <v>12.86148801950007</v>
+        <v>12.86148801950022</v>
       </c>
       <c r="M71" t="n">
         <v>0.224950929640578</v>
       </c>
       <c r="N71" t="n">
-        <v>0.2504409517469671</v>
+        <v>0.2504409517469713</v>
       </c>
       <c r="O71" t="n">
         <v>0.3855295790644589</v>
@@ -3815,22 +3815,22 @@
         <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>0.08102967644508628</v>
+        <v>0.08102967644508627</v>
       </c>
       <c r="H72" t="n">
-        <v>0.04252156872771578</v>
+        <v>0.04252156913916048</v>
       </c>
       <c r="I72" t="n">
-        <v>0.05017595975349042</v>
+        <v>0.05017595975381715</v>
       </c>
       <c r="J72" t="n">
-        <v>6.032237977037229</v>
+        <v>6.032237977037231</v>
       </c>
       <c r="K72" t="n">
-        <v>29.77475594546965</v>
+        <v>29.77475551531234</v>
       </c>
       <c r="L72" t="n">
-        <v>15.50030379117783</v>
+        <v>15.50030379108488</v>
       </c>
       <c r="M72" t="n">
         <v>0.2251878609156901</v>
@@ -3844,7 +3844,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>3.603138488130419</v>
+        <v>3.603138488119877</v>
       </c>
       <c r="B73" t="n">
         <v>0</v>
@@ -3862,28 +3862,28 @@
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>0.09030283936502725</v>
+        <v>0.09030283936502721</v>
       </c>
       <c r="H73" t="n">
-        <v>0.03367093419815972</v>
+        <v>0.03367093314372721</v>
       </c>
       <c r="I73" t="n">
-        <v>0.03983894172867027</v>
+        <v>0.03983894172626346</v>
       </c>
       <c r="J73" t="n">
-        <v>5.410834816976491</v>
+        <v>5.410834816976494</v>
       </c>
       <c r="K73" t="n">
-        <v>38.83825833629182</v>
+        <v>38.83826049322944</v>
       </c>
       <c r="L73" t="n">
-        <v>19.66896230269321</v>
+        <v>19.66896230388018</v>
       </c>
       <c r="M73" t="n">
-        <v>0.2253623600619389</v>
+        <v>0.225362360061939</v>
       </c>
       <c r="N73" t="n">
-        <v>0.2503438825093872</v>
+        <v>0.2503438825093889</v>
       </c>
       <c r="O73" t="n">
         <v>0.3855295790644589</v>
@@ -3891,7 +3891,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>3.449142741714106</v>
+        <v>3.449142741714199</v>
       </c>
       <c r="B74" t="n">
         <v>0</v>
@@ -3909,22 +3909,22 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>0.0988649465067936</v>
+        <v>0.09886494650679359</v>
       </c>
       <c r="H74" t="n">
-        <v>0.02610341344142092</v>
+        <v>0.02610341279462003</v>
       </c>
       <c r="I74" t="n">
-        <v>0.02989360933762751</v>
+        <v>0.02989360965347651</v>
       </c>
       <c r="J74" t="n">
-        <v>4.941013633050771</v>
+        <v>4.941013633050773</v>
       </c>
       <c r="K74" t="n">
-        <v>53.99159103989486</v>
+        <v>53.9915895180409</v>
       </c>
       <c r="L74" t="n">
-        <v>26.65159194378405</v>
+        <v>26.65159161121834</v>
       </c>
       <c r="M74" t="n">
         <v>0.2254649664177308</v>
@@ -3938,7 +3938,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>-3.438866149406217</v>
+        <v>-3.438866149446009</v>
       </c>
       <c r="B75" t="n">
         <v>90</v>
@@ -3956,28 +3956,28 @@
         <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>0.0615462911724427</v>
+        <v>0.06154629117246656</v>
       </c>
       <c r="H75" t="n">
-        <v>0.05879831855407171</v>
+        <v>0.05879831855407185</v>
       </c>
       <c r="I75" t="n">
-        <v>0.05499992440104674</v>
+        <v>0.05499992440104677</v>
       </c>
       <c r="J75" t="n">
-        <v>7.952679075946946</v>
+        <v>7.952679075938473</v>
       </c>
       <c r="K75" t="n">
-        <v>21.04637177567115</v>
+        <v>21.04637177567111</v>
       </c>
       <c r="L75" t="n">
-        <v>14.11116142850669</v>
+        <v>14.11116142850674</v>
       </c>
       <c r="M75" t="n">
-        <v>0.2243026922815197</v>
+        <v>0.2243026922814994</v>
       </c>
       <c r="N75" t="n">
-        <v>0.2513760312601658</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O75" t="n">
         <v>0.3855295790644589</v>
@@ -3985,7 +3985,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>2.616182374108389</v>
+        <v>2.616182374160751</v>
       </c>
       <c r="B76" t="n">
         <v>90</v>
@@ -4003,28 +4003,28 @@
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>0.07123578465959617</v>
+        <v>0.07123578465959614</v>
       </c>
       <c r="H76" t="n">
-        <v>0.05137435493609432</v>
+        <v>0.05137435493611123</v>
       </c>
       <c r="I76" t="n">
-        <v>0.04618037325629579</v>
+        <v>0.04618037325587039</v>
       </c>
       <c r="J76" t="n">
-        <v>6.865330878014246</v>
+        <v>6.865330878014248</v>
       </c>
       <c r="K76" t="n">
-        <v>24.26888371725414</v>
+        <v>24.26888371725647</v>
       </c>
       <c r="L76" t="n">
-        <v>16.87985375469492</v>
+        <v>16.87985375484184</v>
       </c>
       <c r="M76" t="n">
         <v>0.224950929640578</v>
       </c>
       <c r="N76" t="n">
-        <v>0.2504409517469806</v>
+        <v>0.2504409517469711</v>
       </c>
       <c r="O76" t="n">
         <v>0.3855295790644589</v>
@@ -4050,22 +4050,22 @@
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>0.08102967644508623</v>
+        <v>0.08102967644508627</v>
       </c>
       <c r="H77" t="n">
-        <v>0.04252156914041653</v>
+        <v>0.0425215691396317</v>
       </c>
       <c r="I77" t="n">
-        <v>0.03657296377556265</v>
+        <v>0.03657296366026039</v>
       </c>
       <c r="J77" t="n">
-        <v>6.032237977037234</v>
+        <v>6.032237977037231</v>
       </c>
       <c r="K77" t="n">
-        <v>29.77475551392189</v>
+        <v>29.77475551477808</v>
       </c>
       <c r="L77" t="n">
-        <v>21.50869238381966</v>
+        <v>21.50869244443578</v>
       </c>
       <c r="M77" t="n">
         <v>0.2251878609156901</v>
@@ -4079,7 +4079,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>3.603138488137268</v>
+        <v>3.603138488130529</v>
       </c>
       <c r="B78" t="n">
         <v>90</v>
@@ -4097,22 +4097,22 @@
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>0.09030283936502713</v>
+        <v>0.09030283936502716</v>
       </c>
       <c r="H78" t="n">
-        <v>0.03367093419819458</v>
+        <v>0.03367093419840163</v>
       </c>
       <c r="I78" t="n">
-        <v>0.02685826388011748</v>
+        <v>0.02685825559878237</v>
       </c>
       <c r="J78" t="n">
-        <v>5.410834816976499</v>
+        <v>5.410834816976497</v>
       </c>
       <c r="K78" t="n">
-        <v>38.83825833642793</v>
+        <v>38.83825833712859</v>
       </c>
       <c r="L78" t="n">
-        <v>29.95091013268939</v>
+        <v>29.9509202316852</v>
       </c>
       <c r="M78" t="n">
         <v>0.225362360061939</v>
@@ -4121,7 +4121,7 @@
         <v>0.2503438825093872</v>
       </c>
       <c r="O78" t="n">
-        <v>0.3855295790644563</v>
+        <v>0.3855295790644589</v>
       </c>
     </row>
     <row r="79">
@@ -4144,22 +4144,22 @@
         <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>0.09886494650679351</v>
+        <v>0.09886494650679348</v>
       </c>
       <c r="H79" t="n">
-        <v>0.02610341344139507</v>
+        <v>0.02610341344142605</v>
       </c>
       <c r="I79" t="n">
-        <v>0.01827050818593203</v>
+        <v>0.01827050818593176</v>
       </c>
       <c r="J79" t="n">
-        <v>4.941013633050777</v>
+        <v>4.941013633050778</v>
       </c>
       <c r="K79" t="n">
-        <v>53.99159103998119</v>
+        <v>53.99159103987864</v>
       </c>
       <c r="L79" t="n">
-        <v>47.21653013893589</v>
+        <v>47.2165301389365</v>
       </c>
       <c r="M79" t="n">
         <v>0.2254649664177308</v>
@@ -4173,7 +4173,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>-3.655407251231122</v>
+        <v>-3.655407251649357</v>
       </c>
       <c r="B80" t="n">
         <v>0</v>
@@ -4191,36 +4191,36 @@
         <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>0.0608189950831126</v>
+        <v>0.06081899508311623</v>
       </c>
       <c r="H80" t="n">
-        <v>0.05879831855407186</v>
+        <v>0.05879831855407187</v>
       </c>
       <c r="I80" t="n">
-        <v>0.06870583418309247</v>
+        <v>0.06870583418290985</v>
       </c>
       <c r="J80" t="n">
-        <v>8.048406845210586</v>
+        <v>8.048406845208371</v>
       </c>
       <c r="K80" t="n">
         <v>21.0463717756711</v>
       </c>
       <c r="L80" t="n">
-        <v>11.25455325768399</v>
+        <v>11.2545532577169</v>
       </c>
       <c r="M80" t="n">
-        <v>0.2250371366478253</v>
+        <v>0.2250371366478245</v>
       </c>
       <c r="N80" t="n">
         <v>0.2513760312601657</v>
       </c>
       <c r="O80" t="n">
-        <v>0.3863489999530916</v>
+        <v>0.3863489999532777</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>5.557509309192358</v>
+        <v>5.557509309242717</v>
       </c>
       <c r="B81" t="n">
         <v>0</v>
@@ -4238,28 +4238,28 @@
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>0.07001701422114191</v>
+        <v>0.07001701422114186</v>
       </c>
       <c r="H81" t="n">
-        <v>0.05137435493600268</v>
+        <v>0.05137435493610881</v>
       </c>
       <c r="I81" t="n">
-        <v>0.06024037485416417</v>
+        <v>0.06024037485416535</v>
       </c>
       <c r="J81" t="n">
-        <v>6.985424616815113</v>
+        <v>6.985424616815118</v>
       </c>
       <c r="K81" t="n">
-        <v>24.26888371735969</v>
+        <v>24.26888371725562</v>
       </c>
       <c r="L81" t="n">
-        <v>12.8614880195031</v>
+        <v>12.86148801950013</v>
       </c>
       <c r="M81" t="n">
         <v>0.2261786568671618</v>
       </c>
       <c r="N81" t="n">
-        <v>0.2504409517469849</v>
+        <v>0.2504409517469758</v>
       </c>
       <c r="O81" t="n">
         <v>0.3855295790644589</v>
@@ -4267,7 +4267,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>6.884734885084504</v>
+        <v>6.88473488508424</v>
       </c>
       <c r="B82" t="n">
         <v>0</v>
@@ -4285,22 +4285,22 @@
         <v>0</v>
       </c>
       <c r="G82" t="n">
-        <v>0.07963111756833033</v>
+        <v>0.07963111756833034</v>
       </c>
       <c r="H82" t="n">
-        <v>0.04252156914041653</v>
+        <v>0.04252156886748124</v>
       </c>
       <c r="I82" t="n">
-        <v>0.05017595975381715</v>
+        <v>0.05017595975382149</v>
       </c>
       <c r="J82" t="n">
-        <v>6.1385856632189</v>
+        <v>6.138585663218898</v>
       </c>
       <c r="K82" t="n">
-        <v>29.77475551392198</v>
+        <v>29.77475580630981</v>
       </c>
       <c r="L82" t="n">
-        <v>15.50030379108488</v>
+        <v>15.50030379108178</v>
       </c>
       <c r="M82" t="n">
         <v>0.2265943447717173</v>
@@ -4335,19 +4335,19 @@
         <v>0.08879812259790099</v>
       </c>
       <c r="H83" t="n">
-        <v>0.03367093419833526</v>
+        <v>0.03367093419817131</v>
       </c>
       <c r="I83" t="n">
-        <v>0.03983894170489027</v>
+        <v>0.0398389417205567</v>
       </c>
       <c r="J83" t="n">
         <v>5.502803974491979</v>
       </c>
       <c r="K83" t="n">
-        <v>38.8382583369122</v>
+        <v>38.83825833633745</v>
       </c>
       <c r="L83" t="n">
-        <v>19.66896231418335</v>
+        <v>19.66896230630415</v>
       </c>
       <c r="M83" t="n">
         <v>0.2268739265381451</v>
@@ -4379,22 +4379,22 @@
         <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>0.09730058997241227</v>
+        <v>0.09730058997241231</v>
       </c>
       <c r="H84" t="n">
-        <v>0.02610340788215523</v>
+        <v>0.02610340878171103</v>
       </c>
       <c r="I84" t="n">
-        <v>0.02989360846260111</v>
+        <v>0.02989360919739158</v>
       </c>
       <c r="J84" t="n">
-        <v>5.020655423512832</v>
+        <v>5.020655423512829</v>
       </c>
       <c r="K84" t="n">
-        <v>53.99157705487541</v>
+        <v>53.99157919112164</v>
       </c>
       <c r="L84" t="n">
-        <v>26.65159272456656</v>
+        <v>26.65159204591503</v>
       </c>
       <c r="M84" t="n">
         <v>0.2270352522940929</v>
@@ -4408,7 +4408,7 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>-1.889640618916508</v>
+        <v>-1.889640618959856</v>
       </c>
       <c r="B85" t="n">
         <v>90</v>
@@ -4426,25 +4426,25 @@
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>0.06081899508305515</v>
+        <v>0.06081899508310853</v>
       </c>
       <c r="H85" t="n">
-        <v>0.05879831855407186</v>
+        <v>0.05879831855407187</v>
       </c>
       <c r="I85" t="n">
-        <v>0.05499992440104682</v>
+        <v>0.05499992440104681</v>
       </c>
       <c r="J85" t="n">
-        <v>8.048406845244122</v>
+        <v>8.048406845212961</v>
       </c>
       <c r="K85" t="n">
         <v>21.0463717756711</v>
       </c>
       <c r="L85" t="n">
-        <v>14.11116142850681</v>
+        <v>14.11116142850756</v>
       </c>
       <c r="M85" t="n">
-        <v>0.2250371366478461</v>
+        <v>0.2250371366478267</v>
       </c>
       <c r="N85" t="n">
         <v>0.2513760312601657</v>
@@ -4455,7 +4455,7 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>5.557509309210114</v>
+        <v>5.557509309268</v>
       </c>
       <c r="B86" t="n">
         <v>90</v>
@@ -4476,25 +4476,25 @@
         <v>0.07001701422114176</v>
       </c>
       <c r="H86" t="n">
-        <v>0.05137435493601845</v>
+        <v>0.051374354936113</v>
       </c>
       <c r="I86" t="n">
-        <v>0.0461803732550134</v>
+        <v>0.04618037325445165</v>
       </c>
       <c r="J86" t="n">
-        <v>6.985424616815127</v>
+        <v>6.985424616815128</v>
       </c>
       <c r="K86" t="n">
-        <v>24.26888371734877</v>
+        <v>24.26888371725406</v>
       </c>
       <c r="L86" t="n">
-        <v>16.87985375514392</v>
+        <v>16.87985375527884</v>
       </c>
       <c r="M86" t="n">
         <v>0.2261786568671618</v>
       </c>
       <c r="N86" t="n">
-        <v>0.2504409517469818</v>
+        <v>0.2504409517469713</v>
       </c>
       <c r="O86" t="n">
         <v>0.3855295790644589</v>
@@ -4502,7 +4502,7 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>6.88473488508447</v>
+        <v>6.884734885084336</v>
       </c>
       <c r="B87" t="n">
         <v>90</v>
@@ -4520,22 +4520,22 @@
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>0.07963111756833031</v>
+        <v>0.0796311175683303</v>
       </c>
       <c r="H87" t="n">
-        <v>0.0425215688814233</v>
+        <v>0.04252156906482724</v>
       </c>
       <c r="I87" t="n">
-        <v>0.0365729638148084</v>
+        <v>0.0365729635165785</v>
       </c>
       <c r="J87" t="n">
-        <v>6.1385856632189</v>
+        <v>6.138585663218902</v>
       </c>
       <c r="K87" t="n">
-        <v>29.77475579429602</v>
+        <v>29.77475559471587</v>
       </c>
       <c r="L87" t="n">
-        <v>21.50869236001778</v>
+        <v>21.50869252297392</v>
       </c>
       <c r="M87" t="n">
         <v>0.2265943447717173</v>
@@ -4567,22 +4567,22 @@
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>0.0887981225979009</v>
+        <v>0.08879812259790089</v>
       </c>
       <c r="H88" t="n">
-        <v>0.03367093419843081</v>
+        <v>0.03367093419825047</v>
       </c>
       <c r="I88" t="n">
-        <v>0.02685826388012641</v>
+        <v>0.02685826388011716</v>
       </c>
       <c r="J88" t="n">
-        <v>5.502803974491982</v>
+        <v>5.502803974491984</v>
       </c>
       <c r="K88" t="n">
-        <v>38.83825833722134</v>
+        <v>38.83825833661104</v>
       </c>
       <c r="L88" t="n">
-        <v>29.95091013276723</v>
+        <v>29.95091013268642</v>
       </c>
       <c r="M88" t="n">
         <v>0.2268739265381451</v>
@@ -4614,22 +4614,22 @@
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>0.09730058997241216</v>
+        <v>0.09730058997241213</v>
       </c>
       <c r="H89" t="n">
-        <v>0.02610341344145187</v>
+        <v>0.02610341256874947</v>
       </c>
       <c r="I89" t="n">
-        <v>0.0182705081859316</v>
+        <v>0.01827050651353862</v>
       </c>
       <c r="J89" t="n">
         <v>5.020655423512838</v>
       </c>
       <c r="K89" t="n">
-        <v>53.99159103978931</v>
+        <v>53.99158897288589</v>
       </c>
       <c r="L89" t="n">
-        <v>47.21653013893688</v>
+        <v>47.21651844304695</v>
       </c>
       <c r="M89" t="n">
         <v>0.2270352522940929</v>
@@ -4643,7 +4643,7 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>-2.302910531717379</v>
+        <v>-2.302910531697544</v>
       </c>
       <c r="B90" t="n">
         <v>0</v>
@@ -4661,36 +4661,36 @@
         <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>0.0602462207279462</v>
+        <v>0.06024622072802757</v>
       </c>
       <c r="H90" t="n">
-        <v>0.05879831855407184</v>
+        <v>0.05879831855407185</v>
       </c>
       <c r="I90" t="n">
-        <v>0.06870583418309244</v>
+        <v>0.06870583418304031</v>
       </c>
       <c r="J90" t="n">
-        <v>8.125439495733662</v>
+        <v>8.125439495721256</v>
       </c>
       <c r="K90" t="n">
-        <v>21.04637177567112</v>
+        <v>21.04637177567111</v>
       </c>
       <c r="L90" t="n">
-        <v>11.254553257684</v>
+        <v>11.25455325771254</v>
       </c>
       <c r="M90" t="n">
-        <v>0.2256156638693907</v>
+        <v>0.225615663869395</v>
       </c>
       <c r="N90" t="n">
         <v>0.2513760312601657</v>
       </c>
       <c r="O90" t="n">
-        <v>0.3863489999530916</v>
+        <v>0.3863489999530875</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>8.32171814698858</v>
+        <v>8.321718146444381</v>
       </c>
       <c r="B91" t="n">
         <v>0</v>
@@ -4711,25 +4711,25 @@
         <v>0.0690528576385022</v>
       </c>
       <c r="H91" t="n">
-        <v>0.0513743549360354</v>
+        <v>0.05137435493591196</v>
       </c>
       <c r="I91" t="n">
-        <v>0.06024037485416537</v>
+        <v>0.06024037485416493</v>
       </c>
       <c r="J91" t="n">
-        <v>7.083455691513422</v>
+        <v>7.083455691513421</v>
       </c>
       <c r="K91" t="n">
-        <v>24.26888371732304</v>
+        <v>24.26888371726444</v>
       </c>
       <c r="L91" t="n">
-        <v>12.86148801950076</v>
+        <v>12.86148801950186</v>
       </c>
       <c r="M91" t="n">
         <v>0.2271501256168141</v>
       </c>
       <c r="N91" t="n">
-        <v>0.2504409517469838</v>
+        <v>0.2504409517470825</v>
       </c>
       <c r="O91" t="n">
         <v>0.3855295790644589</v>
@@ -4758,22 +4758,22 @@
         <v>0.07851249777817861</v>
       </c>
       <c r="H92" t="n">
-        <v>0.04252156913946801</v>
+        <v>0.04252156914041652</v>
       </c>
       <c r="I92" t="n">
-        <v>0.05017595975382162</v>
+        <v>0.05017595975382196</v>
       </c>
       <c r="J92" t="n">
         <v>6.22638963432703</v>
       </c>
       <c r="K92" t="n">
-        <v>29.77475551491919</v>
+        <v>29.77475551392185</v>
       </c>
       <c r="L92" t="n">
-        <v>15.50030379108166</v>
+        <v>15.50030379108013</v>
       </c>
       <c r="M92" t="n">
-        <v>0.2277195082661254</v>
+        <v>0.2277195082661255</v>
       </c>
       <c r="N92" t="n">
         <v>0.2503438825093889</v>
@@ -4784,7 +4784,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>10.52073405921142</v>
+        <v>10.52073405921157</v>
       </c>
       <c r="B93" t="n">
         <v>0</v>
@@ -4802,25 +4802,25 @@
         <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>0.08760811224332596</v>
+        <v>0.08760811224332589</v>
       </c>
       <c r="H93" t="n">
-        <v>0.03367093419841335</v>
+        <v>0.03367093419838799</v>
       </c>
       <c r="I93" t="n">
-        <v>0.03983894172651406</v>
+        <v>0.03983894172827522</v>
       </c>
       <c r="J93" t="n">
-        <v>5.577785826878742</v>
+        <v>5.577785826878745</v>
       </c>
       <c r="K93" t="n">
-        <v>38.83825833716671</v>
+        <v>38.83825833708483</v>
       </c>
       <c r="L93" t="n">
-        <v>19.66896230378643</v>
+        <v>19.66896230287334</v>
       </c>
       <c r="M93" t="n">
-        <v>0.228069521806337</v>
+        <v>0.2280695218063371</v>
       </c>
       <c r="N93" t="n">
         <v>0.2503438825093872</v>
@@ -4831,7 +4831,7 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>10.16413022328432</v>
+        <v>10.16413022329318</v>
       </c>
       <c r="B94" t="n">
         <v>0</v>
@@ -4849,25 +4849,25 @@
         <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>0.09604499427408333</v>
+        <v>0.09604499427408038</v>
       </c>
       <c r="H94" t="n">
-        <v>0.0261034134414308</v>
+        <v>0.02610340956698381</v>
       </c>
       <c r="I94" t="n">
-        <v>0.02989360903028021</v>
+        <v>0.02989360912267975</v>
       </c>
       <c r="J94" t="n">
-        <v>5.08646226964758</v>
+        <v>5.086462269647719</v>
       </c>
       <c r="K94" t="n">
-        <v>53.99159103986335</v>
+        <v>53.99158148944287</v>
       </c>
       <c r="L94" t="n">
-        <v>26.6515921635807</v>
+        <v>26.65159209903368</v>
       </c>
       <c r="M94" t="n">
-        <v>0.2282957475933322</v>
+        <v>0.2282957475933352</v>
       </c>
       <c r="N94" t="n">
         <v>0.2503438825093872</v>
@@ -4878,7 +4878,7 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>-0.5371438993407593</v>
+        <v>-0.5371438994406617</v>
       </c>
       <c r="B95" t="n">
         <v>90</v>
@@ -4896,25 +4896,25 @@
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>0.06024622072805539</v>
+        <v>0.06024622072785668</v>
       </c>
       <c r="H95" t="n">
         <v>0.05879831855407185</v>
       </c>
       <c r="I95" t="n">
-        <v>0.05499992440104685</v>
+        <v>0.05499992440104614</v>
       </c>
       <c r="J95" t="n">
-        <v>8.125439495702128</v>
+        <v>8.125439495742517</v>
       </c>
       <c r="K95" t="n">
         <v>21.04637177567111</v>
       </c>
       <c r="L95" t="n">
-        <v>14.11116142850724</v>
+        <v>14.1111614285085</v>
       </c>
       <c r="M95" t="n">
-        <v>0.2256156638694349</v>
+        <v>0.2256156638693941</v>
       </c>
       <c r="N95" t="n">
         <v>0.2513760312601657</v>
@@ -4925,7 +4925,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>8.321718147919455</v>
+        <v>8.321718148004894</v>
       </c>
       <c r="B96" t="n">
         <v>90</v>
@@ -4943,28 +4943,28 @@
         <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>0.06905285763850212</v>
+        <v>0.06905285763850204</v>
       </c>
       <c r="H96" t="n">
-        <v>0.05137435493463165</v>
+        <v>0.05137435493487521</v>
       </c>
       <c r="I96" t="n">
-        <v>0.04618037325657236</v>
+        <v>0.04618037325597581</v>
       </c>
       <c r="J96" t="n">
-        <v>7.083455691513431</v>
+        <v>7.083455691513438</v>
       </c>
       <c r="K96" t="n">
-        <v>24.2688837191622</v>
+        <v>24.26888371896354</v>
       </c>
       <c r="L96" t="n">
-        <v>16.87985375460765</v>
+        <v>16.87985375481558</v>
       </c>
       <c r="M96" t="n">
         <v>0.2271501256168141</v>
       </c>
       <c r="N96" t="n">
-        <v>0.2504409517468151</v>
+        <v>0.2504409517467996</v>
       </c>
       <c r="O96" t="n">
         <v>0.3855295790644589</v>
@@ -4993,22 +4993,22 @@
         <v>0.07851249777817856</v>
       </c>
       <c r="H97" t="n">
-        <v>0.04252156913333017</v>
+        <v>0.04252156912668873</v>
       </c>
       <c r="I97" t="n">
-        <v>0.03657296374619579</v>
+        <v>0.03657296374928674</v>
       </c>
       <c r="J97" t="n">
         <v>6.226389634327034</v>
       </c>
       <c r="K97" t="n">
-        <v>29.77475552142408</v>
+        <v>29.77475552908017</v>
       </c>
       <c r="L97" t="n">
-        <v>21.50869239642571</v>
+        <v>21.50869239514417</v>
       </c>
       <c r="M97" t="n">
-        <v>0.2277195082661255</v>
+        <v>0.2277195082661254</v>
       </c>
       <c r="N97" t="n">
         <v>0.2503438825093889</v>
@@ -5019,7 +5019,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>10.52073405921817</v>
+        <v>10.52073405921832</v>
       </c>
       <c r="B98" t="n">
         <v>90</v>
@@ -5037,25 +5037,25 @@
         <v>0</v>
       </c>
       <c r="G98" t="n">
-        <v>0.08760811224332582</v>
+        <v>0.08760811224332579</v>
       </c>
       <c r="H98" t="n">
-        <v>0.03367093419817904</v>
+        <v>0.03367093419841399</v>
       </c>
       <c r="I98" t="n">
-        <v>0.0268582638801258</v>
+        <v>0.02685826388012199</v>
       </c>
       <c r="J98" t="n">
-        <v>5.577785826878749</v>
+        <v>5.577785826878752</v>
       </c>
       <c r="K98" t="n">
-        <v>38.83825833636766</v>
+        <v>38.83825833716894</v>
       </c>
       <c r="L98" t="n">
-        <v>29.95091013276209</v>
+        <v>29.95091013272918</v>
       </c>
       <c r="M98" t="n">
-        <v>0.228069521806337</v>
+        <v>0.2280695218063371</v>
       </c>
       <c r="N98" t="n">
         <v>0.2503438825093872</v>
@@ -5066,7 +5066,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>10.16413022329101</v>
+        <v>10.16413022329117</v>
       </c>
       <c r="B99" t="n">
         <v>90</v>
@@ -5084,22 +5084,22 @@
         <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>0.09604499427408314</v>
+        <v>0.09604499427408315</v>
       </c>
       <c r="H99" t="n">
-        <v>0.02610341063302</v>
+        <v>0.026103411728027</v>
       </c>
       <c r="I99" t="n">
-        <v>0.01827050818592534</v>
+        <v>0.0182705041476185</v>
       </c>
       <c r="J99" t="n">
-        <v>5.08646226964759</v>
+        <v>5.086462269647589</v>
       </c>
       <c r="K99" t="n">
-        <v>53.99158420606746</v>
+        <v>53.99158687099488</v>
       </c>
       <c r="L99" t="n">
-        <v>47.21653013895178</v>
+        <v>47.21650025449031</v>
       </c>
       <c r="M99" t="n">
         <v>0.2282957475933323</v>
@@ -5113,7 +5113,7 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>-1.095359069909058</v>
+        <v>-1.095359070140522</v>
       </c>
       <c r="B100" t="n">
         <v>0</v>
@@ -5131,36 +5131,36 @@
         <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>0.05977546064619065</v>
+        <v>0.05977546064619062</v>
       </c>
       <c r="H100" t="n">
-        <v>0.05879831855407149</v>
+        <v>0.05879831855407183</v>
       </c>
       <c r="I100" t="n">
-        <v>0.0687058341830747</v>
+        <v>0.06870583418298744</v>
       </c>
       <c r="J100" t="n">
-        <v>8.189868841214482</v>
+        <v>8.189868841214487</v>
       </c>
       <c r="K100" t="n">
-        <v>21.04637177567121</v>
+        <v>21.04637177567112</v>
       </c>
       <c r="L100" t="n">
-        <v>11.25455325771015</v>
+        <v>11.25455325771519</v>
       </c>
       <c r="M100" t="n">
         <v>0.226091236013598</v>
       </c>
       <c r="N100" t="n">
-        <v>0.2513760312601661</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O100" t="n">
-        <v>0.386348999953092</v>
+        <v>0.3863489999531965</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>10.93107156703519</v>
+        <v>10.93107156722848</v>
       </c>
       <c r="B101" t="n">
         <v>0</v>
@@ -5178,28 +5178,28 @@
         <v>0</v>
       </c>
       <c r="G101" t="n">
-        <v>0.06826064423184733</v>
+        <v>0.06826064423178985</v>
       </c>
       <c r="H101" t="n">
-        <v>0.05137435493610944</v>
+        <v>0.05137435493610856</v>
       </c>
       <c r="I101" t="n">
-        <v>0.06024037485415547</v>
+        <v>0.06024037485416537</v>
       </c>
       <c r="J101" t="n">
-        <v>7.166093084687619</v>
+        <v>7.166093084689718</v>
       </c>
       <c r="K101" t="n">
-        <v>24.26888371725545</v>
+        <v>24.2688837172557</v>
       </c>
       <c r="L101" t="n">
-        <v>12.86148801951243</v>
+        <v>12.86148801950019</v>
       </c>
       <c r="M101" t="n">
-        <v>0.2279485035722895</v>
+        <v>0.2279485035723465</v>
       </c>
       <c r="N101" t="n">
-        <v>0.2504409517469752</v>
+        <v>0.2504409517469761</v>
       </c>
       <c r="O101" t="n">
         <v>0.3855295790644589</v>
@@ -5225,22 +5225,22 @@
         <v>0</v>
       </c>
       <c r="G102" t="n">
-        <v>0.07758019783380793</v>
+        <v>0.07758019783380787</v>
       </c>
       <c r="H102" t="n">
-        <v>0.04252156912676363</v>
+        <v>0.0425215691404031</v>
       </c>
       <c r="I102" t="n">
-        <v>0.05017595975382202</v>
+        <v>0.05017595975381703</v>
       </c>
       <c r="J102" t="n">
-        <v>6.301514994819788</v>
+        <v>6.301514994819794</v>
       </c>
       <c r="K102" t="n">
-        <v>29.77475552901311</v>
+        <v>29.77475551393905</v>
       </c>
       <c r="L102" t="n">
-        <v>15.50030379108043</v>
+        <v>15.50030379108493</v>
       </c>
       <c r="M102" t="n">
         <v>0.2286574074576231</v>
@@ -5272,25 +5272,25 @@
         <v>0</v>
       </c>
       <c r="G103" t="n">
-        <v>0.0866234930773169</v>
+        <v>0.08662349307731691</v>
       </c>
       <c r="H103" t="n">
-        <v>0.03367093278687357</v>
+        <v>0.03367093354070443</v>
       </c>
       <c r="I103" t="n">
-        <v>0.03983894169931793</v>
+        <v>0.03983894172538575</v>
       </c>
       <c r="J103" t="n">
         <v>5.641391091044854</v>
       </c>
       <c r="K103" t="n">
-        <v>38.83826119984874</v>
+        <v>38.83825966879478</v>
       </c>
       <c r="L103" t="n">
-        <v>19.66896231613955</v>
+        <v>19.66896230419079</v>
       </c>
       <c r="M103" t="n">
-        <v>0.2290588787963555</v>
+        <v>0.2290588787963556</v>
       </c>
       <c r="N103" t="n">
         <v>0.2503438825093889</v>
@@ -5301,7 +5301,7 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>13.4879342283176</v>
+        <v>13.48793422831777</v>
       </c>
       <c r="B104" t="n">
         <v>0</v>
@@ -5319,25 +5319,25 @@
         <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>0.09500775693448216</v>
+        <v>0.09500775693448206</v>
       </c>
       <c r="H104" t="n">
-        <v>0.02610341104860563</v>
+        <v>0.02610341344140705</v>
       </c>
       <c r="I104" t="n">
-        <v>0.02989360894852296</v>
+        <v>0.02989360654252865</v>
       </c>
       <c r="J104" t="n">
-        <v>5.142141953979939</v>
+        <v>5.142141953979944</v>
       </c>
       <c r="K104" t="n">
-        <v>53.9915851357802</v>
+        <v>53.99159103994368</v>
       </c>
       <c r="L104" t="n">
-        <v>26.65159221969706</v>
+        <v>26.65159426308986</v>
       </c>
       <c r="M104" t="n">
-        <v>0.2293371307184592</v>
+        <v>0.2293371307184593</v>
       </c>
       <c r="N104" t="n">
         <v>0.2503438825093872</v>
@@ -5348,7 +5348,7 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>0.6704075623623933</v>
+        <v>0.6704075623620842</v>
       </c>
       <c r="B105" t="n">
         <v>90</v>
@@ -5366,28 +5366,28 @@
         <v>0</v>
       </c>
       <c r="G105" t="n">
-        <v>0.05977546064619064</v>
+        <v>0.05977546064619066</v>
       </c>
       <c r="H105" t="n">
-        <v>0.05879831855407186</v>
+        <v>0.05879831855407178</v>
       </c>
       <c r="I105" t="n">
-        <v>0.05499992440104682</v>
+        <v>0.05499992440104676</v>
       </c>
       <c r="J105" t="n">
-        <v>8.189868841214484</v>
+        <v>8.189868841214482</v>
       </c>
       <c r="K105" t="n">
-        <v>21.0463717756711</v>
+        <v>21.04637177567113</v>
       </c>
       <c r="L105" t="n">
-        <v>14.11116142850687</v>
+        <v>14.11116142850776</v>
       </c>
       <c r="M105" t="n">
         <v>0.226091236013598</v>
       </c>
       <c r="N105" t="n">
-        <v>0.2513760312601657</v>
+        <v>0.2513760312601658</v>
       </c>
       <c r="O105" t="n">
         <v>0.3855295790644589</v>
@@ -5395,7 +5395,7 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>10.9310715672701</v>
+        <v>10.93107156795904</v>
       </c>
       <c r="B106" t="n">
         <v>90</v>
@@ -5413,28 +5413,28 @@
         <v>0</v>
       </c>
       <c r="G106" t="n">
-        <v>0.06826064423177142</v>
+        <v>0.06826064423158582</v>
       </c>
       <c r="H106" t="n">
-        <v>0.05137435493597955</v>
+        <v>0.05137435493610411</v>
       </c>
       <c r="I106" t="n">
-        <v>0.04618037325594582</v>
+        <v>0.04618037325519099</v>
       </c>
       <c r="J106" t="n">
-        <v>7.166093084690407</v>
+        <v>7.166093084702979</v>
       </c>
       <c r="K106" t="n">
-        <v>24.26888371739829</v>
+        <v>24.26888371726275</v>
       </c>
       <c r="L106" t="n">
-        <v>16.87985375482317</v>
+        <v>16.87985375509835</v>
       </c>
       <c r="M106" t="n">
-        <v>0.2279485035723647</v>
+        <v>0.2279485035725509</v>
       </c>
       <c r="N106" t="n">
-        <v>0.2504409517469801</v>
+        <v>0.2504409517469726</v>
       </c>
       <c r="O106" t="n">
         <v>0.3855295790644589</v>
@@ -5460,22 +5460,22 @@
         <v>0</v>
       </c>
       <c r="G107" t="n">
-        <v>0.07758019783380785</v>
+        <v>0.0775801978338078</v>
       </c>
       <c r="H107" t="n">
-        <v>0.04252156914036431</v>
+        <v>0.04252156914041613</v>
       </c>
       <c r="I107" t="n">
-        <v>0.0365729638604208</v>
+        <v>0.03657296385982881</v>
       </c>
       <c r="J107" t="n">
-        <v>6.301514994819797</v>
+        <v>6.301514994819799</v>
       </c>
       <c r="K107" t="n">
-        <v>29.77475551398377</v>
+        <v>29.77475551392337</v>
       </c>
       <c r="L107" t="n">
-        <v>21.50869233369364</v>
+        <v>21.5086923339699</v>
       </c>
       <c r="M107" t="n">
         <v>0.2286574074576231</v>
@@ -5489,7 +5489,7 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>13.87773016768094</v>
+        <v>13.87773016768076</v>
       </c>
       <c r="B108" t="n">
         <v>90</v>
@@ -5510,19 +5510,19 @@
         <v>0.08662349307731684</v>
       </c>
       <c r="H108" t="n">
-        <v>0.03367093145879866</v>
+        <v>0.03367093334642412</v>
       </c>
       <c r="I108" t="n">
-        <v>0.02685826388011892</v>
+        <v>0.02685826388012449</v>
       </c>
       <c r="J108" t="n">
-        <v>5.641391091044858</v>
+        <v>5.641391091044859</v>
       </c>
       <c r="K108" t="n">
-        <v>38.83826369629649</v>
+        <v>38.83826006421094</v>
       </c>
       <c r="L108" t="n">
-        <v>29.95091013270455</v>
+        <v>29.95091013275078</v>
       </c>
       <c r="M108" t="n">
         <v>0.2290588787963555</v>
@@ -5536,7 +5536,7 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>13.4879342283245</v>
+        <v>13.48793422832416</v>
       </c>
       <c r="B109" t="n">
         <v>90</v>
@@ -5554,25 +5554,25 @@
         <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>0.09500775693448196</v>
+        <v>0.09500775693448202</v>
       </c>
       <c r="H109" t="n">
-        <v>0.02610341217494922</v>
+        <v>0.02610341344141874</v>
       </c>
       <c r="I109" t="n">
-        <v>0.01827050818593219</v>
+        <v>0.01827050416686093</v>
       </c>
       <c r="J109" t="n">
-        <v>5.142141953979949</v>
+        <v>5.142141953979946</v>
       </c>
       <c r="K109" t="n">
-        <v>53.99158798381738</v>
+        <v>53.99159103990169</v>
       </c>
       <c r="L109" t="n">
-        <v>47.2165301389355</v>
+        <v>47.2165004361297</v>
       </c>
       <c r="M109" t="n">
-        <v>0.2293371307184593</v>
+        <v>0.2293371307184592</v>
       </c>
       <c r="N109" t="n">
         <v>0.2503438825093872</v>
@@ -5583,7 +5583,7 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>0.0003023184003916324</v>
+        <v>0.0003023182175330152</v>
       </c>
       <c r="B110" t="n">
         <v>0</v>
@@ -5601,36 +5601,36 @@
         <v>0</v>
       </c>
       <c r="G110" t="n">
-        <v>0.05937680525739395</v>
+        <v>0.05937680525739398</v>
       </c>
       <c r="H110" t="n">
-        <v>0.05879831855402685</v>
+        <v>0.05879831855407184</v>
       </c>
       <c r="I110" t="n">
-        <v>0.06870583418307451</v>
+        <v>0.068705834182909</v>
       </c>
       <c r="J110" t="n">
-        <v>8.245236993488438</v>
+        <v>8.245236993488435</v>
       </c>
       <c r="K110" t="n">
-        <v>21.04637177568418</v>
+        <v>21.04637177567111</v>
       </c>
       <c r="L110" t="n">
-        <v>11.25455325770891</v>
+        <v>11.25455325771676</v>
       </c>
       <c r="M110" t="n">
         <v>0.226494027016834</v>
       </c>
       <c r="N110" t="n">
-        <v>0.2513760312602135</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O110" t="n">
-        <v>0.3863489999530796</v>
+        <v>0.3863489999532786</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>13.40366856570424</v>
+        <v>13.4036685634126</v>
       </c>
       <c r="B111" t="n">
         <v>0</v>
@@ -5648,28 +5648,28 @@
         <v>0</v>
       </c>
       <c r="G111" t="n">
-        <v>0.06759185910388883</v>
+        <v>0.06759185910389409</v>
       </c>
       <c r="H111" t="n">
-        <v>0.05137435493611309</v>
+        <v>0.05137435493535634</v>
       </c>
       <c r="I111" t="n">
-        <v>0.06024037485416309</v>
+        <v>0.06024037485416538</v>
       </c>
       <c r="J111" t="n">
-        <v>7.2373753669325</v>
+        <v>7.237375366931776</v>
       </c>
       <c r="K111" t="n">
-        <v>24.26888371725402</v>
+        <v>24.2688837173054</v>
       </c>
       <c r="L111" t="n">
-        <v>12.86148801950443</v>
+        <v>12.86148801950016</v>
       </c>
       <c r="M111" t="n">
-        <v>0.2286226066323986</v>
+        <v>0.2286226066323933</v>
       </c>
       <c r="N111" t="n">
-        <v>0.2504409517469713</v>
+        <v>0.250440951747383</v>
       </c>
       <c r="O111" t="n">
         <v>0.3855295790644589</v>
@@ -5695,22 +5695,22 @@
         <v>0</v>
       </c>
       <c r="G112" t="n">
-        <v>0.07678132778057042</v>
+        <v>0.07678132778057041</v>
       </c>
       <c r="H112" t="n">
-        <v>0.04252156913892318</v>
+        <v>0.04252156914041652</v>
       </c>
       <c r="I112" t="n">
-        <v>0.05017595975376031</v>
+        <v>0.05017595975380051</v>
       </c>
       <c r="J112" t="n">
-        <v>6.367348835526475</v>
+        <v>6.367348835526477</v>
       </c>
       <c r="K112" t="n">
-        <v>29.77475551552105</v>
+        <v>29.77475551392184</v>
       </c>
       <c r="L112" t="n">
-        <v>15.50030379110678</v>
+        <v>15.50030379109202</v>
       </c>
       <c r="M112" t="n">
         <v>0.2294611845740662</v>
@@ -5724,7 +5724,7 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>17.1844556067535</v>
+        <v>17.18445560674286</v>
       </c>
       <c r="B113" t="n">
         <v>0</v>
@@ -5742,28 +5742,28 @@
         <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>0.08578345209091989</v>
+        <v>0.08578345209091993</v>
       </c>
       <c r="H113" t="n">
-        <v>0.03367093419842854</v>
+        <v>0.03367093100260194</v>
       </c>
       <c r="I113" t="n">
-        <v>0.03983894172076215</v>
+        <v>0.03983894172831658</v>
       </c>
       <c r="J113" t="n">
-        <v>5.696816715522584</v>
+        <v>5.69681671552258</v>
       </c>
       <c r="K113" t="n">
-        <v>38.83825833721429</v>
+        <v>38.83826468293864</v>
       </c>
       <c r="L113" t="n">
-        <v>19.66896230623579</v>
+        <v>19.66896230285926</v>
       </c>
       <c r="M113" t="n">
         <v>0.2299030485335895</v>
       </c>
       <c r="N113" t="n">
-        <v>0.2503438825093872</v>
+        <v>0.2503438825093889</v>
       </c>
       <c r="O113" t="n">
         <v>0.3855295790644589</v>
@@ -5789,22 +5789,22 @@
         <v>0</v>
       </c>
       <c r="G114" t="n">
-        <v>0.09412528562904438</v>
+        <v>0.09412528562904443</v>
       </c>
       <c r="H114" t="n">
-        <v>0.02610341183404055</v>
+        <v>0.02610341135382665</v>
       </c>
       <c r="I114" t="n">
-        <v>0.02989360220637799</v>
+        <v>0.02989360198628908</v>
       </c>
       <c r="J114" t="n">
-        <v>5.190483785710256</v>
+        <v>5.190483785710254</v>
       </c>
       <c r="K114" t="n">
-        <v>53.99158716856608</v>
+        <v>53.99158600148492</v>
       </c>
       <c r="L114" t="n">
-        <v>26.65159794495982</v>
+        <v>26.65159807978327</v>
       </c>
       <c r="M114" t="n">
         <v>0.2302232015958814</v>
@@ -5818,7 +5818,7 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>1.766068951178435</v>
+        <v>1.766068950903967</v>
       </c>
       <c r="B115" t="n">
         <v>90</v>
@@ -5836,28 +5836,28 @@
         <v>0</v>
       </c>
       <c r="G115" t="n">
-        <v>0.05937680525739398</v>
+        <v>0.05937680525739396</v>
       </c>
       <c r="H115" t="n">
-        <v>0.05879831855405647</v>
+        <v>0.05879831855407183</v>
       </c>
       <c r="I115" t="n">
-        <v>0.05499992440104618</v>
+        <v>0.05499992440104687</v>
       </c>
       <c r="J115" t="n">
-        <v>8.245236993488435</v>
+        <v>8.245236993488438</v>
       </c>
       <c r="K115" t="n">
-        <v>21.0463717757597</v>
+        <v>21.04637177567112</v>
       </c>
       <c r="L115" t="n">
-        <v>14.11116142850849</v>
+        <v>14.11116142850731</v>
       </c>
       <c r="M115" t="n">
         <v>0.226494027016834</v>
       </c>
       <c r="N115" t="n">
-        <v>0.2513760312601157</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O115" t="n">
         <v>0.3855295790644589</v>
@@ -5865,7 +5865,7 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>13.40366856562338</v>
+        <v>13.40366856570353</v>
       </c>
       <c r="B116" t="n">
         <v>90</v>
@@ -5883,28 +5883,28 @@
         <v>0</v>
       </c>
       <c r="G116" t="n">
-        <v>0.0675918591038938</v>
+        <v>0.06759185910388921</v>
       </c>
       <c r="H116" t="n">
-        <v>0.05137435493601571</v>
+        <v>0.05137435493611237</v>
       </c>
       <c r="I116" t="n">
-        <v>0.04618037325665596</v>
+        <v>0.04618037325662799</v>
       </c>
       <c r="J116" t="n">
-        <v>7.237375366931804</v>
+        <v>7.237375366932447</v>
       </c>
       <c r="K116" t="n">
-        <v>24.2688837173507</v>
+        <v>24.26888371725536</v>
       </c>
       <c r="L116" t="n">
-        <v>16.87985375457297</v>
+        <v>16.87985375458553</v>
       </c>
       <c r="M116" t="n">
-        <v>0.2286226066323934</v>
+        <v>0.228622606632398</v>
       </c>
       <c r="N116" t="n">
-        <v>0.2504409517469823</v>
+        <v>0.2504409517469711</v>
       </c>
       <c r="O116" t="n">
         <v>0.3855295790644589</v>
@@ -5912,7 +5912,7 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>16.59013954854465</v>
+        <v>16.59013954854444</v>
       </c>
       <c r="B117" t="n">
         <v>90</v>
@@ -5930,22 +5930,22 @@
         <v>0</v>
       </c>
       <c r="G117" t="n">
-        <v>0.07678132778057038</v>
+        <v>0.07678132778057041</v>
       </c>
       <c r="H117" t="n">
-        <v>0.04252156913385362</v>
+        <v>0.04252156914041651</v>
       </c>
       <c r="I117" t="n">
-        <v>0.0365729636745083</v>
+        <v>0.0365729638667493</v>
       </c>
       <c r="J117" t="n">
-        <v>6.36734883552648</v>
+        <v>6.367348835526476</v>
       </c>
       <c r="K117" t="n">
-        <v>29.77475552097209</v>
+        <v>29.7747555139219</v>
       </c>
       <c r="L117" t="n">
-        <v>21.50869243851605</v>
+        <v>21.5086923297105</v>
       </c>
       <c r="M117" t="n">
         <v>0.2294611845740662</v>
@@ -5959,7 +5959,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>17.18445560674962</v>
+        <v>17.18445560676026</v>
       </c>
       <c r="B118" t="n">
         <v>90</v>
@@ -5980,25 +5980,25 @@
         <v>0.0857834520909198</v>
       </c>
       <c r="H118" t="n">
-        <v>0.03367093227376902</v>
+        <v>0.03367093419818044</v>
       </c>
       <c r="I118" t="n">
-        <v>0.02685826388012597</v>
+        <v>0.0268582638801252</v>
       </c>
       <c r="J118" t="n">
         <v>5.696816715522591</v>
       </c>
       <c r="K118" t="n">
-        <v>38.83826218983717</v>
+        <v>38.83825833637303</v>
       </c>
       <c r="L118" t="n">
-        <v>29.95091013276385</v>
+        <v>29.95091013275747</v>
       </c>
       <c r="M118" t="n">
         <v>0.2299030485335895</v>
       </c>
       <c r="N118" t="n">
-        <v>0.2503438825093889</v>
+        <v>0.2503438825093872</v>
       </c>
       <c r="O118" t="n">
         <v>0.3855295790644563</v>
@@ -6024,22 +6024,22 @@
         <v>0</v>
       </c>
       <c r="G119" t="n">
-        <v>0.09412528562904428</v>
+        <v>0.09412528562904426</v>
       </c>
       <c r="H119" t="n">
-        <v>0.02610341344145173</v>
+        <v>0.02610340759447288</v>
       </c>
       <c r="I119" t="n">
-        <v>0.01827050516025587</v>
+        <v>0.01827050412347143</v>
       </c>
       <c r="J119" t="n">
         <v>5.190483785710263</v>
       </c>
       <c r="K119" t="n">
-        <v>53.9915910397898</v>
+        <v>53.99157620341642</v>
       </c>
       <c r="L119" t="n">
-        <v>47.21650751002456</v>
+        <v>47.21650002612878</v>
       </c>
       <c r="M119" t="n">
         <v>0.2302232015958814</v>
@@ -6053,7 +6053,7 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>1.006592763380128</v>
+        <v>1.006592763457831</v>
       </c>
       <c r="B120" t="n">
         <v>0</v>
@@ -6071,36 +6071,36 @@
         <v>0</v>
       </c>
       <c r="G120" t="n">
-        <v>0.05903166816745823</v>
+        <v>0.05903166816745814</v>
       </c>
       <c r="H120" t="n">
-        <v>0.05879831855407184</v>
+        <v>0.05879831855375917</v>
       </c>
       <c r="I120" t="n">
-        <v>0.06870583418297556</v>
+        <v>0.06870583418299378</v>
       </c>
       <c r="J120" t="n">
-        <v>8.293782490621892</v>
+        <v>8.293782490621901</v>
       </c>
       <c r="K120" t="n">
-        <v>21.04637177567111</v>
+        <v>21.04637177608076</v>
       </c>
       <c r="L120" t="n">
-        <v>11.25455325771389</v>
+        <v>11.25455325771581</v>
       </c>
       <c r="M120" t="n">
-        <v>0.2268427903534433</v>
+        <v>0.2268427903534434</v>
       </c>
       <c r="N120" t="n">
-        <v>0.2513760312601657</v>
+        <v>0.2513760312601598</v>
       </c>
       <c r="O120" t="n">
-        <v>0.3863489999532096</v>
+        <v>0.3863489999531894</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>15.75462236170258</v>
+        <v>15.75462235921534</v>
       </c>
       <c r="B121" t="n">
         <v>0</v>
@@ -6118,28 +6118,28 @@
         <v>0</v>
       </c>
       <c r="G121" t="n">
-        <v>0.06701563290042538</v>
+        <v>0.06701563290030682</v>
       </c>
       <c r="H121" t="n">
-        <v>0.051374354936112</v>
+        <v>0.05137435493514467</v>
       </c>
       <c r="I121" t="n">
-        <v>0.06024037485416543</v>
+        <v>0.06024037485416536</v>
       </c>
       <c r="J121" t="n">
-        <v>7.299942556377298</v>
+        <v>7.299942556397835</v>
       </c>
       <c r="K121" t="n">
-        <v>24.26888371725477</v>
+        <v>24.26888371730971</v>
       </c>
       <c r="L121" t="n">
-        <v>12.86148801950044</v>
+        <v>12.86148801950074</v>
       </c>
       <c r="M121" t="n">
-        <v>0.229203500933285</v>
+        <v>0.2292035009334031</v>
       </c>
       <c r="N121" t="n">
-        <v>0.2504409517469725</v>
+        <v>0.2504409517475139</v>
       </c>
       <c r="O121" t="n">
         <v>0.3855295790644589</v>
@@ -6147,7 +6147,7 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>19.71352536272368</v>
+        <v>19.71352536281619</v>
       </c>
       <c r="B122" t="n">
         <v>0</v>
@@ -6165,25 +6165,25 @@
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>0.07608296003690369</v>
+        <v>0.07608296003688363</v>
       </c>
       <c r="H122" t="n">
-        <v>0.04252156904269656</v>
+        <v>0.0425215691390262</v>
       </c>
       <c r="I122" t="n">
-        <v>0.05017595975381861</v>
+        <v>0.05017595975379517</v>
       </c>
       <c r="J122" t="n">
-        <v>6.426040084236202</v>
+        <v>6.426040084236137</v>
       </c>
       <c r="K122" t="n">
-        <v>29.77475562015965</v>
+        <v>29.77475551543131</v>
       </c>
       <c r="L122" t="n">
-        <v>15.50030379108414</v>
+        <v>15.50030379109357</v>
       </c>
       <c r="M122" t="n">
-        <v>0.2301639272572183</v>
+        <v>0.230163927257238</v>
       </c>
       <c r="N122" t="n">
         <v>0.2503438825093889</v>
@@ -6194,7 +6194,7 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>20.44940414632742</v>
+        <v>20.44940414633806</v>
       </c>
       <c r="B123" t="n">
         <v>0</v>
@@ -6212,28 +6212,28 @@
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>0.08505071721380517</v>
+        <v>0.08505071721380511</v>
       </c>
       <c r="H123" t="n">
-        <v>0.03367093329415682</v>
+        <v>0.03367093419836872</v>
       </c>
       <c r="I123" t="n">
-        <v>0.0398389416699501</v>
+        <v>0.03983894171635449</v>
       </c>
       <c r="J123" t="n">
-        <v>5.746060821054358</v>
+        <v>5.746060821054361</v>
       </c>
       <c r="K123" t="n">
-        <v>38.83826014934005</v>
+        <v>38.83825833702297</v>
       </c>
       <c r="L123" t="n">
-        <v>19.66896232904363</v>
+        <v>19.6689623086251</v>
       </c>
       <c r="M123" t="n">
         <v>0.2306394518561364</v>
       </c>
       <c r="N123" t="n">
-        <v>0.2503438825093889</v>
+        <v>0.2503438825093872</v>
       </c>
       <c r="O123" t="n">
         <v>0.3855295790644589</v>
@@ -6259,22 +6259,22 @@
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>0.09335794916455854</v>
+        <v>0.09335794916455853</v>
       </c>
       <c r="H124" t="n">
-        <v>0.02610340894880783</v>
+        <v>0.02610341344144553</v>
       </c>
       <c r="I124" t="n">
-        <v>0.02989360893711528</v>
+        <v>0.02989360955685958</v>
       </c>
       <c r="J124" t="n">
         <v>5.233264444536083</v>
       </c>
       <c r="K124" t="n">
-        <v>53.99157968670422</v>
+        <v>53.99159103981165</v>
       </c>
       <c r="L124" t="n">
-        <v>26.65159222745579</v>
+        <v>26.65159167976872</v>
       </c>
       <c r="M124" t="n">
         <v>0.230993723657685</v>
@@ -6288,7 +6288,7 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>2.772359395752674</v>
+        <v>2.772359395912004</v>
       </c>
       <c r="B125" t="n">
         <v>90</v>
@@ -6306,28 +6306,28 @@
         <v>0</v>
       </c>
       <c r="G125" t="n">
-        <v>0.05903166816745824</v>
+        <v>0.05903166816745829</v>
       </c>
       <c r="H125" t="n">
-        <v>0.05879831855400246</v>
+        <v>0.05879831855407186</v>
       </c>
       <c r="I125" t="n">
-        <v>0.05499992440104675</v>
+        <v>0.0549999244010469</v>
       </c>
       <c r="J125" t="n">
-        <v>8.293782490621892</v>
+        <v>8.293782490621888</v>
       </c>
       <c r="K125" t="n">
-        <v>21.046371775794</v>
+        <v>21.0463717756711</v>
       </c>
       <c r="L125" t="n">
-        <v>14.11116142850666</v>
+        <v>14.11116142850723</v>
       </c>
       <c r="M125" t="n">
-        <v>0.2268427903534433</v>
+        <v>0.2268427903534432</v>
       </c>
       <c r="N125" t="n">
-        <v>0.2513760312601948</v>
+        <v>0.2513760312601657</v>
       </c>
       <c r="O125" t="n">
         <v>0.3855295790644589</v>
@@ -6335,7 +6335,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>15.75462236221469</v>
+        <v>15.75462236170877</v>
       </c>
       <c r="B126" t="n">
         <v>90</v>
@@ -6353,25 +6353,25 @@
         <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>0.06701563290030535</v>
+        <v>0.0670156329004253</v>
       </c>
       <c r="H126" t="n">
-        <v>0.05137435493611304</v>
+        <v>0.05137435493611302</v>
       </c>
       <c r="I126" t="n">
-        <v>0.04618037325599046</v>
+        <v>0.04618037325428546</v>
       </c>
       <c r="J126" t="n">
-        <v>7.299942556398161</v>
+        <v>7.299942556377309</v>
       </c>
       <c r="K126" t="n">
-        <v>24.26888371725404</v>
+        <v>24.26888371725405</v>
       </c>
       <c r="L126" t="n">
-        <v>16.87985375481183</v>
+        <v>16.87985375531651</v>
       </c>
       <c r="M126" t="n">
-        <v>0.2292035009334044</v>
+        <v>0.229203500933285</v>
       </c>
       <c r="N126" t="n">
         <v>0.2504409517469713</v>
@@ -6382,7 +6382,7 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>19.71352536272216</v>
+        <v>19.71352536272517</v>
       </c>
       <c r="B127" t="n">
         <v>90</v>
@@ -6400,25 +6400,25 @@
         <v>0</v>
       </c>
       <c r="G127" t="n">
-        <v>0.07608296003690397</v>
+        <v>0.07608296003690333</v>
       </c>
       <c r="H127" t="n">
-        <v>0.04252156878117114</v>
+        <v>0.04252156914041652</v>
       </c>
       <c r="I127" t="n">
-        <v>0.03657296379961163</v>
+        <v>0.03657296383503037</v>
       </c>
       <c r="J127" t="n">
-        <v>6.426040084236247</v>
+        <v>6.426040084236175</v>
       </c>
       <c r="K127" t="n">
-        <v>29.7747559002623</v>
+        <v>29.77475551392185</v>
       </c>
       <c r="L127" t="n">
-        <v>21.50869236650773</v>
+        <v>21.50869234712528</v>
       </c>
       <c r="M127" t="n">
-        <v>0.2301639272572179</v>
+        <v>0.2301639272572185</v>
       </c>
       <c r="N127" t="n">
         <v>0.2503438825093889</v>
@@ -6450,19 +6450,19 @@
         <v>0.08505071721380504</v>
       </c>
       <c r="H128" t="n">
-        <v>0.03367093419831436</v>
+        <v>0.03367093419824635</v>
       </c>
       <c r="I128" t="n">
-        <v>0.02685826388012524</v>
+        <v>0.02685826388012271</v>
       </c>
       <c r="J128" t="n">
-        <v>5.746060821054366</v>
+        <v>5.746060821054367</v>
       </c>
       <c r="K128" t="n">
-        <v>38.8382583368337</v>
+        <v>38.838258336595</v>
       </c>
       <c r="L128" t="n">
-        <v>29.95091013275823</v>
+        <v>29.95091013273639</v>
       </c>
       <c r="M128" t="n">
         <v>0.2306394518561364</v>
@@ -6494,22 +6494,22 @@
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>0.09335794916455839</v>
+        <v>0.09335794916455845</v>
       </c>
       <c r="H129" t="n">
-        <v>0.02610341344145075</v>
+        <v>0.02610341344145001</v>
       </c>
       <c r="I129" t="n">
-        <v>0.0182705040748632</v>
+        <v>0.01827050411378333</v>
       </c>
       <c r="J129" t="n">
-        <v>5.233264444536091</v>
+        <v>5.233264444536088</v>
       </c>
       <c r="K129" t="n">
-        <v>53.9915910397935</v>
+        <v>53.99159103979598</v>
       </c>
       <c r="L129" t="n">
-        <v>47.21649956500421</v>
+        <v>47.21649993437438</v>
       </c>
       <c r="M129" t="n">
         <v>0.230993723657685</v>

</xml_diff>